<commit_message>
feat(pricing): them Sheet Chenh Lech Tang Gia (Gia Nhap - NPP Online - Facebook - TMDT - Niem Yet)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Bang_Gia_LockKing_Takin" sheetId="1" r:id="rId1"/>
+    <sheet name="Bang_Gia_Chuan_65_Ma" sheetId="1" r:id="rId1"/>
+    <sheet name="ChenhLech_Gia_FB_TMDT_NY" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -642,7 +643,7 @@
         <v>450000</v>
       </c>
       <c r="G7">
-        <v>950000</v>
+        <v>850000</v>
       </c>
       <c r="H7">
         <v>961200</v>
@@ -651,10 +652,10 @@
         <v>1200000</v>
       </c>
       <c r="J7">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="K7" t="str">
-        <v>52.6%</v>
+        <v>47.1%</v>
       </c>
     </row>
     <row r="8">
@@ -2727,4 +2728,3333 @@
     <ignoredError numberStoredAsText="1" sqref="A1:K66"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P66"/>
+  <cols>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="26.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="28.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Thương Hiệu</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Phân Loại</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Model (Mã Sản Phẩm)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Tên Sản Phẩm</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Giá Nhập Hiện Tại (VNĐ)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Giá NPP Online (VNĐ)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Giá Facebook (Làm Tròn Nghìn)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Lãi FB vs Vốn Nhập (VNĐ)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>% Biên LN FB vs Giá Nhập</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Giá Sàn TMĐT (+5% FB, Tròn Nghìn)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Chênh Lệch TMĐT vs FB (VNĐ)</v>
+      </c>
+      <c r="M1" t="str">
+        <v>% Biên Độ TMĐT vs FB</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Giá Niêm Yết (+15% TMĐT, Tròn Nghìn)</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Chênh Lệch Niêm Yết vs TMĐT (VNĐ)</v>
+      </c>
+      <c r="P1" t="str">
+        <v>% Biên Độ Niêm Yết vs TMĐT</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C2" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D2" t="str">
+        <v>LK-2202A</v>
+      </c>
+      <c r="E2" t="str">
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) LK-2202A</v>
+      </c>
+      <c r="F2">
+        <v>204786</v>
+      </c>
+      <c r="G2">
+        <v>265000</v>
+      </c>
+      <c r="H2">
+        <v>467000</v>
+      </c>
+      <c r="I2">
+        <v>262214</v>
+      </c>
+      <c r="J2" t="str">
+        <v>56.1%</v>
+      </c>
+      <c r="K2">
+        <v>491000</v>
+      </c>
+      <c r="L2">
+        <v>24000</v>
+      </c>
+      <c r="M2" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N2">
+        <v>565000</v>
+      </c>
+      <c r="O2">
+        <v>74000</v>
+      </c>
+      <c r="P2" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>LK-2404S</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Chảo sâu Titan vàng 24*8,5cm (2,3 mm) LK-2404S</v>
+      </c>
+      <c r="F3">
+        <v>251705</v>
+      </c>
+      <c r="G3">
+        <v>360000</v>
+      </c>
+      <c r="H3">
+        <v>649000</v>
+      </c>
+      <c r="I3">
+        <v>397295</v>
+      </c>
+      <c r="J3" t="str">
+        <v>61.2%</v>
+      </c>
+      <c r="K3">
+        <v>682000</v>
+      </c>
+      <c r="L3">
+        <v>33000</v>
+      </c>
+      <c r="M3" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N3">
+        <v>785000</v>
+      </c>
+      <c r="O3">
+        <v>103000</v>
+      </c>
+      <c r="P3" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>LK-2433</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Chảo Belly Lock&amp;King</v>
+      </c>
+      <c r="F4">
+        <v>307555</v>
+      </c>
+      <c r="G4">
+        <v>395000</v>
+      </c>
+      <c r="H4">
+        <v>750000</v>
+      </c>
+      <c r="I4">
+        <v>442445</v>
+      </c>
+      <c r="J4" t="str">
+        <v>59.0%</v>
+      </c>
+      <c r="K4">
+        <v>788000</v>
+      </c>
+      <c r="L4">
+        <v>38000</v>
+      </c>
+      <c r="M4" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N4">
+        <v>907000</v>
+      </c>
+      <c r="O4">
+        <v>119000</v>
+      </c>
+      <c r="P4" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>LK-2466S</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Chảo Titanium  ELITE Lock&amp;King</v>
+      </c>
+      <c r="F5">
+        <v>289484</v>
+      </c>
+      <c r="G5">
+        <v>390000</v>
+      </c>
+      <c r="H5">
+        <v>690000</v>
+      </c>
+      <c r="I5">
+        <v>400516</v>
+      </c>
+      <c r="J5" t="str">
+        <v>58.0%</v>
+      </c>
+      <c r="K5">
+        <v>725000</v>
+      </c>
+      <c r="L5">
+        <v>35000</v>
+      </c>
+      <c r="M5" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N5">
+        <v>834000</v>
+      </c>
+      <c r="O5">
+        <v>109000</v>
+      </c>
+      <c r="P5" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D6" t="str">
+        <v>LK-2606A</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Chảo cạn Titanium Lock&amp;king 26cm</v>
+      </c>
+      <c r="F6">
+        <v>238375</v>
+      </c>
+      <c r="G6">
+        <v>320000</v>
+      </c>
+      <c r="H6">
+        <v>590000</v>
+      </c>
+      <c r="I6">
+        <v>351625</v>
+      </c>
+      <c r="J6" t="str">
+        <v>59.6%</v>
+      </c>
+      <c r="K6">
+        <v>620000</v>
+      </c>
+      <c r="L6">
+        <v>30000</v>
+      </c>
+      <c r="M6" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N6">
+        <v>713000</v>
+      </c>
+      <c r="O6">
+        <v>93000</v>
+      </c>
+      <c r="P6" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D7" t="str">
+        <v>LK-2633</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Chảo Belly Lock&amp;King Titanium 26cm</v>
+      </c>
+      <c r="F7">
+        <v>350676</v>
+      </c>
+      <c r="G7">
+        <v>450000</v>
+      </c>
+      <c r="H7">
+        <v>850000</v>
+      </c>
+      <c r="I7">
+        <v>499324</v>
+      </c>
+      <c r="J7" t="str">
+        <v>58.7%</v>
+      </c>
+      <c r="K7">
+        <v>893000</v>
+      </c>
+      <c r="L7">
+        <v>43000</v>
+      </c>
+      <c r="M7" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N7">
+        <v>1027000</v>
+      </c>
+      <c r="O7">
+        <v>134000</v>
+      </c>
+      <c r="P7" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D8" t="str">
+        <v>LK-2808</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+      </c>
+      <c r="F8">
+        <v>267721</v>
+      </c>
+      <c r="G8">
+        <v>351000</v>
+      </c>
+      <c r="H8">
+        <v>630000</v>
+      </c>
+      <c r="I8">
+        <v>362279</v>
+      </c>
+      <c r="J8" t="str">
+        <v>57.5%</v>
+      </c>
+      <c r="K8">
+        <v>662000</v>
+      </c>
+      <c r="L8">
+        <v>32000</v>
+      </c>
+      <c r="M8" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N8">
+        <v>762000</v>
+      </c>
+      <c r="O8">
+        <v>100000</v>
+      </c>
+      <c r="P8" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D9" t="str">
+        <v>LK-2808S(VK)</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Chảo sâu vung kính Titanium Lock&amp;king 28cm</v>
+      </c>
+      <c r="F9">
+        <v>320736</v>
+      </c>
+      <c r="G9">
+        <v>370000</v>
+      </c>
+      <c r="H9">
+        <v>642000</v>
+      </c>
+      <c r="I9">
+        <v>321264</v>
+      </c>
+      <c r="J9" t="str">
+        <v>50.0%</v>
+      </c>
+      <c r="K9">
+        <v>675000</v>
+      </c>
+      <c r="L9">
+        <v>33000</v>
+      </c>
+      <c r="M9" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N9">
+        <v>777000</v>
+      </c>
+      <c r="O9">
+        <v>102000</v>
+      </c>
+      <c r="P9" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C10" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D10" t="str">
+        <v>LK-2808SA</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA</v>
+      </c>
+      <c r="F10">
+        <v>319135</v>
+      </c>
+      <c r="G10">
+        <v>431000</v>
+      </c>
+      <c r="H10">
+        <v>760000</v>
+      </c>
+      <c r="I10">
+        <v>440865</v>
+      </c>
+      <c r="J10" t="str">
+        <v>58.0%</v>
+      </c>
+      <c r="K10">
+        <v>798000</v>
+      </c>
+      <c r="L10">
+        <v>38000</v>
+      </c>
+      <c r="M10" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N10">
+        <v>918000</v>
+      </c>
+      <c r="O10">
+        <v>120000</v>
+      </c>
+      <c r="P10" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D11" t="str">
+        <v>LK-2808SA KHÔNG NẮP</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA KHÔNG NẮP</v>
+      </c>
+      <c r="F11">
+        <v>320736</v>
+      </c>
+      <c r="G11">
+        <v>412000</v>
+      </c>
+      <c r="H11">
+        <v>740000</v>
+      </c>
+      <c r="I11">
+        <v>419264</v>
+      </c>
+      <c r="J11" t="str">
+        <v>56.7%</v>
+      </c>
+      <c r="K11">
+        <v>777000</v>
+      </c>
+      <c r="L11">
+        <v>37000</v>
+      </c>
+      <c r="M11" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N11">
+        <v>894000</v>
+      </c>
+      <c r="O11">
+        <v>117000</v>
+      </c>
+      <c r="P11" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C12" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D12" t="str">
+        <v>LK-3003</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Chảo cạn titanium Lock&amp;King 30cm</v>
+      </c>
+      <c r="F12">
+        <v>291830</v>
+      </c>
+      <c r="G12">
+        <v>375000</v>
+      </c>
+      <c r="H12">
+        <v>750000</v>
+      </c>
+      <c r="I12">
+        <v>458170</v>
+      </c>
+      <c r="J12" t="str">
+        <v>61.1%</v>
+      </c>
+      <c r="K12">
+        <v>788000</v>
+      </c>
+      <c r="L12">
+        <v>38000</v>
+      </c>
+      <c r="M12" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N12">
+        <v>907000</v>
+      </c>
+      <c r="O12">
+        <v>119000</v>
+      </c>
+      <c r="P12" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C13" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D13" t="str">
+        <v>LK-3212</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Chảo xào lớn</v>
+      </c>
+      <c r="F13">
+        <v>472432</v>
+      </c>
+      <c r="G13">
+        <v>645000</v>
+      </c>
+      <c r="H13">
+        <v>1290000</v>
+      </c>
+      <c r="I13">
+        <v>817568</v>
+      </c>
+      <c r="J13" t="str">
+        <v>63.4%</v>
+      </c>
+      <c r="K13">
+        <v>1355000</v>
+      </c>
+      <c r="L13">
+        <v>65000</v>
+      </c>
+      <c r="M13" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N13">
+        <v>1559000</v>
+      </c>
+      <c r="O13">
+        <v>204000</v>
+      </c>
+      <c r="P13" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C14" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D14" t="str">
+        <v>LK-30NC1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Nồi luộc gà Lock&amp;King size 30</v>
+      </c>
+      <c r="F14">
+        <v>336906</v>
+      </c>
+      <c r="G14">
+        <v>414000</v>
+      </c>
+      <c r="H14">
+        <v>750000</v>
+      </c>
+      <c r="I14">
+        <v>413094</v>
+      </c>
+      <c r="J14" t="str">
+        <v>55.1%</v>
+      </c>
+      <c r="K14">
+        <v>788000</v>
+      </c>
+      <c r="L14">
+        <v>38000</v>
+      </c>
+      <c r="M14" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N14">
+        <v>907000</v>
+      </c>
+      <c r="O14">
+        <v>119000</v>
+      </c>
+      <c r="P14" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C15" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D15" t="str">
+        <v>LK-32NC1</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Nồi luộc gà Lock&amp;King size 32</v>
+      </c>
+      <c r="F15">
+        <v>400473</v>
+      </c>
+      <c r="G15">
+        <v>470000</v>
+      </c>
+      <c r="H15">
+        <v>830000</v>
+      </c>
+      <c r="I15">
+        <v>429527</v>
+      </c>
+      <c r="J15" t="str">
+        <v>51.8%</v>
+      </c>
+      <c r="K15">
+        <v>872000</v>
+      </c>
+      <c r="L15">
+        <v>42000</v>
+      </c>
+      <c r="M15" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N15">
+        <v>1003000</v>
+      </c>
+      <c r="O15">
+        <v>131000</v>
+      </c>
+      <c r="P15" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C16" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D16" t="str">
+        <v>LK-336A</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Bộ nồi 3 Lock&amp;King ( 18,20,24 )</v>
+      </c>
+      <c r="F16">
+        <v>411881</v>
+      </c>
+      <c r="G16">
+        <v>540000</v>
+      </c>
+      <c r="H16">
+        <v>990000</v>
+      </c>
+      <c r="I16">
+        <v>578119</v>
+      </c>
+      <c r="J16" t="str">
+        <v>58.4%</v>
+      </c>
+      <c r="K16">
+        <v>1040000</v>
+      </c>
+      <c r="L16">
+        <v>50000</v>
+      </c>
+      <c r="M16" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N16">
+        <v>1196000</v>
+      </c>
+      <c r="O16">
+        <v>156000</v>
+      </c>
+      <c r="P16" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C17" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D17" t="str">
+        <v>LK-3018A</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Nồi lẻ Lock&amp;king 18</v>
+      </c>
+      <c r="F17">
+        <v>131000</v>
+      </c>
+      <c r="G17">
+        <v>170000</v>
+      </c>
+      <c r="H17">
+        <v>295000</v>
+      </c>
+      <c r="I17">
+        <v>164000</v>
+      </c>
+      <c r="J17" t="str">
+        <v>55.6%</v>
+      </c>
+      <c r="K17">
+        <v>310000</v>
+      </c>
+      <c r="L17">
+        <v>15000</v>
+      </c>
+      <c r="M17" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N17">
+        <v>357000</v>
+      </c>
+      <c r="O17">
+        <v>47000</v>
+      </c>
+      <c r="P17" t="str">
+        <v>15.2%</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C18" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D18" t="str">
+        <v>LK-3020A</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Nồi lẻ Lock&amp;king 20</v>
+      </c>
+      <c r="F18">
+        <v>148885</v>
+      </c>
+      <c r="G18">
+        <v>185000</v>
+      </c>
+      <c r="H18">
+        <v>315000</v>
+      </c>
+      <c r="I18">
+        <v>166115</v>
+      </c>
+      <c r="J18" t="str">
+        <v>52.7%</v>
+      </c>
+      <c r="K18">
+        <v>331000</v>
+      </c>
+      <c r="L18">
+        <v>16000</v>
+      </c>
+      <c r="M18" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N18">
+        <v>381000</v>
+      </c>
+      <c r="O18">
+        <v>50000</v>
+      </c>
+      <c r="P18" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C19" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D19" t="str">
+        <v>LK-3024</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Nồi lẻ Lock&amp;king 24</v>
+      </c>
+      <c r="F19">
+        <v>183215</v>
+      </c>
+      <c r="G19">
+        <v>230000</v>
+      </c>
+      <c r="H19">
+        <v>395000</v>
+      </c>
+      <c r="I19">
+        <v>211785</v>
+      </c>
+      <c r="J19" t="str">
+        <v>53.6%</v>
+      </c>
+      <c r="K19">
+        <v>415000</v>
+      </c>
+      <c r="L19">
+        <v>20000</v>
+      </c>
+      <c r="M19" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N19">
+        <v>478000</v>
+      </c>
+      <c r="O19">
+        <v>63000</v>
+      </c>
+      <c r="P19" t="str">
+        <v>15.2%</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C20" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D20" t="str">
+        <v>LK-3116</v>
+      </c>
+      <c r="E20" t="str">
+        <v>16*9CM Quánh liền khối titan (2.2mm) LK-3116</v>
+      </c>
+      <c r="F20">
+        <v>236683</v>
+      </c>
+      <c r="G20">
+        <v>325000</v>
+      </c>
+      <c r="H20">
+        <v>689000</v>
+      </c>
+      <c r="I20">
+        <v>452317</v>
+      </c>
+      <c r="J20" t="str">
+        <v>65.6%</v>
+      </c>
+      <c r="K20">
+        <v>724000</v>
+      </c>
+      <c r="L20">
+        <v>35000</v>
+      </c>
+      <c r="M20" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N20">
+        <v>833000</v>
+      </c>
+      <c r="O20">
+        <v>109000</v>
+      </c>
+      <c r="P20" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C21" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D21" t="str">
+        <v>LK-3118</v>
+      </c>
+      <c r="E21" t="str">
+        <v>18*10CM Nồi lẻ kèm nắp (2.3mm) LK-3118</v>
+      </c>
+      <c r="F21">
+        <v>265000</v>
+      </c>
+      <c r="G21">
+        <v>340000</v>
+      </c>
+      <c r="H21">
+        <v>779000</v>
+      </c>
+      <c r="I21">
+        <v>514000</v>
+      </c>
+      <c r="J21" t="str">
+        <v>66.0%</v>
+      </c>
+      <c r="K21">
+        <v>818000</v>
+      </c>
+      <c r="L21">
+        <v>39000</v>
+      </c>
+      <c r="M21" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N21">
+        <v>941000</v>
+      </c>
+      <c r="O21">
+        <v>123000</v>
+      </c>
+      <c r="P21" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C22" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D22" t="str">
+        <v>LK-3120</v>
+      </c>
+      <c r="E22" t="str">
+        <v>20*12CM Nồi lẻ kèm nắp (2.3mm) LK-3120</v>
+      </c>
+      <c r="F22">
+        <v>297124</v>
+      </c>
+      <c r="G22">
+        <v>390000</v>
+      </c>
+      <c r="H22">
+        <v>889000</v>
+      </c>
+      <c r="I22">
+        <v>591876</v>
+      </c>
+      <c r="J22" t="str">
+        <v>66.6%</v>
+      </c>
+      <c r="K22">
+        <v>934000</v>
+      </c>
+      <c r="L22">
+        <v>45000</v>
+      </c>
+      <c r="M22" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N22">
+        <v>1075000</v>
+      </c>
+      <c r="O22">
+        <v>141000</v>
+      </c>
+      <c r="P22" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C23" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D23" t="str">
+        <v>LK-3124</v>
+      </c>
+      <c r="E23" t="str">
+        <v>24*14CM Nồi lẻ kèm nắp (2.3mm) LK-3124</v>
+      </c>
+      <c r="F23">
+        <v>359737</v>
+      </c>
+      <c r="G23">
+        <v>460000</v>
+      </c>
+      <c r="H23">
+        <v>1049000</v>
+      </c>
+      <c r="I23">
+        <v>689263</v>
+      </c>
+      <c r="J23" t="str">
+        <v>65.7%</v>
+      </c>
+      <c r="K23">
+        <v>1102000</v>
+      </c>
+      <c r="L23">
+        <v>53000</v>
+      </c>
+      <c r="M23" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N23">
+        <v>1268000</v>
+      </c>
+      <c r="O23">
+        <v>166000</v>
+      </c>
+      <c r="P23" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C24" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D24" t="str">
+        <v>LK-3338</v>
+      </c>
+      <c r="E24" t="str">
+        <v>18+20+24CM Bộ nồi 3 liền khối kèm nắp (2.3mm) LK-3338</v>
+      </c>
+      <c r="F24">
+        <v>883000</v>
+      </c>
+      <c r="G24">
+        <v>1100000</v>
+      </c>
+      <c r="H24">
+        <v>2090000</v>
+      </c>
+      <c r="I24">
+        <v>1207000</v>
+      </c>
+      <c r="J24" t="str">
+        <v>57.8%</v>
+      </c>
+      <c r="K24">
+        <v>2195000</v>
+      </c>
+      <c r="L24">
+        <v>105000</v>
+      </c>
+      <c r="M24" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N24">
+        <v>2525000</v>
+      </c>
+      <c r="O24">
+        <v>330000</v>
+      </c>
+      <c r="P24" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C25" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D25" t="str">
+        <v>LK-3386A</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
+      </c>
+      <c r="F25">
+        <v>453015</v>
+      </c>
+      <c r="G25">
+        <v>550000</v>
+      </c>
+      <c r="H25">
+        <v>990000</v>
+      </c>
+      <c r="I25">
+        <v>536985</v>
+      </c>
+      <c r="J25" t="str">
+        <v>54.2%</v>
+      </c>
+      <c r="K25">
+        <v>1040000</v>
+      </c>
+      <c r="L25">
+        <v>50000</v>
+      </c>
+      <c r="M25" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N25">
+        <v>1196000</v>
+      </c>
+      <c r="O25">
+        <v>156000</v>
+      </c>
+      <c r="P25" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C26" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D26" t="str">
+        <v>LK-3568A</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
+      </c>
+      <c r="F26">
+        <v>815667</v>
+      </c>
+      <c r="G26">
+        <v>960000</v>
+      </c>
+      <c r="H26">
+        <v>1690000</v>
+      </c>
+      <c r="I26">
+        <v>874333</v>
+      </c>
+      <c r="J26" t="str">
+        <v>51.7%</v>
+      </c>
+      <c r="K26">
+        <v>1775000</v>
+      </c>
+      <c r="L26">
+        <v>85000</v>
+      </c>
+      <c r="M26" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N26">
+        <v>2042000</v>
+      </c>
+      <c r="O26">
+        <v>267000</v>
+      </c>
+      <c r="P26" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C27" t="str">
+        <v>NỒI TĂNG ÁP</v>
+      </c>
+      <c r="D27" t="str">
+        <v>LK-3122</v>
+      </c>
+      <c r="E27" t="str">
+        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
+      </c>
+      <c r="F27">
+        <v>357441</v>
+      </c>
+      <c r="G27">
+        <v>470000</v>
+      </c>
+      <c r="H27">
+        <v>820000</v>
+      </c>
+      <c r="I27">
+        <v>462559</v>
+      </c>
+      <c r="J27" t="str">
+        <v>56.4%</v>
+      </c>
+      <c r="K27">
+        <v>861000</v>
+      </c>
+      <c r="L27">
+        <v>41000</v>
+      </c>
+      <c r="M27" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N27">
+        <v>991000</v>
+      </c>
+      <c r="O27">
+        <v>130000</v>
+      </c>
+      <c r="P27" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C28" t="str">
+        <v>NỒI TĂNG ÁP</v>
+      </c>
+      <c r="D28" t="str">
+        <v>LK-3126</v>
+      </c>
+      <c r="E28" t="str">
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
+      </c>
+      <c r="F28">
+        <v>387848</v>
+      </c>
+      <c r="G28">
+        <v>535000</v>
+      </c>
+      <c r="H28">
+        <v>990000</v>
+      </c>
+      <c r="I28">
+        <v>602152</v>
+      </c>
+      <c r="J28" t="str">
+        <v>60.8%</v>
+      </c>
+      <c r="K28">
+        <v>1040000</v>
+      </c>
+      <c r="L28">
+        <v>50000</v>
+      </c>
+      <c r="M28" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N28">
+        <v>1196000</v>
+      </c>
+      <c r="O28">
+        <v>156000</v>
+      </c>
+      <c r="P28" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C29" t="str">
+        <v>ẤM &amp; BÌNH</v>
+      </c>
+      <c r="D29" t="str">
+        <v>LK-1035</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Ấm đun nước LK-1035</v>
+      </c>
+      <c r="F29">
+        <v>217057</v>
+      </c>
+      <c r="G29">
+        <v>275000</v>
+      </c>
+      <c r="H29">
+        <v>549000</v>
+      </c>
+      <c r="I29">
+        <v>331943</v>
+      </c>
+      <c r="J29" t="str">
+        <v>60.5%</v>
+      </c>
+      <c r="K29">
+        <v>577000</v>
+      </c>
+      <c r="L29">
+        <v>28000</v>
+      </c>
+      <c r="M29" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N29">
+        <v>664000</v>
+      </c>
+      <c r="O29">
+        <v>87000</v>
+      </c>
+      <c r="P29" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C30" t="str">
+        <v>ẤM &amp; BÌNH</v>
+      </c>
+      <c r="D30" t="str">
+        <v>LK-1038</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Ấm đun nước LK-1038</v>
+      </c>
+      <c r="F30">
+        <v>235094</v>
+      </c>
+      <c r="G30">
+        <v>300000</v>
+      </c>
+      <c r="H30">
+        <v>525000</v>
+      </c>
+      <c r="I30">
+        <v>289906</v>
+      </c>
+      <c r="J30" t="str">
+        <v>55.2%</v>
+      </c>
+      <c r="K30">
+        <v>552000</v>
+      </c>
+      <c r="L30">
+        <v>27000</v>
+      </c>
+      <c r="M30" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N30">
+        <v>635000</v>
+      </c>
+      <c r="O30">
+        <v>83000</v>
+      </c>
+      <c r="P30" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C31" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D31" t="str">
+        <v>LK-92</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Nồi chiên không dầu Lock&amp;king</v>
+      </c>
+      <c r="F31">
+        <v>727600</v>
+      </c>
+      <c r="G31">
+        <v>835000</v>
+      </c>
+      <c r="H31">
+        <v>1590000</v>
+      </c>
+      <c r="I31">
+        <v>862400</v>
+      </c>
+      <c r="J31" t="str">
+        <v>54.2%</v>
+      </c>
+      <c r="K31">
+        <v>1670000</v>
+      </c>
+      <c r="L31">
+        <v>80000</v>
+      </c>
+      <c r="M31" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N31">
+        <v>1921000</v>
+      </c>
+      <c r="O31">
+        <v>251000</v>
+      </c>
+      <c r="P31" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C32" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D32" t="str">
+        <v>LK-586</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Sưởi gốm thấp</v>
+      </c>
+      <c r="F32">
+        <v>366857</v>
+      </c>
+      <c r="G32">
+        <v>430000</v>
+      </c>
+      <c r="H32">
+        <v>745000</v>
+      </c>
+      <c r="I32">
+        <v>378143</v>
+      </c>
+      <c r="J32" t="str">
+        <v>50.8%</v>
+      </c>
+      <c r="K32">
+        <v>783000</v>
+      </c>
+      <c r="L32">
+        <v>38000</v>
+      </c>
+      <c r="M32" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N32">
+        <v>901000</v>
+      </c>
+      <c r="O32">
+        <v>118000</v>
+      </c>
+      <c r="P32" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C33" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D33" t="str">
+        <v>LK-588</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Sưởi gốm thân cao</v>
+      </c>
+      <c r="F33">
+        <v>468762</v>
+      </c>
+      <c r="G33">
+        <v>585000</v>
+      </c>
+      <c r="H33">
+        <v>1050000</v>
+      </c>
+      <c r="I33">
+        <v>581238</v>
+      </c>
+      <c r="J33" t="str">
+        <v>55.4%</v>
+      </c>
+      <c r="K33">
+        <v>1103000</v>
+      </c>
+      <c r="L33">
+        <v>53000</v>
+      </c>
+      <c r="M33" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N33">
+        <v>1269000</v>
+      </c>
+      <c r="O33">
+        <v>166000</v>
+      </c>
+      <c r="P33" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C34" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D34" t="str">
+        <v>LK-668</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
+      </c>
+      <c r="F34">
+        <v>395900</v>
+      </c>
+      <c r="G34">
+        <v>460000</v>
+      </c>
+      <c r="H34">
+        <v>920000</v>
+      </c>
+      <c r="I34">
+        <v>524100</v>
+      </c>
+      <c r="J34" t="str">
+        <v>57.0%</v>
+      </c>
+      <c r="K34">
+        <v>966000</v>
+      </c>
+      <c r="L34">
+        <v>46000</v>
+      </c>
+      <c r="M34" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N34">
+        <v>1111000</v>
+      </c>
+      <c r="O34">
+        <v>145000</v>
+      </c>
+      <c r="P34" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C35" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D35" t="str">
+        <v>LK-688</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
+      </c>
+      <c r="F35">
+        <v>727600</v>
+      </c>
+      <c r="G35">
+        <v>850000</v>
+      </c>
+      <c r="H35">
+        <v>1690000</v>
+      </c>
+      <c r="I35">
+        <v>962400</v>
+      </c>
+      <c r="J35" t="str">
+        <v>56.9%</v>
+      </c>
+      <c r="K35">
+        <v>1775000</v>
+      </c>
+      <c r="L35">
+        <v>85000</v>
+      </c>
+      <c r="M35" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N35">
+        <v>2042000</v>
+      </c>
+      <c r="O35">
+        <v>267000</v>
+      </c>
+      <c r="P35" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C36" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D36" t="str">
+        <v>LK-1003</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+      </c>
+      <c r="F36">
+        <v>167990</v>
+      </c>
+      <c r="G36">
+        <v>197000</v>
+      </c>
+      <c r="H36">
+        <v>354000</v>
+      </c>
+      <c r="I36">
+        <v>186010</v>
+      </c>
+      <c r="J36" t="str">
+        <v>52.5%</v>
+      </c>
+      <c r="K36">
+        <v>372000</v>
+      </c>
+      <c r="L36">
+        <v>18000</v>
+      </c>
+      <c r="M36" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N36">
+        <v>428000</v>
+      </c>
+      <c r="O36">
+        <v>56000</v>
+      </c>
+      <c r="P36" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C37" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D37" t="str">
+        <v>LK-1030</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+      </c>
+      <c r="F37">
+        <v>795408</v>
+      </c>
+      <c r="G37">
+        <v>1020000</v>
+      </c>
+      <c r="H37">
+        <v>1890000</v>
+      </c>
+      <c r="I37">
+        <v>1094592</v>
+      </c>
+      <c r="J37" t="str">
+        <v>57.9%</v>
+      </c>
+      <c r="K37">
+        <v>1985000</v>
+      </c>
+      <c r="L37">
+        <v>95000</v>
+      </c>
+      <c r="M37" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N37">
+        <v>2283000</v>
+      </c>
+      <c r="O37">
+        <v>298000</v>
+      </c>
+      <c r="P37" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C38" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D38" t="str">
+        <v>LK-1033</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+      </c>
+      <c r="F38">
+        <v>306020</v>
+      </c>
+      <c r="G38">
+        <v>372000</v>
+      </c>
+      <c r="H38">
+        <v>670000</v>
+      </c>
+      <c r="I38">
+        <v>363980</v>
+      </c>
+      <c r="J38" t="str">
+        <v>54.3%</v>
+      </c>
+      <c r="K38">
+        <v>704000</v>
+      </c>
+      <c r="L38">
+        <v>34000</v>
+      </c>
+      <c r="M38" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N38">
+        <v>810000</v>
+      </c>
+      <c r="O38">
+        <v>106000</v>
+      </c>
+      <c r="P38" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C39" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D39" t="str">
+        <v>LK-1050</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+      </c>
+      <c r="F39">
+        <v>668157</v>
+      </c>
+      <c r="G39">
+        <v>780000</v>
+      </c>
+      <c r="H39">
+        <v>1495000</v>
+      </c>
+      <c r="I39">
+        <v>826843</v>
+      </c>
+      <c r="J39" t="str">
+        <v>55.3%</v>
+      </c>
+      <c r="K39">
+        <v>1570000</v>
+      </c>
+      <c r="L39">
+        <v>75000</v>
+      </c>
+      <c r="M39" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N39">
+        <v>1806000</v>
+      </c>
+      <c r="O39">
+        <v>236000</v>
+      </c>
+      <c r="P39" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C40" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D40" t="str">
+        <v>LK-1068</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Ấm siêu tốc LK-1068</v>
+      </c>
+      <c r="F40">
+        <v>259549</v>
+      </c>
+      <c r="G40">
+        <v>310000</v>
+      </c>
+      <c r="H40">
+        <v>599000</v>
+      </c>
+      <c r="I40">
+        <v>339451</v>
+      </c>
+      <c r="J40" t="str">
+        <v>56.7%</v>
+      </c>
+      <c r="K40">
+        <v>629000</v>
+      </c>
+      <c r="L40">
+        <v>30000</v>
+      </c>
+      <c r="M40" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N40">
+        <v>724000</v>
+      </c>
+      <c r="O40">
+        <v>95000</v>
+      </c>
+      <c r="P40" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C41" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D41" t="str">
+        <v>LK-4026A</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4026A</v>
+      </c>
+      <c r="F41">
+        <v>350000</v>
+      </c>
+      <c r="G41">
+        <v>440000</v>
+      </c>
+      <c r="H41">
+        <v>850000</v>
+      </c>
+      <c r="I41">
+        <v>500000</v>
+      </c>
+      <c r="J41" t="str">
+        <v>58.8%</v>
+      </c>
+      <c r="K41">
+        <v>893000</v>
+      </c>
+      <c r="L41">
+        <v>43000</v>
+      </c>
+      <c r="M41" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N41">
+        <v>1027000</v>
+      </c>
+      <c r="O41">
+        <v>134000</v>
+      </c>
+      <c r="P41" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C42" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D42" t="str">
+        <v>LK-4160</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+      </c>
+      <c r="F42">
+        <v>828486</v>
+      </c>
+      <c r="G42">
+        <v>1000000</v>
+      </c>
+      <c r="H42">
+        <v>2350000</v>
+      </c>
+      <c r="I42">
+        <v>1521514</v>
+      </c>
+      <c r="J42" t="str">
+        <v>64.7%</v>
+      </c>
+      <c r="K42">
+        <v>2468000</v>
+      </c>
+      <c r="L42">
+        <v>118000</v>
+      </c>
+      <c r="M42" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N42">
+        <v>2839000</v>
+      </c>
+      <c r="O42">
+        <v>371000</v>
+      </c>
+      <c r="P42" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C43" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D43" t="str">
+        <v>LK-4161</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+      </c>
+      <c r="F43">
+        <v>672571</v>
+      </c>
+      <c r="G43">
+        <v>800000</v>
+      </c>
+      <c r="H43">
+        <v>1650000</v>
+      </c>
+      <c r="I43">
+        <v>977429</v>
+      </c>
+      <c r="J43" t="str">
+        <v>59.2%</v>
+      </c>
+      <c r="K43">
+        <v>1733000</v>
+      </c>
+      <c r="L43">
+        <v>83000</v>
+      </c>
+      <c r="M43" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N43">
+        <v>1993000</v>
+      </c>
+      <c r="O43">
+        <v>260000</v>
+      </c>
+      <c r="P43" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C44" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D44" t="str">
+        <v>LK-4208A</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+      </c>
+      <c r="F44">
+        <v>399987</v>
+      </c>
+      <c r="G44">
+        <v>510000</v>
+      </c>
+      <c r="H44">
+        <v>950000</v>
+      </c>
+      <c r="I44">
+        <v>550013</v>
+      </c>
+      <c r="J44" t="str">
+        <v>57.9%</v>
+      </c>
+      <c r="K44">
+        <v>998000</v>
+      </c>
+      <c r="L44">
+        <v>48000</v>
+      </c>
+      <c r="M44" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N44">
+        <v>1148000</v>
+      </c>
+      <c r="O44">
+        <v>150000</v>
+      </c>
+      <c r="P44" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C45" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D45" t="str">
+        <v>LK-4209</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+      </c>
+      <c r="F45">
+        <v>389541</v>
+      </c>
+      <c r="G45">
+        <v>510000</v>
+      </c>
+      <c r="H45">
+        <v>950000</v>
+      </c>
+      <c r="I45">
+        <v>560459</v>
+      </c>
+      <c r="J45" t="str">
+        <v>59.0%</v>
+      </c>
+      <c r="K45">
+        <v>998000</v>
+      </c>
+      <c r="L45">
+        <v>48000</v>
+      </c>
+      <c r="M45" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N45">
+        <v>1148000</v>
+      </c>
+      <c r="O45">
+        <v>150000</v>
+      </c>
+      <c r="P45" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C46" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D46" t="str">
+        <v>LK-5301</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Sưởi để bàn</v>
+      </c>
+      <c r="F46">
+        <v>468762</v>
+      </c>
+      <c r="G46">
+        <v>600000</v>
+      </c>
+      <c r="H46">
+        <v>1190000</v>
+      </c>
+      <c r="I46">
+        <v>721238</v>
+      </c>
+      <c r="J46" t="str">
+        <v>60.6%</v>
+      </c>
+      <c r="K46">
+        <v>1250000</v>
+      </c>
+      <c r="L46">
+        <v>60000</v>
+      </c>
+      <c r="M46" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N46">
+        <v>1438000</v>
+      </c>
+      <c r="O46">
+        <v>188000</v>
+      </c>
+      <c r="P46" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C47" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D47" t="str">
+        <v>LK-6015</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+      </c>
+      <c r="F47">
+        <v>200752</v>
+      </c>
+      <c r="G47">
+        <v>260000</v>
+      </c>
+      <c r="H47">
+        <v>490000</v>
+      </c>
+      <c r="I47">
+        <v>289248</v>
+      </c>
+      <c r="J47" t="str">
+        <v>59.0%</v>
+      </c>
+      <c r="K47">
+        <v>515000</v>
+      </c>
+      <c r="L47">
+        <v>25000</v>
+      </c>
+      <c r="M47" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N47">
+        <v>593000</v>
+      </c>
+      <c r="O47">
+        <v>78000</v>
+      </c>
+      <c r="P47" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C48" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D48" t="str">
+        <v>LK-6201</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+      </c>
+      <c r="F48">
+        <v>550047</v>
+      </c>
+      <c r="G48">
+        <v>685000</v>
+      </c>
+      <c r="H48">
+        <v>1290000</v>
+      </c>
+      <c r="I48">
+        <v>739953</v>
+      </c>
+      <c r="J48" t="str">
+        <v>57.4%</v>
+      </c>
+      <c r="K48">
+        <v>1355000</v>
+      </c>
+      <c r="L48">
+        <v>65000</v>
+      </c>
+      <c r="M48" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N48">
+        <v>1559000</v>
+      </c>
+      <c r="O48">
+        <v>204000</v>
+      </c>
+      <c r="P48" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C49" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D49" t="str">
+        <v>LK-7812</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Máy làm sữa hạt Lock&amp;King</v>
+      </c>
+      <c r="F49">
+        <v>545604</v>
+      </c>
+      <c r="G49">
+        <v>660000</v>
+      </c>
+      <c r="H49">
+        <v>1190000</v>
+      </c>
+      <c r="I49">
+        <v>644396</v>
+      </c>
+      <c r="J49" t="str">
+        <v>54.2%</v>
+      </c>
+      <c r="K49">
+        <v>1250000</v>
+      </c>
+      <c r="L49">
+        <v>60000</v>
+      </c>
+      <c r="M49" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N49">
+        <v>1438000</v>
+      </c>
+      <c r="O49">
+        <v>188000</v>
+      </c>
+      <c r="P49" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C50" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D50" t="str">
+        <v>LK-9014</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Nồi chiên không dầu Lock&amp;king</v>
+      </c>
+      <c r="F50">
+        <v>936250</v>
+      </c>
+      <c r="G50">
+        <v>1130000</v>
+      </c>
+      <c r="H50">
+        <v>2190000</v>
+      </c>
+      <c r="I50">
+        <v>1253750</v>
+      </c>
+      <c r="J50" t="str">
+        <v>57.2%</v>
+      </c>
+      <c r="K50">
+        <v>2300000</v>
+      </c>
+      <c r="L50">
+        <v>110000</v>
+      </c>
+      <c r="M50" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N50">
+        <v>2645000</v>
+      </c>
+      <c r="O50">
+        <v>345000</v>
+      </c>
+      <c r="P50" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C51" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D51" t="str">
+        <v>TK-2201</v>
+      </c>
+      <c r="E51" t="str">
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+      </c>
+      <c r="F51">
+        <v>203634</v>
+      </c>
+      <c r="G51">
+        <v>265000</v>
+      </c>
+      <c r="H51">
+        <v>467000</v>
+      </c>
+      <c r="I51">
+        <v>263366</v>
+      </c>
+      <c r="J51" t="str">
+        <v>56.4%</v>
+      </c>
+      <c r="K51">
+        <v>491000</v>
+      </c>
+      <c r="L51">
+        <v>24000</v>
+      </c>
+      <c r="M51" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N51">
+        <v>565000</v>
+      </c>
+      <c r="O51">
+        <v>74000</v>
+      </c>
+      <c r="P51" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C52" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D52" t="str">
+        <v>TK-2662</v>
+      </c>
+      <c r="E52" t="str">
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+      </c>
+      <c r="F52">
+        <v>238375</v>
+      </c>
+      <c r="G52">
+        <v>320000</v>
+      </c>
+      <c r="H52">
+        <v>590000</v>
+      </c>
+      <c r="I52">
+        <v>351625</v>
+      </c>
+      <c r="J52" t="str">
+        <v>59.6%</v>
+      </c>
+      <c r="K52">
+        <v>620000</v>
+      </c>
+      <c r="L52">
+        <v>30000</v>
+      </c>
+      <c r="M52" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N52">
+        <v>713000</v>
+      </c>
+      <c r="O52">
+        <v>93000</v>
+      </c>
+      <c r="P52" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C53" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D53" t="str">
+        <v>TK-2882C</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+      </c>
+      <c r="F53">
+        <v>266199</v>
+      </c>
+      <c r="G53">
+        <v>351000</v>
+      </c>
+      <c r="H53">
+        <v>630000</v>
+      </c>
+      <c r="I53">
+        <v>363801</v>
+      </c>
+      <c r="J53" t="str">
+        <v>57.7%</v>
+      </c>
+      <c r="K53">
+        <v>662000</v>
+      </c>
+      <c r="L53">
+        <v>32000</v>
+      </c>
+      <c r="M53" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N53">
+        <v>762000</v>
+      </c>
+      <c r="O53">
+        <v>100000</v>
+      </c>
+      <c r="P53" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C54" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D54" t="str">
+        <v>TK-3030C</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+      </c>
+      <c r="F54">
+        <v>290175</v>
+      </c>
+      <c r="G54">
+        <v>375000</v>
+      </c>
+      <c r="H54">
+        <v>750000</v>
+      </c>
+      <c r="I54">
+        <v>459825</v>
+      </c>
+      <c r="J54" t="str">
+        <v>61.3%</v>
+      </c>
+      <c r="K54">
+        <v>788000</v>
+      </c>
+      <c r="L54">
+        <v>38000</v>
+      </c>
+      <c r="M54" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N54">
+        <v>907000</v>
+      </c>
+      <c r="O54">
+        <v>119000</v>
+      </c>
+      <c r="P54" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C55" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D55" t="str">
+        <v>TK-036A</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F55">
+        <v>433985</v>
+      </c>
+      <c r="G55">
+        <v>495000</v>
+      </c>
+      <c r="H55">
+        <v>891000</v>
+      </c>
+      <c r="I55">
+        <v>457015</v>
+      </c>
+      <c r="J55" t="str">
+        <v>51.3%</v>
+      </c>
+      <c r="K55">
+        <v>936000</v>
+      </c>
+      <c r="L55">
+        <v>45000</v>
+      </c>
+      <c r="M55" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N55">
+        <v>1077000</v>
+      </c>
+      <c r="O55">
+        <v>141000</v>
+      </c>
+      <c r="P55" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C56" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D56" t="str">
+        <v>TK-0318A</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Nồi táo inox cao cấp size18</v>
+      </c>
+      <c r="F56">
+        <v>133166</v>
+      </c>
+      <c r="G56">
+        <v>185000</v>
+      </c>
+      <c r="H56">
+        <v>333000</v>
+      </c>
+      <c r="I56">
+        <v>199834</v>
+      </c>
+      <c r="J56" t="str">
+        <v>60.0%</v>
+      </c>
+      <c r="K56">
+        <v>350000</v>
+      </c>
+      <c r="L56">
+        <v>17000</v>
+      </c>
+      <c r="M56" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N56">
+        <v>403000</v>
+      </c>
+      <c r="O56">
+        <v>53000</v>
+      </c>
+      <c r="P56" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C57" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D57" t="str">
+        <v>TK-0320</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Nồi táo inox cao cấp size20</v>
+      </c>
+      <c r="F57">
+        <v>149800</v>
+      </c>
+      <c r="G57">
+        <v>205000</v>
+      </c>
+      <c r="H57">
+        <v>369000</v>
+      </c>
+      <c r="I57">
+        <v>219200</v>
+      </c>
+      <c r="J57" t="str">
+        <v>59.4%</v>
+      </c>
+      <c r="K57">
+        <v>388000</v>
+      </c>
+      <c r="L57">
+        <v>19000</v>
+      </c>
+      <c r="M57" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N57">
+        <v>447000</v>
+      </c>
+      <c r="O57">
+        <v>59000</v>
+      </c>
+      <c r="P57" t="str">
+        <v>15.2%</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C58" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D58" t="str">
+        <v>TK-0324</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Nồi táo inox cao cấp size24</v>
+      </c>
+      <c r="F58">
+        <v>188524</v>
+      </c>
+      <c r="G58">
+        <v>245000</v>
+      </c>
+      <c r="H58">
+        <v>441000</v>
+      </c>
+      <c r="I58">
+        <v>252476</v>
+      </c>
+      <c r="J58" t="str">
+        <v>57.3%</v>
+      </c>
+      <c r="K58">
+        <v>464000</v>
+      </c>
+      <c r="L58">
+        <v>23000</v>
+      </c>
+      <c r="M58" t="str">
+        <v>5.2%</v>
+      </c>
+      <c r="N58">
+        <v>534000</v>
+      </c>
+      <c r="O58">
+        <v>70000</v>
+      </c>
+      <c r="P58" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C59" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D59" t="str">
+        <v>TK-0348A</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+      </c>
+      <c r="F59">
+        <v>492000</v>
+      </c>
+      <c r="G59">
+        <v>580000</v>
+      </c>
+      <c r="H59">
+        <v>1044000</v>
+      </c>
+      <c r="I59">
+        <v>552000</v>
+      </c>
+      <c r="J59" t="str">
+        <v>52.9%</v>
+      </c>
+      <c r="K59">
+        <v>1097000</v>
+      </c>
+      <c r="L59">
+        <v>53000</v>
+      </c>
+      <c r="M59" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N59">
+        <v>1262000</v>
+      </c>
+      <c r="O59">
+        <v>165000</v>
+      </c>
+      <c r="P59" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C60" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D60" t="str">
+        <v>TK-0369</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F60">
+        <v>419848</v>
+      </c>
+      <c r="G60">
+        <v>535000</v>
+      </c>
+      <c r="H60">
+        <v>969000</v>
+      </c>
+      <c r="I60">
+        <v>549152</v>
+      </c>
+      <c r="J60" t="str">
+        <v>56.7%</v>
+      </c>
+      <c r="K60">
+        <v>1018000</v>
+      </c>
+      <c r="L60">
+        <v>49000</v>
+      </c>
+      <c r="M60" t="str">
+        <v>5.1%</v>
+      </c>
+      <c r="N60">
+        <v>1171000</v>
+      </c>
+      <c r="O60">
+        <v>153000</v>
+      </c>
+      <c r="P60" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C61" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D61" t="str">
+        <v>TK-0488</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F61">
+        <v>672571</v>
+      </c>
+      <c r="G61">
+        <v>810000</v>
+      </c>
+      <c r="H61">
+        <v>1469000</v>
+      </c>
+      <c r="I61">
+        <v>796429</v>
+      </c>
+      <c r="J61" t="str">
+        <v>54.2%</v>
+      </c>
+      <c r="K61">
+        <v>1543000</v>
+      </c>
+      <c r="L61">
+        <v>74000</v>
+      </c>
+      <c r="M61" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N61">
+        <v>1775000</v>
+      </c>
+      <c r="O61">
+        <v>232000</v>
+      </c>
+      <c r="P61" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C62" t="str">
+        <v>NỒI TĂNG ÁP</v>
+      </c>
+      <c r="D62" t="str">
+        <v>TK-0126</v>
+      </c>
+      <c r="E62" t="str">
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) TK 0126</v>
+      </c>
+      <c r="F62">
+        <v>404910</v>
+      </c>
+      <c r="G62">
+        <v>560000</v>
+      </c>
+      <c r="H62">
+        <v>1179000</v>
+      </c>
+      <c r="I62">
+        <v>774090</v>
+      </c>
+      <c r="J62" t="str">
+        <v>65.7%</v>
+      </c>
+      <c r="K62">
+        <v>1238000</v>
+      </c>
+      <c r="L62">
+        <v>59000</v>
+      </c>
+      <c r="M62" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N62">
+        <v>1424000</v>
+      </c>
+      <c r="O62">
+        <v>186000</v>
+      </c>
+      <c r="P62" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C63" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D63" t="str">
+        <v>TK-468</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Sưởi gốm thấp</v>
+      </c>
+      <c r="F63">
+        <v>366857</v>
+      </c>
+      <c r="G63">
+        <v>452000</v>
+      </c>
+      <c r="H63">
+        <v>900000</v>
+      </c>
+      <c r="I63">
+        <v>533143</v>
+      </c>
+      <c r="J63" t="str">
+        <v>59.2%</v>
+      </c>
+      <c r="K63">
+        <v>945000</v>
+      </c>
+      <c r="L63">
+        <v>45000</v>
+      </c>
+      <c r="M63" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N63">
+        <v>1087000</v>
+      </c>
+      <c r="O63">
+        <v>142000</v>
+      </c>
+      <c r="P63" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C64" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D64" t="str">
+        <v>TK-469</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Sưởi gốm thân cao</v>
+      </c>
+      <c r="F64">
+        <v>468762</v>
+      </c>
+      <c r="G64">
+        <v>615000</v>
+      </c>
+      <c r="H64">
+        <v>1050000</v>
+      </c>
+      <c r="I64">
+        <v>581238</v>
+      </c>
+      <c r="J64" t="str">
+        <v>55.4%</v>
+      </c>
+      <c r="K64">
+        <v>1103000</v>
+      </c>
+      <c r="L64">
+        <v>53000</v>
+      </c>
+      <c r="M64" t="str">
+        <v>5.0%</v>
+      </c>
+      <c r="N64">
+        <v>1269000</v>
+      </c>
+      <c r="O64">
+        <v>166000</v>
+      </c>
+      <c r="P64" t="str">
+        <v>15.0%</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C65" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D65" t="str">
+        <v>TK-1002</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
+      </c>
+      <c r="F65">
+        <v>128400</v>
+      </c>
+      <c r="G65">
+        <v>158000</v>
+      </c>
+      <c r="H65">
+        <v>270000</v>
+      </c>
+      <c r="I65">
+        <v>141600</v>
+      </c>
+      <c r="J65" t="str">
+        <v>52.4%</v>
+      </c>
+      <c r="K65">
+        <v>284000</v>
+      </c>
+      <c r="L65">
+        <v>14000</v>
+      </c>
+      <c r="M65" t="str">
+        <v>5.2%</v>
+      </c>
+      <c r="N65">
+        <v>327000</v>
+      </c>
+      <c r="O65">
+        <v>43000</v>
+      </c>
+      <c r="P65" t="str">
+        <v>15.1%</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C66" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D66" t="str">
+        <v>TK-1003</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Bộ đèn sưởi 3 bóng Takin</v>
+      </c>
+      <c r="F66">
+        <v>157290</v>
+      </c>
+      <c r="G66">
+        <v>194000</v>
+      </c>
+      <c r="H66">
+        <v>330000</v>
+      </c>
+      <c r="I66">
+        <v>172710</v>
+      </c>
+      <c r="J66" t="str">
+        <v>52.3%</v>
+      </c>
+      <c r="K66">
+        <v>347000</v>
+      </c>
+      <c r="L66">
+        <v>17000</v>
+      </c>
+      <c r="M66" t="str">
+        <v>5.2%</v>
+      </c>
+      <c r="N66">
+        <v>400000</v>
+      </c>
+      <c r="O66">
+        <v>53000</v>
+      </c>
+      <c r="P66" t="str">
+        <v>15.3%</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:P66"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(pricing): dieu chinh bien loi nhuan Facebook so sanh voi gia NPP Online o Sheet Chenh Lech
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -2778,10 +2778,10 @@
         <v>Giá Facebook (Làm Tròn Nghìn)</v>
       </c>
       <c r="I1" t="str">
-        <v>Lãi FB vs Vốn Nhập (VNĐ)</v>
+        <v>Lợi Nhuận FB vs NPP Online (VNĐ)</v>
       </c>
       <c r="J1" t="str">
-        <v>% Biên LN FB vs Giá Nhập</v>
+        <v>% Biên LN FB / NPP Online</v>
       </c>
       <c r="K1" t="str">
         <v>Giá Sàn TMĐT (+5% FB, Tròn Nghìn)</v>
@@ -2828,10 +2828,10 @@
         <v>467000</v>
       </c>
       <c r="I2">
-        <v>262214</v>
+        <v>202000</v>
       </c>
       <c r="J2" t="str">
-        <v>56.1%</v>
+        <v>43.3%</v>
       </c>
       <c r="K2">
         <v>491000</v>
@@ -2878,10 +2878,10 @@
         <v>649000</v>
       </c>
       <c r="I3">
-        <v>397295</v>
+        <v>289000</v>
       </c>
       <c r="J3" t="str">
-        <v>61.2%</v>
+        <v>44.5%</v>
       </c>
       <c r="K3">
         <v>682000</v>
@@ -2928,10 +2928,10 @@
         <v>750000</v>
       </c>
       <c r="I4">
-        <v>442445</v>
+        <v>355000</v>
       </c>
       <c r="J4" t="str">
-        <v>59.0%</v>
+        <v>47.3%</v>
       </c>
       <c r="K4">
         <v>788000</v>
@@ -2978,10 +2978,10 @@
         <v>690000</v>
       </c>
       <c r="I5">
-        <v>400516</v>
+        <v>300000</v>
       </c>
       <c r="J5" t="str">
-        <v>58.0%</v>
+        <v>43.5%</v>
       </c>
       <c r="K5">
         <v>725000</v>
@@ -3028,10 +3028,10 @@
         <v>590000</v>
       </c>
       <c r="I6">
-        <v>351625</v>
+        <v>270000</v>
       </c>
       <c r="J6" t="str">
-        <v>59.6%</v>
+        <v>45.8%</v>
       </c>
       <c r="K6">
         <v>620000</v>
@@ -3078,10 +3078,10 @@
         <v>850000</v>
       </c>
       <c r="I7">
-        <v>499324</v>
+        <v>400000</v>
       </c>
       <c r="J7" t="str">
-        <v>58.7%</v>
+        <v>47.1%</v>
       </c>
       <c r="K7">
         <v>893000</v>
@@ -3128,10 +3128,10 @@
         <v>630000</v>
       </c>
       <c r="I8">
-        <v>362279</v>
+        <v>279000</v>
       </c>
       <c r="J8" t="str">
-        <v>57.5%</v>
+        <v>44.3%</v>
       </c>
       <c r="K8">
         <v>662000</v>
@@ -3178,10 +3178,10 @@
         <v>642000</v>
       </c>
       <c r="I9">
-        <v>321264</v>
+        <v>272000</v>
       </c>
       <c r="J9" t="str">
-        <v>50.0%</v>
+        <v>42.4%</v>
       </c>
       <c r="K9">
         <v>675000</v>
@@ -3228,10 +3228,10 @@
         <v>760000</v>
       </c>
       <c r="I10">
-        <v>440865</v>
+        <v>329000</v>
       </c>
       <c r="J10" t="str">
-        <v>58.0%</v>
+        <v>43.3%</v>
       </c>
       <c r="K10">
         <v>798000</v>
@@ -3278,10 +3278,10 @@
         <v>740000</v>
       </c>
       <c r="I11">
-        <v>419264</v>
+        <v>328000</v>
       </c>
       <c r="J11" t="str">
-        <v>56.7%</v>
+        <v>44.3%</v>
       </c>
       <c r="K11">
         <v>777000</v>
@@ -3328,10 +3328,10 @@
         <v>750000</v>
       </c>
       <c r="I12">
-        <v>458170</v>
+        <v>375000</v>
       </c>
       <c r="J12" t="str">
-        <v>61.1%</v>
+        <v>50.0%</v>
       </c>
       <c r="K12">
         <v>788000</v>
@@ -3378,10 +3378,10 @@
         <v>1290000</v>
       </c>
       <c r="I13">
-        <v>817568</v>
+        <v>645000</v>
       </c>
       <c r="J13" t="str">
-        <v>63.4%</v>
+        <v>50.0%</v>
       </c>
       <c r="K13">
         <v>1355000</v>
@@ -3428,10 +3428,10 @@
         <v>750000</v>
       </c>
       <c r="I14">
-        <v>413094</v>
+        <v>336000</v>
       </c>
       <c r="J14" t="str">
-        <v>55.1%</v>
+        <v>44.8%</v>
       </c>
       <c r="K14">
         <v>788000</v>
@@ -3478,10 +3478,10 @@
         <v>830000</v>
       </c>
       <c r="I15">
-        <v>429527</v>
+        <v>360000</v>
       </c>
       <c r="J15" t="str">
-        <v>51.8%</v>
+        <v>43.4%</v>
       </c>
       <c r="K15">
         <v>872000</v>
@@ -3528,10 +3528,10 @@
         <v>990000</v>
       </c>
       <c r="I16">
-        <v>578119</v>
+        <v>450000</v>
       </c>
       <c r="J16" t="str">
-        <v>58.4%</v>
+        <v>45.5%</v>
       </c>
       <c r="K16">
         <v>1040000</v>
@@ -3578,10 +3578,10 @@
         <v>295000</v>
       </c>
       <c r="I17">
-        <v>164000</v>
+        <v>125000</v>
       </c>
       <c r="J17" t="str">
-        <v>55.6%</v>
+        <v>42.4%</v>
       </c>
       <c r="K17">
         <v>310000</v>
@@ -3628,10 +3628,10 @@
         <v>315000</v>
       </c>
       <c r="I18">
-        <v>166115</v>
+        <v>130000</v>
       </c>
       <c r="J18" t="str">
-        <v>52.7%</v>
+        <v>41.3%</v>
       </c>
       <c r="K18">
         <v>331000</v>
@@ -3678,10 +3678,10 @@
         <v>395000</v>
       </c>
       <c r="I19">
-        <v>211785</v>
+        <v>165000</v>
       </c>
       <c r="J19" t="str">
-        <v>53.6%</v>
+        <v>41.8%</v>
       </c>
       <c r="K19">
         <v>415000</v>
@@ -3728,10 +3728,10 @@
         <v>689000</v>
       </c>
       <c r="I20">
-        <v>452317</v>
+        <v>364000</v>
       </c>
       <c r="J20" t="str">
-        <v>65.6%</v>
+        <v>52.8%</v>
       </c>
       <c r="K20">
         <v>724000</v>
@@ -3778,10 +3778,10 @@
         <v>779000</v>
       </c>
       <c r="I21">
-        <v>514000</v>
+        <v>439000</v>
       </c>
       <c r="J21" t="str">
-        <v>66.0%</v>
+        <v>56.4%</v>
       </c>
       <c r="K21">
         <v>818000</v>
@@ -3828,10 +3828,10 @@
         <v>889000</v>
       </c>
       <c r="I22">
-        <v>591876</v>
+        <v>499000</v>
       </c>
       <c r="J22" t="str">
-        <v>66.6%</v>
+        <v>56.1%</v>
       </c>
       <c r="K22">
         <v>934000</v>
@@ -3878,10 +3878,10 @@
         <v>1049000</v>
       </c>
       <c r="I23">
-        <v>689263</v>
+        <v>589000</v>
       </c>
       <c r="J23" t="str">
-        <v>65.7%</v>
+        <v>56.1%</v>
       </c>
       <c r="K23">
         <v>1102000</v>
@@ -3928,10 +3928,10 @@
         <v>2090000</v>
       </c>
       <c r="I24">
-        <v>1207000</v>
+        <v>990000</v>
       </c>
       <c r="J24" t="str">
-        <v>57.8%</v>
+        <v>47.4%</v>
       </c>
       <c r="K24">
         <v>2195000</v>
@@ -3978,10 +3978,10 @@
         <v>990000</v>
       </c>
       <c r="I25">
-        <v>536985</v>
+        <v>440000</v>
       </c>
       <c r="J25" t="str">
-        <v>54.2%</v>
+        <v>44.4%</v>
       </c>
       <c r="K25">
         <v>1040000</v>
@@ -4028,10 +4028,10 @@
         <v>1690000</v>
       </c>
       <c r="I26">
-        <v>874333</v>
+        <v>730000</v>
       </c>
       <c r="J26" t="str">
-        <v>51.7%</v>
+        <v>43.2%</v>
       </c>
       <c r="K26">
         <v>1775000</v>
@@ -4078,10 +4078,10 @@
         <v>820000</v>
       </c>
       <c r="I27">
-        <v>462559</v>
+        <v>350000</v>
       </c>
       <c r="J27" t="str">
-        <v>56.4%</v>
+        <v>42.7%</v>
       </c>
       <c r="K27">
         <v>861000</v>
@@ -4128,10 +4128,10 @@
         <v>990000</v>
       </c>
       <c r="I28">
-        <v>602152</v>
+        <v>455000</v>
       </c>
       <c r="J28" t="str">
-        <v>60.8%</v>
+        <v>46.0%</v>
       </c>
       <c r="K28">
         <v>1040000</v>
@@ -4178,10 +4178,10 @@
         <v>549000</v>
       </c>
       <c r="I29">
-        <v>331943</v>
+        <v>274000</v>
       </c>
       <c r="J29" t="str">
-        <v>60.5%</v>
+        <v>49.9%</v>
       </c>
       <c r="K29">
         <v>577000</v>
@@ -4228,10 +4228,10 @@
         <v>525000</v>
       </c>
       <c r="I30">
-        <v>289906</v>
+        <v>225000</v>
       </c>
       <c r="J30" t="str">
-        <v>55.2%</v>
+        <v>42.9%</v>
       </c>
       <c r="K30">
         <v>552000</v>
@@ -4278,10 +4278,10 @@
         <v>1590000</v>
       </c>
       <c r="I31">
-        <v>862400</v>
+        <v>755000</v>
       </c>
       <c r="J31" t="str">
-        <v>54.2%</v>
+        <v>47.5%</v>
       </c>
       <c r="K31">
         <v>1670000</v>
@@ -4328,10 +4328,10 @@
         <v>745000</v>
       </c>
       <c r="I32">
-        <v>378143</v>
+        <v>315000</v>
       </c>
       <c r="J32" t="str">
-        <v>50.8%</v>
+        <v>42.3%</v>
       </c>
       <c r="K32">
         <v>783000</v>
@@ -4378,10 +4378,10 @@
         <v>1050000</v>
       </c>
       <c r="I33">
-        <v>581238</v>
+        <v>465000</v>
       </c>
       <c r="J33" t="str">
-        <v>55.4%</v>
+        <v>44.3%</v>
       </c>
       <c r="K33">
         <v>1103000</v>
@@ -4428,10 +4428,10 @@
         <v>920000</v>
       </c>
       <c r="I34">
-        <v>524100</v>
+        <v>460000</v>
       </c>
       <c r="J34" t="str">
-        <v>57.0%</v>
+        <v>50.0%</v>
       </c>
       <c r="K34">
         <v>966000</v>
@@ -4478,10 +4478,10 @@
         <v>1690000</v>
       </c>
       <c r="I35">
-        <v>962400</v>
+        <v>840000</v>
       </c>
       <c r="J35" t="str">
-        <v>56.9%</v>
+        <v>49.7%</v>
       </c>
       <c r="K35">
         <v>1775000</v>
@@ -4528,10 +4528,10 @@
         <v>354000</v>
       </c>
       <c r="I36">
-        <v>186010</v>
+        <v>157000</v>
       </c>
       <c r="J36" t="str">
-        <v>52.5%</v>
+        <v>44.4%</v>
       </c>
       <c r="K36">
         <v>372000</v>
@@ -4578,10 +4578,10 @@
         <v>1890000</v>
       </c>
       <c r="I37">
-        <v>1094592</v>
+        <v>870000</v>
       </c>
       <c r="J37" t="str">
-        <v>57.9%</v>
+        <v>46.0%</v>
       </c>
       <c r="K37">
         <v>1985000</v>
@@ -4628,10 +4628,10 @@
         <v>670000</v>
       </c>
       <c r="I38">
-        <v>363980</v>
+        <v>298000</v>
       </c>
       <c r="J38" t="str">
-        <v>54.3%</v>
+        <v>44.5%</v>
       </c>
       <c r="K38">
         <v>704000</v>
@@ -4678,10 +4678,10 @@
         <v>1495000</v>
       </c>
       <c r="I39">
-        <v>826843</v>
+        <v>715000</v>
       </c>
       <c r="J39" t="str">
-        <v>55.3%</v>
+        <v>47.8%</v>
       </c>
       <c r="K39">
         <v>1570000</v>
@@ -4728,10 +4728,10 @@
         <v>599000</v>
       </c>
       <c r="I40">
-        <v>339451</v>
+        <v>289000</v>
       </c>
       <c r="J40" t="str">
-        <v>56.7%</v>
+        <v>48.2%</v>
       </c>
       <c r="K40">
         <v>629000</v>
@@ -4778,10 +4778,10 @@
         <v>850000</v>
       </c>
       <c r="I41">
-        <v>500000</v>
+        <v>410000</v>
       </c>
       <c r="J41" t="str">
-        <v>58.8%</v>
+        <v>48.2%</v>
       </c>
       <c r="K41">
         <v>893000</v>
@@ -4828,10 +4828,10 @@
         <v>2350000</v>
       </c>
       <c r="I42">
-        <v>1521514</v>
+        <v>1350000</v>
       </c>
       <c r="J42" t="str">
-        <v>64.7%</v>
+        <v>57.4%</v>
       </c>
       <c r="K42">
         <v>2468000</v>
@@ -4878,10 +4878,10 @@
         <v>1650000</v>
       </c>
       <c r="I43">
-        <v>977429</v>
+        <v>850000</v>
       </c>
       <c r="J43" t="str">
-        <v>59.2%</v>
+        <v>51.5%</v>
       </c>
       <c r="K43">
         <v>1733000</v>
@@ -4928,10 +4928,10 @@
         <v>950000</v>
       </c>
       <c r="I44">
-        <v>550013</v>
+        <v>440000</v>
       </c>
       <c r="J44" t="str">
-        <v>57.9%</v>
+        <v>46.3%</v>
       </c>
       <c r="K44">
         <v>998000</v>
@@ -4978,10 +4978,10 @@
         <v>950000</v>
       </c>
       <c r="I45">
-        <v>560459</v>
+        <v>440000</v>
       </c>
       <c r="J45" t="str">
-        <v>59.0%</v>
+        <v>46.3%</v>
       </c>
       <c r="K45">
         <v>998000</v>
@@ -5028,10 +5028,10 @@
         <v>1190000</v>
       </c>
       <c r="I46">
-        <v>721238</v>
+        <v>590000</v>
       </c>
       <c r="J46" t="str">
-        <v>60.6%</v>
+        <v>49.6%</v>
       </c>
       <c r="K46">
         <v>1250000</v>
@@ -5078,10 +5078,10 @@
         <v>490000</v>
       </c>
       <c r="I47">
-        <v>289248</v>
+        <v>230000</v>
       </c>
       <c r="J47" t="str">
-        <v>59.0%</v>
+        <v>46.9%</v>
       </c>
       <c r="K47">
         <v>515000</v>
@@ -5128,10 +5128,10 @@
         <v>1290000</v>
       </c>
       <c r="I48">
-        <v>739953</v>
+        <v>605000</v>
       </c>
       <c r="J48" t="str">
-        <v>57.4%</v>
+        <v>46.9%</v>
       </c>
       <c r="K48">
         <v>1355000</v>
@@ -5178,10 +5178,10 @@
         <v>1190000</v>
       </c>
       <c r="I49">
-        <v>644396</v>
+        <v>530000</v>
       </c>
       <c r="J49" t="str">
-        <v>54.2%</v>
+        <v>44.5%</v>
       </c>
       <c r="K49">
         <v>1250000</v>
@@ -5228,10 +5228,10 @@
         <v>2190000</v>
       </c>
       <c r="I50">
-        <v>1253750</v>
+        <v>1060000</v>
       </c>
       <c r="J50" t="str">
-        <v>57.2%</v>
+        <v>48.4%</v>
       </c>
       <c r="K50">
         <v>2300000</v>
@@ -5278,10 +5278,10 @@
         <v>467000</v>
       </c>
       <c r="I51">
-        <v>263366</v>
+        <v>202000</v>
       </c>
       <c r="J51" t="str">
-        <v>56.4%</v>
+        <v>43.3%</v>
       </c>
       <c r="K51">
         <v>491000</v>
@@ -5328,10 +5328,10 @@
         <v>590000</v>
       </c>
       <c r="I52">
-        <v>351625</v>
+        <v>270000</v>
       </c>
       <c r="J52" t="str">
-        <v>59.6%</v>
+        <v>45.8%</v>
       </c>
       <c r="K52">
         <v>620000</v>
@@ -5378,10 +5378,10 @@
         <v>630000</v>
       </c>
       <c r="I53">
-        <v>363801</v>
+        <v>279000</v>
       </c>
       <c r="J53" t="str">
-        <v>57.7%</v>
+        <v>44.3%</v>
       </c>
       <c r="K53">
         <v>662000</v>
@@ -5428,10 +5428,10 @@
         <v>750000</v>
       </c>
       <c r="I54">
-        <v>459825</v>
+        <v>375000</v>
       </c>
       <c r="J54" t="str">
-        <v>61.3%</v>
+        <v>50.0%</v>
       </c>
       <c r="K54">
         <v>788000</v>
@@ -5478,10 +5478,10 @@
         <v>891000</v>
       </c>
       <c r="I55">
-        <v>457015</v>
+        <v>396000</v>
       </c>
       <c r="J55" t="str">
-        <v>51.3%</v>
+        <v>44.4%</v>
       </c>
       <c r="K55">
         <v>936000</v>
@@ -5528,10 +5528,10 @@
         <v>333000</v>
       </c>
       <c r="I56">
-        <v>199834</v>
+        <v>148000</v>
       </c>
       <c r="J56" t="str">
-        <v>60.0%</v>
+        <v>44.4%</v>
       </c>
       <c r="K56">
         <v>350000</v>
@@ -5578,10 +5578,10 @@
         <v>369000</v>
       </c>
       <c r="I57">
-        <v>219200</v>
+        <v>164000</v>
       </c>
       <c r="J57" t="str">
-        <v>59.4%</v>
+        <v>44.4%</v>
       </c>
       <c r="K57">
         <v>388000</v>
@@ -5628,10 +5628,10 @@
         <v>441000</v>
       </c>
       <c r="I58">
-        <v>252476</v>
+        <v>196000</v>
       </c>
       <c r="J58" t="str">
-        <v>57.3%</v>
+        <v>44.4%</v>
       </c>
       <c r="K58">
         <v>464000</v>
@@ -5678,10 +5678,10 @@
         <v>1044000</v>
       </c>
       <c r="I59">
-        <v>552000</v>
+        <v>464000</v>
       </c>
       <c r="J59" t="str">
-        <v>52.9%</v>
+        <v>44.4%</v>
       </c>
       <c r="K59">
         <v>1097000</v>
@@ -5728,10 +5728,10 @@
         <v>969000</v>
       </c>
       <c r="I60">
-        <v>549152</v>
+        <v>434000</v>
       </c>
       <c r="J60" t="str">
-        <v>56.7%</v>
+        <v>44.8%</v>
       </c>
       <c r="K60">
         <v>1018000</v>
@@ -5778,10 +5778,10 @@
         <v>1469000</v>
       </c>
       <c r="I61">
-        <v>796429</v>
+        <v>659000</v>
       </c>
       <c r="J61" t="str">
-        <v>54.2%</v>
+        <v>44.9%</v>
       </c>
       <c r="K61">
         <v>1543000</v>
@@ -5828,10 +5828,10 @@
         <v>1179000</v>
       </c>
       <c r="I62">
-        <v>774090</v>
+        <v>619000</v>
       </c>
       <c r="J62" t="str">
-        <v>65.7%</v>
+        <v>52.5%</v>
       </c>
       <c r="K62">
         <v>1238000</v>
@@ -5878,10 +5878,10 @@
         <v>900000</v>
       </c>
       <c r="I63">
-        <v>533143</v>
+        <v>448000</v>
       </c>
       <c r="J63" t="str">
-        <v>59.2%</v>
+        <v>49.8%</v>
       </c>
       <c r="K63">
         <v>945000</v>
@@ -5928,10 +5928,10 @@
         <v>1050000</v>
       </c>
       <c r="I64">
-        <v>581238</v>
+        <v>435000</v>
       </c>
       <c r="J64" t="str">
-        <v>55.4%</v>
+        <v>41.4%</v>
       </c>
       <c r="K64">
         <v>1103000</v>
@@ -5978,10 +5978,10 @@
         <v>270000</v>
       </c>
       <c r="I65">
-        <v>141600</v>
+        <v>112000</v>
       </c>
       <c r="J65" t="str">
-        <v>52.4%</v>
+        <v>41.5%</v>
       </c>
       <c r="K65">
         <v>284000</v>
@@ -6028,10 +6028,10 @@
         <v>330000</v>
       </c>
       <c r="I66">
-        <v>172710</v>
+        <v>136000</v>
       </c>
       <c r="J66" t="str">
-        <v>52.3%</v>
+        <v>41.2%</v>
       </c>
       <c r="K66">
         <v>347000</v>

</xml_diff>

<commit_message>
fix(ui): an cot Bien Do Niem Yet vs TMDT trong Sheet Chenh Lech Gia
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -2732,7 +2732,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P66"/>
+  <dimension ref="A1:N66"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2795,12 +2795,6 @@
       <c r="N1" t="str">
         <v>Giá Niêm Yết (+15% TMĐT, Tròn Nghìn)</v>
       </c>
-      <c r="O1" t="str">
-        <v>Chênh Lệch Niêm Yết vs TMĐT (VNĐ)</v>
-      </c>
-      <c r="P1" t="str">
-        <v>% Biên Độ Niêm Yết vs TMĐT</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -2845,12 +2839,6 @@
       <c r="N2">
         <v>565000</v>
       </c>
-      <c r="O2">
-        <v>74000</v>
-      </c>
-      <c r="P2" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -2895,12 +2883,6 @@
       <c r="N3">
         <v>785000</v>
       </c>
-      <c r="O3">
-        <v>103000</v>
-      </c>
-      <c r="P3" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -2945,12 +2927,6 @@
       <c r="N4">
         <v>907000</v>
       </c>
-      <c r="O4">
-        <v>119000</v>
-      </c>
-      <c r="P4" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -2995,12 +2971,6 @@
       <c r="N5">
         <v>834000</v>
       </c>
-      <c r="O5">
-        <v>109000</v>
-      </c>
-      <c r="P5" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -3045,12 +3015,6 @@
       <c r="N6">
         <v>713000</v>
       </c>
-      <c r="O6">
-        <v>93000</v>
-      </c>
-      <c r="P6" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -3095,12 +3059,6 @@
       <c r="N7">
         <v>1027000</v>
       </c>
-      <c r="O7">
-        <v>134000</v>
-      </c>
-      <c r="P7" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -3145,12 +3103,6 @@
       <c r="N8">
         <v>762000</v>
       </c>
-      <c r="O8">
-        <v>100000</v>
-      </c>
-      <c r="P8" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -3195,12 +3147,6 @@
       <c r="N9">
         <v>777000</v>
       </c>
-      <c r="O9">
-        <v>102000</v>
-      </c>
-      <c r="P9" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -3245,12 +3191,6 @@
       <c r="N10">
         <v>918000</v>
       </c>
-      <c r="O10">
-        <v>120000</v>
-      </c>
-      <c r="P10" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -3295,12 +3235,6 @@
       <c r="N11">
         <v>894000</v>
       </c>
-      <c r="O11">
-        <v>117000</v>
-      </c>
-      <c r="P11" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -3345,12 +3279,6 @@
       <c r="N12">
         <v>907000</v>
       </c>
-      <c r="O12">
-        <v>119000</v>
-      </c>
-      <c r="P12" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -3395,12 +3323,6 @@
       <c r="N13">
         <v>1559000</v>
       </c>
-      <c r="O13">
-        <v>204000</v>
-      </c>
-      <c r="P13" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -3445,12 +3367,6 @@
       <c r="N14">
         <v>907000</v>
       </c>
-      <c r="O14">
-        <v>119000</v>
-      </c>
-      <c r="P14" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -3495,12 +3411,6 @@
       <c r="N15">
         <v>1003000</v>
       </c>
-      <c r="O15">
-        <v>131000</v>
-      </c>
-      <c r="P15" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -3545,12 +3455,6 @@
       <c r="N16">
         <v>1196000</v>
       </c>
-      <c r="O16">
-        <v>156000</v>
-      </c>
-      <c r="P16" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -3595,12 +3499,6 @@
       <c r="N17">
         <v>357000</v>
       </c>
-      <c r="O17">
-        <v>47000</v>
-      </c>
-      <c r="P17" t="str">
-        <v>15.2%</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -3645,12 +3543,6 @@
       <c r="N18">
         <v>381000</v>
       </c>
-      <c r="O18">
-        <v>50000</v>
-      </c>
-      <c r="P18" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -3695,12 +3587,6 @@
       <c r="N19">
         <v>478000</v>
       </c>
-      <c r="O19">
-        <v>63000</v>
-      </c>
-      <c r="P19" t="str">
-        <v>15.2%</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -3745,12 +3631,6 @@
       <c r="N20">
         <v>833000</v>
       </c>
-      <c r="O20">
-        <v>109000</v>
-      </c>
-      <c r="P20" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -3795,12 +3675,6 @@
       <c r="N21">
         <v>941000</v>
       </c>
-      <c r="O21">
-        <v>123000</v>
-      </c>
-      <c r="P21" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -3845,12 +3719,6 @@
       <c r="N22">
         <v>1075000</v>
       </c>
-      <c r="O22">
-        <v>141000</v>
-      </c>
-      <c r="P22" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -3895,12 +3763,6 @@
       <c r="N23">
         <v>1268000</v>
       </c>
-      <c r="O23">
-        <v>166000</v>
-      </c>
-      <c r="P23" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -3945,12 +3807,6 @@
       <c r="N24">
         <v>2525000</v>
       </c>
-      <c r="O24">
-        <v>330000</v>
-      </c>
-      <c r="P24" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -3995,12 +3851,6 @@
       <c r="N25">
         <v>1196000</v>
       </c>
-      <c r="O25">
-        <v>156000</v>
-      </c>
-      <c r="P25" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -4045,12 +3895,6 @@
       <c r="N26">
         <v>2042000</v>
       </c>
-      <c r="O26">
-        <v>267000</v>
-      </c>
-      <c r="P26" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -4095,12 +3939,6 @@
       <c r="N27">
         <v>991000</v>
       </c>
-      <c r="O27">
-        <v>130000</v>
-      </c>
-      <c r="P27" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -4145,12 +3983,6 @@
       <c r="N28">
         <v>1196000</v>
       </c>
-      <c r="O28">
-        <v>156000</v>
-      </c>
-      <c r="P28" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -4195,12 +4027,6 @@
       <c r="N29">
         <v>664000</v>
       </c>
-      <c r="O29">
-        <v>87000</v>
-      </c>
-      <c r="P29" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -4245,12 +4071,6 @@
       <c r="N30">
         <v>635000</v>
       </c>
-      <c r="O30">
-        <v>83000</v>
-      </c>
-      <c r="P30" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -4295,12 +4115,6 @@
       <c r="N31">
         <v>1921000</v>
       </c>
-      <c r="O31">
-        <v>251000</v>
-      </c>
-      <c r="P31" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -4345,12 +4159,6 @@
       <c r="N32">
         <v>901000</v>
       </c>
-      <c r="O32">
-        <v>118000</v>
-      </c>
-      <c r="P32" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -4395,12 +4203,6 @@
       <c r="N33">
         <v>1269000</v>
       </c>
-      <c r="O33">
-        <v>166000</v>
-      </c>
-      <c r="P33" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -4445,12 +4247,6 @@
       <c r="N34">
         <v>1111000</v>
       </c>
-      <c r="O34">
-        <v>145000</v>
-      </c>
-      <c r="P34" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -4495,12 +4291,6 @@
       <c r="N35">
         <v>2042000</v>
       </c>
-      <c r="O35">
-        <v>267000</v>
-      </c>
-      <c r="P35" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -4545,12 +4335,6 @@
       <c r="N36">
         <v>428000</v>
       </c>
-      <c r="O36">
-        <v>56000</v>
-      </c>
-      <c r="P36" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -4595,12 +4379,6 @@
       <c r="N37">
         <v>2283000</v>
       </c>
-      <c r="O37">
-        <v>298000</v>
-      </c>
-      <c r="P37" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -4645,12 +4423,6 @@
       <c r="N38">
         <v>810000</v>
       </c>
-      <c r="O38">
-        <v>106000</v>
-      </c>
-      <c r="P38" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -4695,12 +4467,6 @@
       <c r="N39">
         <v>1806000</v>
       </c>
-      <c r="O39">
-        <v>236000</v>
-      </c>
-      <c r="P39" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -4745,12 +4511,6 @@
       <c r="N40">
         <v>724000</v>
       </c>
-      <c r="O40">
-        <v>95000</v>
-      </c>
-      <c r="P40" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -4795,12 +4555,6 @@
       <c r="N41">
         <v>1027000</v>
       </c>
-      <c r="O41">
-        <v>134000</v>
-      </c>
-      <c r="P41" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -4845,12 +4599,6 @@
       <c r="N42">
         <v>2839000</v>
       </c>
-      <c r="O42">
-        <v>371000</v>
-      </c>
-      <c r="P42" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -4895,12 +4643,6 @@
       <c r="N43">
         <v>1993000</v>
       </c>
-      <c r="O43">
-        <v>260000</v>
-      </c>
-      <c r="P43" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -4945,12 +4687,6 @@
       <c r="N44">
         <v>1148000</v>
       </c>
-      <c r="O44">
-        <v>150000</v>
-      </c>
-      <c r="P44" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -4995,12 +4731,6 @@
       <c r="N45">
         <v>1148000</v>
       </c>
-      <c r="O45">
-        <v>150000</v>
-      </c>
-      <c r="P45" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -5045,12 +4775,6 @@
       <c r="N46">
         <v>1438000</v>
       </c>
-      <c r="O46">
-        <v>188000</v>
-      </c>
-      <c r="P46" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -5095,12 +4819,6 @@
       <c r="N47">
         <v>593000</v>
       </c>
-      <c r="O47">
-        <v>78000</v>
-      </c>
-      <c r="P47" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -5145,12 +4863,6 @@
       <c r="N48">
         <v>1559000</v>
       </c>
-      <c r="O48">
-        <v>204000</v>
-      </c>
-      <c r="P48" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -5195,12 +4907,6 @@
       <c r="N49">
         <v>1438000</v>
       </c>
-      <c r="O49">
-        <v>188000</v>
-      </c>
-      <c r="P49" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -5245,12 +4951,6 @@
       <c r="N50">
         <v>2645000</v>
       </c>
-      <c r="O50">
-        <v>345000</v>
-      </c>
-      <c r="P50" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -5295,12 +4995,6 @@
       <c r="N51">
         <v>565000</v>
       </c>
-      <c r="O51">
-        <v>74000</v>
-      </c>
-      <c r="P51" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -5345,12 +5039,6 @@
       <c r="N52">
         <v>713000</v>
       </c>
-      <c r="O52">
-        <v>93000</v>
-      </c>
-      <c r="P52" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -5395,12 +5083,6 @@
       <c r="N53">
         <v>762000</v>
       </c>
-      <c r="O53">
-        <v>100000</v>
-      </c>
-      <c r="P53" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -5445,12 +5127,6 @@
       <c r="N54">
         <v>907000</v>
       </c>
-      <c r="O54">
-        <v>119000</v>
-      </c>
-      <c r="P54" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -5495,12 +5171,6 @@
       <c r="N55">
         <v>1077000</v>
       </c>
-      <c r="O55">
-        <v>141000</v>
-      </c>
-      <c r="P55" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -5545,12 +5215,6 @@
       <c r="N56">
         <v>403000</v>
       </c>
-      <c r="O56">
-        <v>53000</v>
-      </c>
-      <c r="P56" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -5595,12 +5259,6 @@
       <c r="N57">
         <v>447000</v>
       </c>
-      <c r="O57">
-        <v>59000</v>
-      </c>
-      <c r="P57" t="str">
-        <v>15.2%</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -5645,12 +5303,6 @@
       <c r="N58">
         <v>534000</v>
       </c>
-      <c r="O58">
-        <v>70000</v>
-      </c>
-      <c r="P58" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -5695,12 +5347,6 @@
       <c r="N59">
         <v>1262000</v>
       </c>
-      <c r="O59">
-        <v>165000</v>
-      </c>
-      <c r="P59" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -5745,12 +5391,6 @@
       <c r="N60">
         <v>1171000</v>
       </c>
-      <c r="O60">
-        <v>153000</v>
-      </c>
-      <c r="P60" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -5795,12 +5435,6 @@
       <c r="N61">
         <v>1775000</v>
       </c>
-      <c r="O61">
-        <v>232000</v>
-      </c>
-      <c r="P61" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -5845,12 +5479,6 @@
       <c r="N62">
         <v>1424000</v>
       </c>
-      <c r="O62">
-        <v>186000</v>
-      </c>
-      <c r="P62" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -5895,12 +5523,6 @@
       <c r="N63">
         <v>1087000</v>
       </c>
-      <c r="O63">
-        <v>142000</v>
-      </c>
-      <c r="P63" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -5945,12 +5567,6 @@
       <c r="N64">
         <v>1269000</v>
       </c>
-      <c r="O64">
-        <v>166000</v>
-      </c>
-      <c r="P64" t="str">
-        <v>15.0%</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -5995,12 +5611,6 @@
       <c r="N65">
         <v>327000</v>
       </c>
-      <c r="O65">
-        <v>43000</v>
-      </c>
-      <c r="P65" t="str">
-        <v>15.1%</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -6045,16 +5655,10 @@
       <c r="N66">
         <v>400000</v>
       </c>
-      <c r="O66">
-        <v>53000</v>
-      </c>
-      <c r="P66" t="str">
-        <v>15.3%</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N66"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(catalog): loai bo ma LK-2466S (he thong con 56 ma: 43 Lock&King + 13 Takin)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Bang_Gia_Chuan_57_Ma" sheetId="1" r:id="rId1"/>
+    <sheet name="Bang_Gia_Chuan_56_Ma" sheetId="1" r:id="rId1"/>
     <sheet name="ChenhLech_Gia_FB_TMDT_NY" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K57"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -529,28 +529,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D4" t="str">
-        <v>LK-2466S</v>
+        <v>LK-2606A</v>
       </c>
       <c r="E4" t="str">
-        <v>Chảo Titanium  ELITE Lock&amp;King</v>
+        <v>Chảo cạn Titanium Lock&amp;king 26cm</v>
       </c>
       <c r="F4">
-        <v>390000</v>
+        <v>320000</v>
       </c>
       <c r="G4">
-        <v>690000</v>
+        <v>590000</v>
       </c>
       <c r="H4">
-        <v>725000</v>
+        <v>637200</v>
       </c>
       <c r="I4">
-        <v>990000</v>
+        <v>767000</v>
       </c>
       <c r="J4">
-        <v>300000</v>
+        <v>270000</v>
       </c>
       <c r="K4" t="str">
-        <v>43.5%</v>
+        <v>45.8%</v>
       </c>
     </row>
     <row r="5">
@@ -564,28 +564,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D5" t="str">
-        <v>LK-2606A</v>
+        <v>LK-2633</v>
       </c>
       <c r="E5" t="str">
-        <v>Chảo cạn Titanium Lock&amp;king 26cm</v>
+        <v>Chảo Belly Lock&amp;King Titanium 26cm</v>
       </c>
       <c r="F5">
-        <v>320000</v>
+        <v>450000</v>
       </c>
       <c r="G5">
-        <v>590000</v>
+        <v>850000</v>
       </c>
       <c r="H5">
-        <v>637200</v>
+        <v>961200</v>
       </c>
       <c r="I5">
-        <v>767000</v>
+        <v>1200000</v>
       </c>
       <c r="J5">
-        <v>270000</v>
+        <v>400000</v>
       </c>
       <c r="K5" t="str">
-        <v>45.8%</v>
+        <v>47.1%</v>
       </c>
     </row>
     <row r="6">
@@ -599,28 +599,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D6" t="str">
-        <v>LK-2633</v>
+        <v>LK-2808</v>
       </c>
       <c r="E6" t="str">
-        <v>Chảo Belly Lock&amp;King Titanium 26cm</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F6">
-        <v>450000</v>
+        <v>351000</v>
       </c>
       <c r="G6">
-        <v>850000</v>
+        <v>630000</v>
       </c>
       <c r="H6">
-        <v>961200</v>
+        <v>680400</v>
       </c>
       <c r="I6">
-        <v>1200000</v>
+        <v>819000</v>
       </c>
       <c r="J6">
-        <v>400000</v>
+        <v>279000</v>
       </c>
       <c r="K6" t="str">
-        <v>47.1%</v>
+        <v>44.3%</v>
       </c>
     </row>
     <row r="7">
@@ -634,25 +634,25 @@
         <v>CHẢO</v>
       </c>
       <c r="D7" t="str">
-        <v>LK-2808</v>
+        <v>LK-2808SA KHÔNG NẮP</v>
       </c>
       <c r="E7" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA KHÔNG NẮP</v>
       </c>
       <c r="F7">
-        <v>351000</v>
+        <v>412000</v>
       </c>
       <c r="G7">
-        <v>630000</v>
+        <v>740000</v>
       </c>
       <c r="H7">
-        <v>680400</v>
+        <v>799200</v>
       </c>
       <c r="I7">
-        <v>819000</v>
+        <v>962000</v>
       </c>
       <c r="J7">
-        <v>279000</v>
+        <v>328000</v>
       </c>
       <c r="K7" t="str">
         <v>44.3%</v>
@@ -669,28 +669,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D8" t="str">
-        <v>LK-2808SA KHÔNG NẮP</v>
+        <v>LK-3003</v>
       </c>
       <c r="E8" t="str">
-        <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA KHÔNG NẮP</v>
+        <v>Chảo cạn titanium Lock&amp;King 30cm</v>
       </c>
       <c r="F8">
-        <v>412000</v>
+        <v>375000</v>
       </c>
       <c r="G8">
-        <v>740000</v>
+        <v>750000</v>
       </c>
       <c r="H8">
-        <v>799200</v>
+        <v>788000</v>
       </c>
       <c r="I8">
-        <v>962000</v>
+        <v>825000</v>
       </c>
       <c r="J8">
-        <v>328000</v>
+        <v>375000</v>
       </c>
       <c r="K8" t="str">
-        <v>44.3%</v>
+        <v>50.0%</v>
       </c>
     </row>
     <row r="9">
@@ -704,25 +704,25 @@
         <v>CHẢO</v>
       </c>
       <c r="D9" t="str">
-        <v>LK-3003</v>
+        <v>LK-3212</v>
       </c>
       <c r="E9" t="str">
-        <v>Chảo cạn titanium Lock&amp;King 30cm</v>
+        <v>Chảo xào lớn</v>
       </c>
       <c r="F9">
-        <v>375000</v>
+        <v>645000</v>
       </c>
       <c r="G9">
-        <v>750000</v>
+        <v>1290000</v>
       </c>
       <c r="H9">
-        <v>788000</v>
+        <v>1380300</v>
       </c>
       <c r="I9">
-        <v>825000</v>
+        <v>1548000</v>
       </c>
       <c r="J9">
-        <v>375000</v>
+        <v>645000</v>
       </c>
       <c r="K9" t="str">
         <v>50.0%</v>
@@ -736,31 +736,31 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C10" t="str">
-        <v>CHẢO</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D10" t="str">
-        <v>LK-3212</v>
+        <v>LK-30NC1</v>
       </c>
       <c r="E10" t="str">
-        <v>Chảo xào lớn</v>
+        <v>Nồi luộc gà Lock&amp;King size 30</v>
       </c>
       <c r="F10">
-        <v>645000</v>
+        <v>414000</v>
       </c>
       <c r="G10">
-        <v>1290000</v>
+        <v>750000</v>
       </c>
       <c r="H10">
-        <v>1380300</v>
+        <v>810000</v>
       </c>
       <c r="I10">
-        <v>1548000</v>
+        <v>975000</v>
       </c>
       <c r="J10">
-        <v>645000</v>
+        <v>336000</v>
       </c>
       <c r="K10" t="str">
-        <v>50.0%</v>
+        <v>44.8%</v>
       </c>
     </row>
     <row r="11">
@@ -774,28 +774,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D11" t="str">
-        <v>LK-30NC1</v>
+        <v>LK-32NC1</v>
       </c>
       <c r="E11" t="str">
-        <v>Nồi luộc gà Lock&amp;King size 30</v>
+        <v>Nồi luộc gà Lock&amp;King size 32</v>
       </c>
       <c r="F11">
-        <v>414000</v>
+        <v>470000</v>
       </c>
       <c r="G11">
-        <v>750000</v>
+        <v>830000</v>
       </c>
       <c r="H11">
-        <v>810000</v>
+        <v>896400</v>
       </c>
       <c r="I11">
-        <v>975000</v>
+        <v>1079000</v>
       </c>
       <c r="J11">
-        <v>336000</v>
+        <v>360000</v>
       </c>
       <c r="K11" t="str">
-        <v>44.8%</v>
+        <v>43.4%</v>
       </c>
     </row>
     <row r="12">
@@ -809,28 +809,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D12" t="str">
-        <v>LK-32NC1</v>
+        <v>LK-336A</v>
       </c>
       <c r="E12" t="str">
-        <v>Nồi luộc gà Lock&amp;King size 32</v>
+        <v>Bộ nồi 3 Lock&amp;King ( 18,20,24 )</v>
       </c>
       <c r="F12">
-        <v>470000</v>
+        <v>540000</v>
       </c>
       <c r="G12">
-        <v>830000</v>
+        <v>990000</v>
       </c>
       <c r="H12">
-        <v>896400</v>
+        <v>1069200</v>
       </c>
       <c r="I12">
-        <v>1079000</v>
+        <v>1287000</v>
       </c>
       <c r="J12">
-        <v>360000</v>
+        <v>450000</v>
       </c>
       <c r="K12" t="str">
-        <v>43.4%</v>
+        <v>45.5%</v>
       </c>
     </row>
     <row r="13">
@@ -844,28 +844,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D13" t="str">
-        <v>LK-336A</v>
+        <v>LK-3018A</v>
       </c>
       <c r="E13" t="str">
-        <v>Bộ nồi 3 Lock&amp;King ( 18,20,24 )</v>
+        <v>Nồi lẻ Lock&amp;king 18</v>
       </c>
       <c r="F13">
-        <v>540000</v>
+        <v>170000</v>
       </c>
       <c r="G13">
-        <v>990000</v>
+        <v>295000</v>
       </c>
       <c r="H13">
-        <v>1069200</v>
+        <v>324500</v>
       </c>
       <c r="I13">
-        <v>1287000</v>
+        <v>383500</v>
       </c>
       <c r="J13">
-        <v>450000</v>
+        <v>125000</v>
       </c>
       <c r="K13" t="str">
-        <v>45.5%</v>
+        <v>42.4%</v>
       </c>
     </row>
     <row r="14">
@@ -879,28 +879,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D14" t="str">
-        <v>LK-3018A</v>
+        <v>LK-3020A</v>
       </c>
       <c r="E14" t="str">
-        <v>Nồi lẻ Lock&amp;king 18</v>
+        <v>Nồi lẻ Lock&amp;king 20</v>
       </c>
       <c r="F14">
-        <v>170000</v>
+        <v>185000</v>
       </c>
       <c r="G14">
-        <v>295000</v>
+        <v>315000</v>
       </c>
       <c r="H14">
-        <v>324500</v>
+        <v>346500</v>
       </c>
       <c r="I14">
-        <v>383500</v>
+        <v>409500</v>
       </c>
       <c r="J14">
-        <v>125000</v>
+        <v>130000</v>
       </c>
       <c r="K14" t="str">
-        <v>42.4%</v>
+        <v>41.3%</v>
       </c>
     </row>
     <row r="15">
@@ -914,28 +914,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D15" t="str">
-        <v>LK-3020A</v>
+        <v>LK-3024</v>
       </c>
       <c r="E15" t="str">
-        <v>Nồi lẻ Lock&amp;king 20</v>
+        <v>Nồi lẻ Lock&amp;king 24</v>
       </c>
       <c r="F15">
-        <v>185000</v>
+        <v>230000</v>
       </c>
       <c r="G15">
-        <v>315000</v>
+        <v>395000</v>
       </c>
       <c r="H15">
-        <v>346500</v>
+        <v>434500</v>
       </c>
       <c r="I15">
-        <v>409500</v>
+        <v>513500</v>
       </c>
       <c r="J15">
-        <v>130000</v>
+        <v>165000</v>
       </c>
       <c r="K15" t="str">
-        <v>41.3%</v>
+        <v>41.8%</v>
       </c>
     </row>
     <row r="16">
@@ -949,28 +949,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D16" t="str">
-        <v>LK-3024</v>
+        <v>LK-3116</v>
       </c>
       <c r="E16" t="str">
-        <v>Nồi lẻ Lock&amp;king 24</v>
+        <v>16*9CM Quánh liền khối titan (2.2mm) LK-3116</v>
       </c>
       <c r="F16">
-        <v>230000</v>
+        <v>325000</v>
       </c>
       <c r="G16">
-        <v>395000</v>
+        <v>689000</v>
       </c>
       <c r="H16">
-        <v>434500</v>
+        <v>744120</v>
       </c>
       <c r="I16">
-        <v>513500</v>
+        <v>895700</v>
       </c>
       <c r="J16">
-        <v>165000</v>
+        <v>364000</v>
       </c>
       <c r="K16" t="str">
-        <v>41.8%</v>
+        <v>52.8%</v>
       </c>
     </row>
     <row r="17">
@@ -984,28 +984,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D17" t="str">
-        <v>LK-3116</v>
+        <v>LK-3118</v>
       </c>
       <c r="E17" t="str">
-        <v>16*9CM Quánh liền khối titan (2.2mm) LK-3116</v>
+        <v>18*10CM Nồi lẻ kèm nắp (2.3mm) LK-3118</v>
       </c>
       <c r="F17">
-        <v>325000</v>
+        <v>340000</v>
       </c>
       <c r="G17">
-        <v>689000</v>
+        <v>779000</v>
       </c>
       <c r="H17">
-        <v>744120</v>
+        <v>841320</v>
       </c>
       <c r="I17">
-        <v>895700</v>
+        <v>1012700</v>
       </c>
       <c r="J17">
-        <v>364000</v>
+        <v>439000</v>
       </c>
       <c r="K17" t="str">
-        <v>52.8%</v>
+        <v>56.4%</v>
       </c>
     </row>
     <row r="18">
@@ -1019,28 +1019,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D18" t="str">
-        <v>LK-3118</v>
+        <v>LK-3120</v>
       </c>
       <c r="E18" t="str">
-        <v>18*10CM Nồi lẻ kèm nắp (2.3mm) LK-3118</v>
+        <v>20*12CM Nồi lẻ kèm nắp (2.3mm) LK-3120</v>
       </c>
       <c r="F18">
-        <v>340000</v>
+        <v>390000</v>
       </c>
       <c r="G18">
-        <v>779000</v>
+        <v>889000</v>
       </c>
       <c r="H18">
-        <v>841320</v>
+        <v>960120</v>
       </c>
       <c r="I18">
-        <v>1012700</v>
+        <v>1155700</v>
       </c>
       <c r="J18">
-        <v>439000</v>
+        <v>499000</v>
       </c>
       <c r="K18" t="str">
-        <v>56.4%</v>
+        <v>56.1%</v>
       </c>
     </row>
     <row r="19">
@@ -1054,25 +1054,25 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D19" t="str">
-        <v>LK-3120</v>
+        <v>LK-3124</v>
       </c>
       <c r="E19" t="str">
-        <v>20*12CM Nồi lẻ kèm nắp (2.3mm) LK-3120</v>
+        <v>24*14CM Nồi lẻ kèm nắp (2.3mm) LK-3124</v>
       </c>
       <c r="F19">
-        <v>390000</v>
+        <v>460000</v>
       </c>
       <c r="G19">
-        <v>889000</v>
+        <v>1049000</v>
       </c>
       <c r="H19">
-        <v>960120</v>
+        <v>1122430</v>
       </c>
       <c r="I19">
-        <v>1155700</v>
+        <v>1258800</v>
       </c>
       <c r="J19">
-        <v>499000</v>
+        <v>589000</v>
       </c>
       <c r="K19" t="str">
         <v>56.1%</v>
@@ -1089,28 +1089,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D20" t="str">
-        <v>LK-3124</v>
+        <v>LK-3338</v>
       </c>
       <c r="E20" t="str">
-        <v>24*14CM Nồi lẻ kèm nắp (2.3mm) LK-3124</v>
+        <v>18+20+24CM Bộ nồi 3 liền khối kèm nắp (2.3mm) LK-3338</v>
       </c>
       <c r="F20">
-        <v>460000</v>
+        <v>1100000</v>
       </c>
       <c r="G20">
-        <v>1049000</v>
+        <v>2090000</v>
       </c>
       <c r="H20">
-        <v>1122430</v>
+        <v>2780930</v>
       </c>
       <c r="I20">
-        <v>1258800</v>
+        <v>3118800</v>
       </c>
       <c r="J20">
-        <v>589000</v>
+        <v>990000</v>
       </c>
       <c r="K20" t="str">
-        <v>56.1%</v>
+        <v>47.4%</v>
       </c>
     </row>
     <row r="21">
@@ -1124,28 +1124,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D21" t="str">
-        <v>LK-3338</v>
+        <v>LK-3386A</v>
       </c>
       <c r="E21" t="str">
-        <v>18+20+24CM Bộ nồi 3 liền khối kèm nắp (2.3mm) LK-3338</v>
+        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
       </c>
       <c r="F21">
-        <v>1100000</v>
+        <v>550000</v>
       </c>
       <c r="G21">
-        <v>2090000</v>
+        <v>990000</v>
       </c>
       <c r="H21">
-        <v>2780930</v>
+        <v>1069200</v>
       </c>
       <c r="I21">
-        <v>3118800</v>
+        <v>1287000</v>
       </c>
       <c r="J21">
-        <v>990000</v>
+        <v>440000</v>
       </c>
       <c r="K21" t="str">
-        <v>47.4%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="22">
@@ -1159,28 +1159,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D22" t="str">
-        <v>LK-3386A</v>
+        <v>LK-3568A</v>
       </c>
       <c r="E22" t="str">
-        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
+        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
       </c>
       <c r="F22">
-        <v>550000</v>
+        <v>960000</v>
       </c>
       <c r="G22">
-        <v>990000</v>
+        <v>1690000</v>
       </c>
       <c r="H22">
-        <v>1069200</v>
+        <v>1808300</v>
       </c>
       <c r="I22">
-        <v>1287000</v>
+        <v>2028000</v>
       </c>
       <c r="J22">
-        <v>440000</v>
+        <v>730000</v>
       </c>
       <c r="K22" t="str">
-        <v>44.4%</v>
+        <v>43.2%</v>
       </c>
     </row>
     <row r="23">
@@ -1191,31 +1191,31 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C23" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D23" t="str">
-        <v>LK-3568A</v>
+        <v>LK-3122</v>
       </c>
       <c r="E23" t="str">
-        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
+        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
       </c>
       <c r="F23">
-        <v>960000</v>
+        <v>470000</v>
       </c>
       <c r="G23">
-        <v>1690000</v>
+        <v>820000</v>
       </c>
       <c r="H23">
-        <v>1808300</v>
+        <v>885600</v>
       </c>
       <c r="I23">
-        <v>2028000</v>
+        <v>1066000</v>
       </c>
       <c r="J23">
-        <v>730000</v>
+        <v>350000</v>
       </c>
       <c r="K23" t="str">
-        <v>43.2%</v>
+        <v>42.7%</v>
       </c>
     </row>
     <row r="24">
@@ -1229,28 +1229,28 @@
         <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D24" t="str">
-        <v>LK-3122</v>
+        <v>LK-3126</v>
       </c>
       <c r="E24" t="str">
-        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
       </c>
       <c r="F24">
-        <v>470000</v>
+        <v>535000</v>
       </c>
       <c r="G24">
-        <v>820000</v>
+        <v>990000</v>
       </c>
       <c r="H24">
-        <v>885600</v>
+        <v>1069200</v>
       </c>
       <c r="I24">
-        <v>1066000</v>
+        <v>1287000</v>
       </c>
       <c r="J24">
-        <v>350000</v>
+        <v>455000</v>
       </c>
       <c r="K24" t="str">
-        <v>42.7%</v>
+        <v>46.0%</v>
       </c>
     </row>
     <row r="25">
@@ -1261,31 +1261,31 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C25" t="str">
-        <v>NỒI TĂNG ÁP</v>
+        <v>ẤM &amp; BÌNH</v>
       </c>
       <c r="D25" t="str">
-        <v>LK-3126</v>
+        <v>LK-1038</v>
       </c>
       <c r="E25" t="str">
-        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
+        <v>Ấm đun nước LK-1038</v>
       </c>
       <c r="F25">
-        <v>535000</v>
+        <v>300000</v>
       </c>
       <c r="G25">
-        <v>990000</v>
+        <v>525000</v>
       </c>
       <c r="H25">
-        <v>1069200</v>
+        <v>567000</v>
       </c>
       <c r="I25">
-        <v>1287000</v>
+        <v>682500</v>
       </c>
       <c r="J25">
-        <v>455000</v>
+        <v>225000</v>
       </c>
       <c r="K25" t="str">
-        <v>46.0%</v>
+        <v>42.9%</v>
       </c>
     </row>
     <row r="26">
@@ -1296,31 +1296,31 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C26" t="str">
-        <v>ẤM &amp; BÌNH</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D26" t="str">
-        <v>LK-1038</v>
+        <v>LK-92</v>
       </c>
       <c r="E26" t="str">
-        <v>Ấm đun nước LK-1038</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F26">
-        <v>300000</v>
+        <v>835000</v>
       </c>
       <c r="G26">
-        <v>525000</v>
+        <v>1590000</v>
       </c>
       <c r="H26">
-        <v>567000</v>
+        <v>1701300</v>
       </c>
       <c r="I26">
-        <v>682500</v>
+        <v>1908000</v>
       </c>
       <c r="J26">
-        <v>225000</v>
+        <v>755000</v>
       </c>
       <c r="K26" t="str">
-        <v>42.9%</v>
+        <v>47.5%</v>
       </c>
     </row>
     <row r="27">
@@ -1334,28 +1334,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D27" t="str">
-        <v>LK-92</v>
+        <v>LK-586</v>
       </c>
       <c r="E27" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F27">
-        <v>835000</v>
+        <v>430000</v>
       </c>
       <c r="G27">
-        <v>1590000</v>
+        <v>745000</v>
       </c>
       <c r="H27">
-        <v>1701300</v>
+        <v>804600</v>
       </c>
       <c r="I27">
-        <v>1908000</v>
+        <v>968500</v>
       </c>
       <c r="J27">
-        <v>755000</v>
+        <v>315000</v>
       </c>
       <c r="K27" t="str">
-        <v>47.5%</v>
+        <v>42.3%</v>
       </c>
     </row>
     <row r="28">
@@ -1369,28 +1369,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D28" t="str">
-        <v>LK-586</v>
+        <v>LK-588</v>
       </c>
       <c r="E28" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F28">
-        <v>430000</v>
+        <v>585000</v>
       </c>
       <c r="G28">
-        <v>745000</v>
+        <v>1050000</v>
       </c>
       <c r="H28">
-        <v>804600</v>
+        <v>1123500</v>
       </c>
       <c r="I28">
-        <v>968500</v>
+        <v>1260000</v>
       </c>
       <c r="J28">
-        <v>315000</v>
+        <v>465000</v>
       </c>
       <c r="K28" t="str">
-        <v>42.3%</v>
+        <v>44.3%</v>
       </c>
     </row>
     <row r="29">
@@ -1404,28 +1404,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D29" t="str">
-        <v>LK-588</v>
+        <v>LK-668</v>
       </c>
       <c r="E29" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
       </c>
       <c r="F29">
-        <v>585000</v>
+        <v>460000</v>
       </c>
       <c r="G29">
-        <v>1050000</v>
+        <v>920000</v>
       </c>
       <c r="H29">
-        <v>1123500</v>
+        <v>993600</v>
       </c>
       <c r="I29">
-        <v>1260000</v>
+        <v>1196000</v>
       </c>
       <c r="J29">
-        <v>465000</v>
+        <v>460000</v>
       </c>
       <c r="K29" t="str">
-        <v>44.3%</v>
+        <v>50.0%</v>
       </c>
     </row>
     <row r="30">
@@ -1439,28 +1439,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D30" t="str">
-        <v>LK-668</v>
+        <v>LK-688</v>
       </c>
       <c r="E30" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
       </c>
       <c r="F30">
-        <v>460000</v>
+        <v>850000</v>
       </c>
       <c r="G30">
-        <v>920000</v>
+        <v>1690000</v>
       </c>
       <c r="H30">
-        <v>993600</v>
+        <v>1808300</v>
       </c>
       <c r="I30">
-        <v>1196000</v>
+        <v>2028000</v>
       </c>
       <c r="J30">
-        <v>460000</v>
+        <v>840000</v>
       </c>
       <c r="K30" t="str">
-        <v>50.0%</v>
+        <v>49.7%</v>
       </c>
     </row>
     <row r="31">
@@ -1474,28 +1474,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D31" t="str">
-        <v>LK-688</v>
+        <v>LK-1003</v>
       </c>
       <c r="E31" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F31">
-        <v>850000</v>
+        <v>197000</v>
       </c>
       <c r="G31">
-        <v>1690000</v>
+        <v>354000</v>
       </c>
       <c r="H31">
-        <v>1808300</v>
+        <v>389400</v>
       </c>
       <c r="I31">
-        <v>2028000</v>
+        <v>460200</v>
       </c>
       <c r="J31">
-        <v>840000</v>
+        <v>157000</v>
       </c>
       <c r="K31" t="str">
-        <v>49.7%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="32">
@@ -1509,28 +1509,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1003</v>
+        <v>LK-1030</v>
       </c>
       <c r="E32" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F32">
-        <v>197000</v>
+        <v>1020000</v>
       </c>
       <c r="G32">
-        <v>354000</v>
+        <v>1890000</v>
       </c>
       <c r="H32">
-        <v>389400</v>
+        <v>1984500</v>
       </c>
       <c r="I32">
-        <v>460200</v>
+        <v>2063000</v>
       </c>
       <c r="J32">
-        <v>157000</v>
+        <v>870000</v>
       </c>
       <c r="K32" t="str">
-        <v>44.4%</v>
+        <v>46.0%</v>
       </c>
     </row>
     <row r="33">
@@ -1544,28 +1544,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1030</v>
+        <v>LK-1033</v>
       </c>
       <c r="E33" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F33">
-        <v>1020000</v>
+        <v>372000</v>
       </c>
       <c r="G33">
-        <v>1890000</v>
+        <v>669600</v>
       </c>
       <c r="H33">
-        <v>1984500</v>
+        <v>723168</v>
       </c>
       <c r="I33">
-        <v>2063000</v>
+        <v>870480</v>
       </c>
       <c r="J33">
-        <v>870000</v>
+        <v>297600</v>
       </c>
       <c r="K33" t="str">
-        <v>46.0%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="34">
@@ -1579,28 +1579,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1033</v>
+        <v>LK-1050</v>
       </c>
       <c r="E34" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F34">
-        <v>372000</v>
+        <v>780000</v>
       </c>
       <c r="G34">
-        <v>669600</v>
+        <v>1495000</v>
       </c>
       <c r="H34">
-        <v>723168</v>
+        <v>1915300</v>
       </c>
       <c r="I34">
-        <v>870480</v>
+        <v>2148000</v>
       </c>
       <c r="J34">
-        <v>297600</v>
+        <v>715000</v>
       </c>
       <c r="K34" t="str">
-        <v>44.4%</v>
+        <v>47.8%</v>
       </c>
     </row>
     <row r="35">
@@ -1614,28 +1614,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1050</v>
+        <v>LK-1068</v>
       </c>
       <c r="E35" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F35">
-        <v>780000</v>
+        <v>310000</v>
       </c>
       <c r="G35">
-        <v>1495000</v>
+        <v>599000</v>
       </c>
       <c r="H35">
-        <v>1915300</v>
+        <v>646920</v>
       </c>
       <c r="I35">
-        <v>2148000</v>
+        <v>778700</v>
       </c>
       <c r="J35">
-        <v>715000</v>
+        <v>289000</v>
       </c>
       <c r="K35" t="str">
-        <v>47.8%</v>
+        <v>48.2%</v>
       </c>
     </row>
     <row r="36">
@@ -1649,28 +1649,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-1068</v>
+        <v>LK-4160</v>
       </c>
       <c r="E36" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F36">
-        <v>310000</v>
+        <v>1000000</v>
       </c>
       <c r="G36">
-        <v>599000</v>
+        <v>2350000</v>
       </c>
       <c r="H36">
-        <v>646920</v>
+        <v>2514500</v>
       </c>
       <c r="I36">
-        <v>778700</v>
+        <v>2820000</v>
       </c>
       <c r="J36">
-        <v>289000</v>
+        <v>1350000</v>
       </c>
       <c r="K36" t="str">
-        <v>48.2%</v>
+        <v>57.4%</v>
       </c>
     </row>
     <row r="37">
@@ -1684,28 +1684,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4160</v>
+        <v>LK-4161</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F37">
-        <v>1000000</v>
+        <v>800000</v>
       </c>
       <c r="G37">
-        <v>2350000</v>
+        <v>1650000</v>
       </c>
       <c r="H37">
-        <v>2514500</v>
+        <v>1765500</v>
       </c>
       <c r="I37">
-        <v>2820000</v>
+        <v>1980000</v>
       </c>
       <c r="J37">
-        <v>1350000</v>
+        <v>850000</v>
       </c>
       <c r="K37" t="str">
-        <v>57.4%</v>
+        <v>51.5%</v>
       </c>
     </row>
     <row r="38">
@@ -1719,28 +1719,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4161</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F38">
-        <v>800000</v>
+        <v>510000</v>
       </c>
       <c r="G38">
-        <v>1650000</v>
+        <v>950000</v>
       </c>
       <c r="H38">
-        <v>1765500</v>
+        <v>1026000</v>
       </c>
       <c r="I38">
-        <v>1980000</v>
+        <v>1235000</v>
       </c>
       <c r="J38">
-        <v>850000</v>
+        <v>440000</v>
       </c>
       <c r="K38" t="str">
-        <v>51.5%</v>
+        <v>46.3%</v>
       </c>
     </row>
     <row r="39">
@@ -1754,10 +1754,10 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4209</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F39">
         <v>510000</v>
@@ -1789,28 +1789,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-4209</v>
+        <v>LK-5301</v>
       </c>
       <c r="E40" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F40">
-        <v>510000</v>
+        <v>600000</v>
       </c>
       <c r="G40">
-        <v>950000</v>
+        <v>1190000</v>
       </c>
       <c r="H40">
-        <v>1026000</v>
+        <v>1273300</v>
       </c>
       <c r="I40">
-        <v>1235000</v>
+        <v>1428000</v>
       </c>
       <c r="J40">
-        <v>440000</v>
+        <v>590000</v>
       </c>
       <c r="K40" t="str">
-        <v>46.3%</v>
+        <v>49.6%</v>
       </c>
     </row>
     <row r="41">
@@ -1824,28 +1824,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-5301</v>
+        <v>LK-6015</v>
       </c>
       <c r="E41" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F41">
-        <v>600000</v>
+        <v>260000</v>
       </c>
       <c r="G41">
-        <v>1190000</v>
+        <v>490000</v>
       </c>
       <c r="H41">
-        <v>1273300</v>
+        <v>539000</v>
       </c>
       <c r="I41">
-        <v>1428000</v>
+        <v>637000</v>
       </c>
       <c r="J41">
-        <v>590000</v>
+        <v>230000</v>
       </c>
       <c r="K41" t="str">
-        <v>49.6%</v>
+        <v>46.9%</v>
       </c>
     </row>
     <row r="42">
@@ -1859,25 +1859,25 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6015</v>
+        <v>LK-6201</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F42">
-        <v>260000</v>
+        <v>685000</v>
       </c>
       <c r="G42">
-        <v>490000</v>
+        <v>1290000</v>
       </c>
       <c r="H42">
-        <v>539000</v>
+        <v>1380300</v>
       </c>
       <c r="I42">
-        <v>637000</v>
+        <v>1548000</v>
       </c>
       <c r="J42">
-        <v>230000</v>
+        <v>605000</v>
       </c>
       <c r="K42" t="str">
         <v>46.9%</v>
@@ -1894,28 +1894,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-6201</v>
+        <v>LK-7812</v>
       </c>
       <c r="E43" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F43">
-        <v>685000</v>
+        <v>660000</v>
       </c>
       <c r="G43">
-        <v>1290000</v>
+        <v>1190000</v>
       </c>
       <c r="H43">
-        <v>1380300</v>
+        <v>1444500</v>
       </c>
       <c r="I43">
-        <v>1548000</v>
+        <v>1620000</v>
       </c>
       <c r="J43">
-        <v>605000</v>
+        <v>530000</v>
       </c>
       <c r="K43" t="str">
-        <v>46.9%</v>
+        <v>44.5%</v>
       </c>
     </row>
     <row r="44">
@@ -1929,28 +1929,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-7812</v>
+        <v>LK-9014</v>
       </c>
       <c r="E44" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F44">
-        <v>660000</v>
+        <v>1130000</v>
       </c>
       <c r="G44">
-        <v>1190000</v>
+        <v>2190000</v>
       </c>
       <c r="H44">
-        <v>1444500</v>
+        <v>2343300</v>
       </c>
       <c r="I44">
-        <v>1620000</v>
+        <v>2628000</v>
       </c>
       <c r="J44">
-        <v>530000</v>
+        <v>1060000</v>
       </c>
       <c r="K44" t="str">
-        <v>44.5%</v>
+        <v>48.4%</v>
       </c>
     </row>
     <row r="45">
@@ -1958,34 +1958,34 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>Lock&amp;King</v>
+        <v>Takin</v>
       </c>
       <c r="C45" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>CHẢO</v>
       </c>
       <c r="D45" t="str">
-        <v>LK-9014</v>
+        <v>TK-2201</v>
       </c>
       <c r="E45" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F45">
-        <v>1130000</v>
+        <v>265000</v>
       </c>
       <c r="G45">
-        <v>2190000</v>
+        <v>466960</v>
       </c>
       <c r="H45">
-        <v>2343300</v>
+        <v>491000</v>
       </c>
       <c r="I45">
-        <v>2628000</v>
+        <v>607048</v>
       </c>
       <c r="J45">
-        <v>1060000</v>
+        <v>201960</v>
       </c>
       <c r="K45" t="str">
-        <v>48.4%</v>
+        <v>43.2%</v>
       </c>
     </row>
     <row r="46">
@@ -1999,28 +1999,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2201</v>
+        <v>TK-2662</v>
       </c>
       <c r="E46" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F46">
-        <v>265000</v>
+        <v>320000</v>
       </c>
       <c r="G46">
-        <v>466960</v>
+        <v>590000</v>
       </c>
       <c r="H46">
-        <v>491000</v>
+        <v>620000</v>
       </c>
       <c r="I46">
-        <v>607048</v>
+        <v>767000</v>
       </c>
       <c r="J46">
-        <v>201960</v>
+        <v>270000</v>
       </c>
       <c r="K46" t="str">
-        <v>43.2%</v>
+        <v>45.8%</v>
       </c>
     </row>
     <row r="47">
@@ -2034,28 +2034,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2662</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E47" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F47">
-        <v>320000</v>
+        <v>351000</v>
       </c>
       <c r="G47">
-        <v>590000</v>
+        <v>630000</v>
       </c>
       <c r="H47">
-        <v>620000</v>
+        <v>662000</v>
       </c>
       <c r="I47">
-        <v>767000</v>
+        <v>819000</v>
       </c>
       <c r="J47">
-        <v>270000</v>
+        <v>279000</v>
       </c>
       <c r="K47" t="str">
-        <v>45.8%</v>
+        <v>44.3%</v>
       </c>
     </row>
     <row r="48">
@@ -2069,28 +2069,28 @@
         <v>CHẢO</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-2882C</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F48">
-        <v>351000</v>
+        <v>375000</v>
       </c>
       <c r="G48">
-        <v>630000</v>
+        <v>750000</v>
       </c>
       <c r="H48">
-        <v>662000</v>
+        <v>788000</v>
       </c>
       <c r="I48">
-        <v>819000</v>
+        <v>825000</v>
       </c>
       <c r="J48">
-        <v>279000</v>
+        <v>375000</v>
       </c>
       <c r="K48" t="str">
-        <v>44.3%</v>
+        <v>50.0%</v>
       </c>
     </row>
     <row r="49">
@@ -2101,31 +2101,31 @@
         <v>Takin</v>
       </c>
       <c r="C49" t="str">
-        <v>CHẢO</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-3030C</v>
+        <v>TK-036A</v>
       </c>
       <c r="E49" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F49">
-        <v>375000</v>
+        <v>495000</v>
       </c>
       <c r="G49">
-        <v>750000</v>
+        <v>891000</v>
       </c>
       <c r="H49">
-        <v>788000</v>
+        <v>936000</v>
       </c>
       <c r="I49">
-        <v>825000</v>
+        <v>1158300</v>
       </c>
       <c r="J49">
-        <v>375000</v>
+        <v>396000</v>
       </c>
       <c r="K49" t="str">
-        <v>50.0%</v>
+        <v>44.4%</v>
       </c>
     </row>
     <row r="50">
@@ -2139,25 +2139,25 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-036A</v>
+        <v>TK-0324</v>
       </c>
       <c r="E50" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F50">
-        <v>495000</v>
+        <v>245000</v>
       </c>
       <c r="G50">
-        <v>891000</v>
+        <v>441000</v>
       </c>
       <c r="H50">
-        <v>936000</v>
+        <v>464000</v>
       </c>
       <c r="I50">
-        <v>1158300</v>
+        <v>573300</v>
       </c>
       <c r="J50">
-        <v>396000</v>
+        <v>196000</v>
       </c>
       <c r="K50" t="str">
         <v>44.4%</v>
@@ -2174,25 +2174,25 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0324</v>
+        <v>TK-0348A</v>
       </c>
       <c r="E51" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
       </c>
       <c r="F51">
-        <v>245000</v>
+        <v>580000</v>
       </c>
       <c r="G51">
-        <v>441000</v>
+        <v>1044000</v>
       </c>
       <c r="H51">
+        <v>1097000</v>
+      </c>
+      <c r="I51">
+        <v>1252800</v>
+      </c>
+      <c r="J51">
         <v>464000</v>
-      </c>
-      <c r="I51">
-        <v>573300</v>
-      </c>
-      <c r="J51">
-        <v>196000</v>
       </c>
       <c r="K51" t="str">
         <v>44.4%</v>
@@ -2209,28 +2209,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0348A</v>
+        <v>TK-0369</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F52">
-        <v>580000</v>
+        <v>535000</v>
       </c>
       <c r="G52">
-        <v>1044000</v>
+        <v>969000</v>
       </c>
       <c r="H52">
-        <v>1097000</v>
+        <v>1018000</v>
       </c>
       <c r="I52">
-        <v>1252800</v>
+        <v>1259700</v>
       </c>
       <c r="J52">
-        <v>464000</v>
+        <v>434000</v>
       </c>
       <c r="K52" t="str">
-        <v>44.4%</v>
+        <v>44.8%</v>
       </c>
     </row>
     <row r="53">
@@ -2244,28 +2244,28 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0369</v>
+        <v>TK-0488</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F53">
-        <v>535000</v>
+        <v>810000</v>
       </c>
       <c r="G53">
-        <v>969000</v>
+        <v>1469000</v>
       </c>
       <c r="H53">
-        <v>1018000</v>
+        <v>1543000</v>
       </c>
       <c r="I53">
-        <v>1259700</v>
+        <v>1762800</v>
       </c>
       <c r="J53">
-        <v>434000</v>
+        <v>659000</v>
       </c>
       <c r="K53" t="str">
-        <v>44.8%</v>
+        <v>44.9%</v>
       </c>
     </row>
     <row r="54">
@@ -2276,31 +2276,31 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-0488</v>
+        <v>TK-468</v>
       </c>
       <c r="E54" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F54">
-        <v>810000</v>
+        <v>452000</v>
       </c>
       <c r="G54">
-        <v>1469000</v>
+        <v>900000</v>
       </c>
       <c r="H54">
-        <v>1543000</v>
+        <v>945000</v>
       </c>
       <c r="I54">
-        <v>1762800</v>
+        <v>1170000</v>
       </c>
       <c r="J54">
-        <v>659000</v>
+        <v>448000</v>
       </c>
       <c r="K54" t="str">
-        <v>44.9%</v>
+        <v>49.8%</v>
       </c>
     </row>
     <row r="55">
@@ -2314,28 +2314,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-468</v>
+        <v>TK-469</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F55">
-        <v>452000</v>
+        <v>615000</v>
       </c>
       <c r="G55">
-        <v>900000</v>
+        <v>1050000</v>
       </c>
       <c r="H55">
-        <v>945000</v>
+        <v>1103000</v>
       </c>
       <c r="I55">
-        <v>1170000</v>
+        <v>1260000</v>
       </c>
       <c r="J55">
-        <v>448000</v>
+        <v>435000</v>
       </c>
       <c r="K55" t="str">
-        <v>49.8%</v>
+        <v>41.4%</v>
       </c>
     </row>
     <row r="56">
@@ -2349,28 +2349,28 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-469</v>
+        <v>TK-1002</v>
       </c>
       <c r="E56" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
       </c>
       <c r="F56">
-        <v>615000</v>
+        <v>158000</v>
       </c>
       <c r="G56">
-        <v>1050000</v>
+        <v>270000</v>
       </c>
       <c r="H56">
-        <v>1103000</v>
+        <v>284000</v>
       </c>
       <c r="I56">
-        <v>1260000</v>
+        <v>351000</v>
       </c>
       <c r="J56">
-        <v>435000</v>
+        <v>112000</v>
       </c>
       <c r="K56" t="str">
-        <v>41.4%</v>
+        <v>41.5%</v>
       </c>
     </row>
     <row r="57">
@@ -2384,75 +2384,40 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D57" t="str">
-        <v>TK-1002</v>
+        <v>TK-1003</v>
       </c>
       <c r="E57" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Bộ đèn sưởi 3 bóng Takin</v>
       </c>
       <c r="F57">
-        <v>158000</v>
+        <v>194000</v>
       </c>
       <c r="G57">
-        <v>270000</v>
+        <v>330000</v>
       </c>
       <c r="H57">
-        <v>284000</v>
+        <v>347000</v>
       </c>
       <c r="I57">
-        <v>351000</v>
+        <v>429000</v>
       </c>
       <c r="J57">
-        <v>112000</v>
+        <v>136000</v>
       </c>
       <c r="K57" t="str">
-        <v>41.5%</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58" t="str">
-        <v>Takin</v>
-      </c>
-      <c r="C58" t="str">
-        <v>ĐỒ ĐIỆN</v>
-      </c>
-      <c r="D58" t="str">
-        <v>TK-1003</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Bộ đèn sưởi 3 bóng Takin</v>
-      </c>
-      <c r="F58">
-        <v>194000</v>
-      </c>
-      <c r="G58">
-        <v>330000</v>
-      </c>
-      <c r="H58">
-        <v>347000</v>
-      </c>
-      <c r="I58">
-        <v>429000</v>
-      </c>
-      <c r="J58">
-        <v>136000</v>
-      </c>
-      <c r="K58" t="str">
         <v>41.2%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K57"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N57"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2615,37 +2580,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D4" t="str">
-        <v>LK-2466S</v>
+        <v>LK-2606A</v>
       </c>
       <c r="E4" t="str">
-        <v>Chảo Titanium  ELITE Lock&amp;King</v>
+        <v>Chảo cạn Titanium Lock&amp;king 26cm</v>
       </c>
       <c r="F4">
-        <v>289484</v>
+        <v>238375</v>
       </c>
       <c r="G4">
-        <v>390000</v>
+        <v>320000</v>
       </c>
       <c r="H4">
-        <v>690000</v>
+        <v>590000</v>
       </c>
       <c r="I4">
-        <v>300000</v>
+        <v>270000</v>
       </c>
       <c r="J4" t="str">
-        <v>43.5%</v>
+        <v>45.8%</v>
       </c>
       <c r="K4">
-        <v>725000</v>
+        <v>620000</v>
       </c>
       <c r="L4">
-        <v>35000</v>
+        <v>30000</v>
       </c>
       <c r="M4" t="str">
         <v>5.1%</v>
       </c>
       <c r="N4">
-        <v>834000</v>
+        <v>713000</v>
       </c>
     </row>
     <row r="5">
@@ -2659,37 +2624,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D5" t="str">
-        <v>LK-2606A</v>
+        <v>LK-2633</v>
       </c>
       <c r="E5" t="str">
-        <v>Chảo cạn Titanium Lock&amp;king 26cm</v>
+        <v>Chảo Belly Lock&amp;King Titanium 26cm</v>
       </c>
       <c r="F5">
-        <v>238375</v>
+        <v>350676</v>
       </c>
       <c r="G5">
-        <v>320000</v>
+        <v>450000</v>
       </c>
       <c r="H5">
-        <v>590000</v>
+        <v>850000</v>
       </c>
       <c r="I5">
-        <v>270000</v>
+        <v>400000</v>
       </c>
       <c r="J5" t="str">
-        <v>45.8%</v>
+        <v>47.1%</v>
       </c>
       <c r="K5">
-        <v>620000</v>
+        <v>893000</v>
       </c>
       <c r="L5">
-        <v>30000</v>
+        <v>43000</v>
       </c>
       <c r="M5" t="str">
         <v>5.1%</v>
       </c>
       <c r="N5">
-        <v>713000</v>
+        <v>1027000</v>
       </c>
     </row>
     <row r="6">
@@ -2703,37 +2668,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D6" t="str">
-        <v>LK-2633</v>
+        <v>LK-2808</v>
       </c>
       <c r="E6" t="str">
-        <v>Chảo Belly Lock&amp;King Titanium 26cm</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F6">
-        <v>350676</v>
+        <v>267721</v>
       </c>
       <c r="G6">
-        <v>450000</v>
+        <v>351000</v>
       </c>
       <c r="H6">
-        <v>850000</v>
+        <v>630000</v>
       </c>
       <c r="I6">
-        <v>400000</v>
+        <v>279000</v>
       </c>
       <c r="J6" t="str">
-        <v>47.1%</v>
+        <v>44.3%</v>
       </c>
       <c r="K6">
-        <v>893000</v>
+        <v>662000</v>
       </c>
       <c r="L6">
-        <v>43000</v>
+        <v>32000</v>
       </c>
       <c r="M6" t="str">
         <v>5.1%</v>
       </c>
       <c r="N6">
-        <v>1027000</v>
+        <v>762000</v>
       </c>
     </row>
     <row r="7">
@@ -2747,37 +2712,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D7" t="str">
-        <v>LK-2808</v>
+        <v>LK-2808SA KHÔNG NẮP</v>
       </c>
       <c r="E7" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA KHÔNG NẮP</v>
       </c>
       <c r="F7">
-        <v>267721</v>
+        <v>320736</v>
       </c>
       <c r="G7">
-        <v>351000</v>
+        <v>412000</v>
       </c>
       <c r="H7">
-        <v>630000</v>
+        <v>740000</v>
       </c>
       <c r="I7">
-        <v>279000</v>
+        <v>328000</v>
       </c>
       <c r="J7" t="str">
         <v>44.3%</v>
       </c>
       <c r="K7">
-        <v>662000</v>
+        <v>777000</v>
       </c>
       <c r="L7">
-        <v>32000</v>
+        <v>37000</v>
       </c>
       <c r="M7" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N7">
-        <v>762000</v>
+        <v>894000</v>
       </c>
     </row>
     <row r="8">
@@ -2791,37 +2756,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D8" t="str">
-        <v>LK-2808SA KHÔNG NẮP</v>
+        <v>LK-3003</v>
       </c>
       <c r="E8" t="str">
-        <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA KHÔNG NẮP</v>
+        <v>Chảo cạn titanium Lock&amp;King 30cm</v>
       </c>
       <c r="F8">
-        <v>320736</v>
+        <v>291830</v>
       </c>
       <c r="G8">
-        <v>412000</v>
+        <v>375000</v>
       </c>
       <c r="H8">
-        <v>740000</v>
+        <v>750000</v>
       </c>
       <c r="I8">
-        <v>328000</v>
+        <v>375000</v>
       </c>
       <c r="J8" t="str">
-        <v>44.3%</v>
+        <v>50.0%</v>
       </c>
       <c r="K8">
-        <v>777000</v>
+        <v>788000</v>
       </c>
       <c r="L8">
-        <v>37000</v>
+        <v>38000</v>
       </c>
       <c r="M8" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N8">
-        <v>894000</v>
+        <v>907000</v>
       </c>
     </row>
     <row r="9">
@@ -2835,37 +2800,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D9" t="str">
-        <v>LK-3003</v>
+        <v>LK-3212</v>
       </c>
       <c r="E9" t="str">
-        <v>Chảo cạn titanium Lock&amp;King 30cm</v>
+        <v>Chảo xào lớn</v>
       </c>
       <c r="F9">
-        <v>291830</v>
+        <v>472432</v>
       </c>
       <c r="G9">
-        <v>375000</v>
+        <v>645000</v>
       </c>
       <c r="H9">
-        <v>750000</v>
+        <v>1290000</v>
       </c>
       <c r="I9">
-        <v>375000</v>
+        <v>645000</v>
       </c>
       <c r="J9" t="str">
         <v>50.0%</v>
       </c>
       <c r="K9">
-        <v>788000</v>
+        <v>1355000</v>
       </c>
       <c r="L9">
-        <v>38000</v>
+        <v>65000</v>
       </c>
       <c r="M9" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N9">
-        <v>907000</v>
+        <v>1559000</v>
       </c>
     </row>
     <row r="10">
@@ -2876,40 +2841,40 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C10" t="str">
-        <v>CHẢO</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D10" t="str">
-        <v>LK-3212</v>
+        <v>LK-30NC1</v>
       </c>
       <c r="E10" t="str">
-        <v>Chảo xào lớn</v>
+        <v>Nồi luộc gà Lock&amp;King size 30</v>
       </c>
       <c r="F10">
-        <v>472432</v>
+        <v>336906</v>
       </c>
       <c r="G10">
-        <v>645000</v>
+        <v>414000</v>
       </c>
       <c r="H10">
-        <v>1290000</v>
+        <v>750000</v>
       </c>
       <c r="I10">
-        <v>645000</v>
+        <v>336000</v>
       </c>
       <c r="J10" t="str">
-        <v>50.0%</v>
+        <v>44.8%</v>
       </c>
       <c r="K10">
-        <v>1355000</v>
+        <v>788000</v>
       </c>
       <c r="L10">
-        <v>65000</v>
+        <v>38000</v>
       </c>
       <c r="M10" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N10">
-        <v>1559000</v>
+        <v>907000</v>
       </c>
     </row>
     <row r="11">
@@ -2923,37 +2888,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D11" t="str">
-        <v>LK-30NC1</v>
+        <v>LK-32NC1</v>
       </c>
       <c r="E11" t="str">
-        <v>Nồi luộc gà Lock&amp;King size 30</v>
+        <v>Nồi luộc gà Lock&amp;King size 32</v>
       </c>
       <c r="F11">
-        <v>336906</v>
+        <v>400473</v>
       </c>
       <c r="G11">
-        <v>414000</v>
+        <v>470000</v>
       </c>
       <c r="H11">
-        <v>750000</v>
+        <v>830000</v>
       </c>
       <c r="I11">
-        <v>336000</v>
+        <v>360000</v>
       </c>
       <c r="J11" t="str">
-        <v>44.8%</v>
+        <v>43.4%</v>
       </c>
       <c r="K11">
-        <v>788000</v>
+        <v>872000</v>
       </c>
       <c r="L11">
-        <v>38000</v>
+        <v>42000</v>
       </c>
       <c r="M11" t="str">
         <v>5.1%</v>
       </c>
       <c r="N11">
-        <v>907000</v>
+        <v>1003000</v>
       </c>
     </row>
     <row r="12">
@@ -2967,37 +2932,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D12" t="str">
-        <v>LK-32NC1</v>
+        <v>LK-336A</v>
       </c>
       <c r="E12" t="str">
-        <v>Nồi luộc gà Lock&amp;King size 32</v>
+        <v>Bộ nồi 3 Lock&amp;King ( 18,20,24 )</v>
       </c>
       <c r="F12">
-        <v>400473</v>
+        <v>411881</v>
       </c>
       <c r="G12">
-        <v>470000</v>
+        <v>540000</v>
       </c>
       <c r="H12">
-        <v>830000</v>
+        <v>990000</v>
       </c>
       <c r="I12">
-        <v>360000</v>
+        <v>450000</v>
       </c>
       <c r="J12" t="str">
-        <v>43.4%</v>
+        <v>45.5%</v>
       </c>
       <c r="K12">
-        <v>872000</v>
+        <v>1040000</v>
       </c>
       <c r="L12">
-        <v>42000</v>
+        <v>50000</v>
       </c>
       <c r="M12" t="str">
         <v>5.1%</v>
       </c>
       <c r="N12">
-        <v>1003000</v>
+        <v>1196000</v>
       </c>
     </row>
     <row r="13">
@@ -3011,37 +2976,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D13" t="str">
-        <v>LK-336A</v>
+        <v>LK-3018A</v>
       </c>
       <c r="E13" t="str">
-        <v>Bộ nồi 3 Lock&amp;King ( 18,20,24 )</v>
+        <v>Nồi lẻ Lock&amp;king 18</v>
       </c>
       <c r="F13">
-        <v>411881</v>
+        <v>131000</v>
       </c>
       <c r="G13">
-        <v>540000</v>
+        <v>170000</v>
       </c>
       <c r="H13">
-        <v>990000</v>
+        <v>295000</v>
       </c>
       <c r="I13">
-        <v>450000</v>
+        <v>125000</v>
       </c>
       <c r="J13" t="str">
-        <v>45.5%</v>
+        <v>42.4%</v>
       </c>
       <c r="K13">
-        <v>1040000</v>
+        <v>310000</v>
       </c>
       <c r="L13">
-        <v>50000</v>
+        <v>15000</v>
       </c>
       <c r="M13" t="str">
         <v>5.1%</v>
       </c>
       <c r="N13">
-        <v>1196000</v>
+        <v>357000</v>
       </c>
     </row>
     <row r="14">
@@ -3055,37 +3020,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D14" t="str">
-        <v>LK-3018A</v>
+        <v>LK-3020A</v>
       </c>
       <c r="E14" t="str">
-        <v>Nồi lẻ Lock&amp;king 18</v>
+        <v>Nồi lẻ Lock&amp;king 20</v>
       </c>
       <c r="F14">
-        <v>131000</v>
+        <v>148885</v>
       </c>
       <c r="G14">
-        <v>170000</v>
+        <v>185000</v>
       </c>
       <c r="H14">
-        <v>295000</v>
+        <v>315000</v>
       </c>
       <c r="I14">
-        <v>125000</v>
+        <v>130000</v>
       </c>
       <c r="J14" t="str">
-        <v>42.4%</v>
+        <v>41.3%</v>
       </c>
       <c r="K14">
-        <v>310000</v>
+        <v>331000</v>
       </c>
       <c r="L14">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="M14" t="str">
         <v>5.1%</v>
       </c>
       <c r="N14">
-        <v>357000</v>
+        <v>381000</v>
       </c>
     </row>
     <row r="15">
@@ -3099,37 +3064,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D15" t="str">
-        <v>LK-3020A</v>
+        <v>LK-3024</v>
       </c>
       <c r="E15" t="str">
-        <v>Nồi lẻ Lock&amp;king 20</v>
+        <v>Nồi lẻ Lock&amp;king 24</v>
       </c>
       <c r="F15">
-        <v>148885</v>
+        <v>183215</v>
       </c>
       <c r="G15">
-        <v>185000</v>
+        <v>230000</v>
       </c>
       <c r="H15">
-        <v>315000</v>
+        <v>395000</v>
       </c>
       <c r="I15">
-        <v>130000</v>
+        <v>165000</v>
       </c>
       <c r="J15" t="str">
-        <v>41.3%</v>
+        <v>41.8%</v>
       </c>
       <c r="K15">
-        <v>331000</v>
+        <v>415000</v>
       </c>
       <c r="L15">
-        <v>16000</v>
+        <v>20000</v>
       </c>
       <c r="M15" t="str">
         <v>5.1%</v>
       </c>
       <c r="N15">
-        <v>381000</v>
+        <v>478000</v>
       </c>
     </row>
     <row r="16">
@@ -3143,37 +3108,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D16" t="str">
-        <v>LK-3024</v>
+        <v>LK-3116</v>
       </c>
       <c r="E16" t="str">
-        <v>Nồi lẻ Lock&amp;king 24</v>
+        <v>16*9CM Quánh liền khối titan (2.2mm) LK-3116</v>
       </c>
       <c r="F16">
-        <v>183215</v>
+        <v>236683</v>
       </c>
       <c r="G16">
-        <v>230000</v>
+        <v>325000</v>
       </c>
       <c r="H16">
-        <v>395000</v>
+        <v>689000</v>
       </c>
       <c r="I16">
-        <v>165000</v>
+        <v>364000</v>
       </c>
       <c r="J16" t="str">
-        <v>41.8%</v>
+        <v>52.8%</v>
       </c>
       <c r="K16">
-        <v>415000</v>
+        <v>724000</v>
       </c>
       <c r="L16">
-        <v>20000</v>
+        <v>35000</v>
       </c>
       <c r="M16" t="str">
         <v>5.1%</v>
       </c>
       <c r="N16">
-        <v>478000</v>
+        <v>833000</v>
       </c>
     </row>
     <row r="17">
@@ -3187,37 +3152,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D17" t="str">
-        <v>LK-3116</v>
+        <v>LK-3118</v>
       </c>
       <c r="E17" t="str">
-        <v>16*9CM Quánh liền khối titan (2.2mm) LK-3116</v>
+        <v>18*10CM Nồi lẻ kèm nắp (2.3mm) LK-3118</v>
       </c>
       <c r="F17">
-        <v>236683</v>
+        <v>265000</v>
       </c>
       <c r="G17">
-        <v>325000</v>
+        <v>340000</v>
       </c>
       <c r="H17">
-        <v>689000</v>
+        <v>779000</v>
       </c>
       <c r="I17">
-        <v>364000</v>
+        <v>439000</v>
       </c>
       <c r="J17" t="str">
-        <v>52.8%</v>
+        <v>56.4%</v>
       </c>
       <c r="K17">
-        <v>724000</v>
+        <v>818000</v>
       </c>
       <c r="L17">
-        <v>35000</v>
+        <v>39000</v>
       </c>
       <c r="M17" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N17">
-        <v>833000</v>
+        <v>941000</v>
       </c>
     </row>
     <row r="18">
@@ -3231,37 +3196,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D18" t="str">
-        <v>LK-3118</v>
+        <v>LK-3120</v>
       </c>
       <c r="E18" t="str">
-        <v>18*10CM Nồi lẻ kèm nắp (2.3mm) LK-3118</v>
+        <v>20*12CM Nồi lẻ kèm nắp (2.3mm) LK-3120</v>
       </c>
       <c r="F18">
-        <v>265000</v>
+        <v>297124</v>
       </c>
       <c r="G18">
-        <v>340000</v>
+        <v>390000</v>
       </c>
       <c r="H18">
-        <v>779000</v>
+        <v>889000</v>
       </c>
       <c r="I18">
-        <v>439000</v>
+        <v>499000</v>
       </c>
       <c r="J18" t="str">
-        <v>56.4%</v>
+        <v>56.1%</v>
       </c>
       <c r="K18">
-        <v>818000</v>
+        <v>934000</v>
       </c>
       <c r="L18">
-        <v>39000</v>
+        <v>45000</v>
       </c>
       <c r="M18" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N18">
-        <v>941000</v>
+        <v>1075000</v>
       </c>
     </row>
     <row r="19">
@@ -3275,37 +3240,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D19" t="str">
-        <v>LK-3120</v>
+        <v>LK-3124</v>
       </c>
       <c r="E19" t="str">
-        <v>20*12CM Nồi lẻ kèm nắp (2.3mm) LK-3120</v>
+        <v>24*14CM Nồi lẻ kèm nắp (2.3mm) LK-3124</v>
       </c>
       <c r="F19">
-        <v>297124</v>
+        <v>359737</v>
       </c>
       <c r="G19">
-        <v>390000</v>
+        <v>460000</v>
       </c>
       <c r="H19">
-        <v>889000</v>
+        <v>1049000</v>
       </c>
       <c r="I19">
-        <v>499000</v>
+        <v>589000</v>
       </c>
       <c r="J19" t="str">
         <v>56.1%</v>
       </c>
       <c r="K19">
-        <v>934000</v>
+        <v>1102000</v>
       </c>
       <c r="L19">
-        <v>45000</v>
+        <v>53000</v>
       </c>
       <c r="M19" t="str">
         <v>5.1%</v>
       </c>
       <c r="N19">
-        <v>1075000</v>
+        <v>1268000</v>
       </c>
     </row>
     <row r="20">
@@ -3319,37 +3284,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D20" t="str">
-        <v>LK-3124</v>
+        <v>LK-3338</v>
       </c>
       <c r="E20" t="str">
-        <v>24*14CM Nồi lẻ kèm nắp (2.3mm) LK-3124</v>
+        <v>18+20+24CM Bộ nồi 3 liền khối kèm nắp (2.3mm) LK-3338</v>
       </c>
       <c r="F20">
-        <v>359737</v>
+        <v>883000</v>
       </c>
       <c r="G20">
-        <v>460000</v>
+        <v>1100000</v>
       </c>
       <c r="H20">
-        <v>1049000</v>
+        <v>2090000</v>
       </c>
       <c r="I20">
-        <v>589000</v>
+        <v>990000</v>
       </c>
       <c r="J20" t="str">
-        <v>56.1%</v>
+        <v>47.4%</v>
       </c>
       <c r="K20">
-        <v>1102000</v>
+        <v>2195000</v>
       </c>
       <c r="L20">
-        <v>53000</v>
+        <v>105000</v>
       </c>
       <c r="M20" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N20">
-        <v>1268000</v>
+        <v>2525000</v>
       </c>
     </row>
     <row r="21">
@@ -3363,37 +3328,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D21" t="str">
-        <v>LK-3338</v>
+        <v>LK-3386A</v>
       </c>
       <c r="E21" t="str">
-        <v>18+20+24CM Bộ nồi 3 liền khối kèm nắp (2.3mm) LK-3338</v>
+        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
       </c>
       <c r="F21">
-        <v>883000</v>
+        <v>453015</v>
       </c>
       <c r="G21">
-        <v>1100000</v>
+        <v>550000</v>
       </c>
       <c r="H21">
-        <v>2090000</v>
+        <v>990000</v>
       </c>
       <c r="I21">
-        <v>990000</v>
+        <v>440000</v>
       </c>
       <c r="J21" t="str">
-        <v>47.4%</v>
+        <v>44.4%</v>
       </c>
       <c r="K21">
-        <v>2195000</v>
+        <v>1040000</v>
       </c>
       <c r="L21">
-        <v>105000</v>
+        <v>50000</v>
       </c>
       <c r="M21" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N21">
-        <v>2525000</v>
+        <v>1196000</v>
       </c>
     </row>
     <row r="22">
@@ -3407,37 +3372,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D22" t="str">
-        <v>LK-3386A</v>
+        <v>LK-3568A</v>
       </c>
       <c r="E22" t="str">
-        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
+        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
       </c>
       <c r="F22">
-        <v>453015</v>
+        <v>815667</v>
       </c>
       <c r="G22">
-        <v>550000</v>
+        <v>960000</v>
       </c>
       <c r="H22">
-        <v>990000</v>
+        <v>1690000</v>
       </c>
       <c r="I22">
-        <v>440000</v>
+        <v>730000</v>
       </c>
       <c r="J22" t="str">
-        <v>44.4%</v>
+        <v>43.2%</v>
       </c>
       <c r="K22">
-        <v>1040000</v>
+        <v>1775000</v>
       </c>
       <c r="L22">
-        <v>50000</v>
+        <v>85000</v>
       </c>
       <c r="M22" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N22">
-        <v>1196000</v>
+        <v>2042000</v>
       </c>
     </row>
     <row r="23">
@@ -3448,40 +3413,40 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C23" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D23" t="str">
-        <v>LK-3568A</v>
+        <v>LK-3122</v>
       </c>
       <c r="E23" t="str">
-        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
+        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
       </c>
       <c r="F23">
-        <v>815667</v>
+        <v>357441</v>
       </c>
       <c r="G23">
-        <v>960000</v>
+        <v>470000</v>
       </c>
       <c r="H23">
-        <v>1690000</v>
+        <v>820000</v>
       </c>
       <c r="I23">
-        <v>730000</v>
+        <v>350000</v>
       </c>
       <c r="J23" t="str">
-        <v>43.2%</v>
+        <v>42.7%</v>
       </c>
       <c r="K23">
-        <v>1775000</v>
+        <v>861000</v>
       </c>
       <c r="L23">
-        <v>85000</v>
+        <v>41000</v>
       </c>
       <c r="M23" t="str">
         <v>5.0%</v>
       </c>
       <c r="N23">
-        <v>2042000</v>
+        <v>991000</v>
       </c>
     </row>
     <row r="24">
@@ -3495,37 +3460,37 @@
         <v>NỒI TĂNG ÁP</v>
       </c>
       <c r="D24" t="str">
-        <v>LK-3122</v>
+        <v>LK-3126</v>
       </c>
       <c r="E24" t="str">
-        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
       </c>
       <c r="F24">
-        <v>357441</v>
+        <v>387848</v>
       </c>
       <c r="G24">
-        <v>470000</v>
+        <v>535000</v>
       </c>
       <c r="H24">
-        <v>820000</v>
+        <v>990000</v>
       </c>
       <c r="I24">
-        <v>350000</v>
+        <v>455000</v>
       </c>
       <c r="J24" t="str">
-        <v>42.7%</v>
+        <v>46.0%</v>
       </c>
       <c r="K24">
-        <v>861000</v>
+        <v>1040000</v>
       </c>
       <c r="L24">
-        <v>41000</v>
+        <v>50000</v>
       </c>
       <c r="M24" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N24">
-        <v>991000</v>
+        <v>1196000</v>
       </c>
     </row>
     <row r="25">
@@ -3536,40 +3501,40 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C25" t="str">
-        <v>NỒI TĂNG ÁP</v>
+        <v>ẤM &amp; BÌNH</v>
       </c>
       <c r="D25" t="str">
-        <v>LK-3126</v>
+        <v>LK-1038</v>
       </c>
       <c r="E25" t="str">
-        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
+        <v>Ấm đun nước LK-1038</v>
       </c>
       <c r="F25">
-        <v>387848</v>
+        <v>235094</v>
       </c>
       <c r="G25">
-        <v>535000</v>
+        <v>300000</v>
       </c>
       <c r="H25">
-        <v>990000</v>
+        <v>525000</v>
       </c>
       <c r="I25">
-        <v>455000</v>
+        <v>225000</v>
       </c>
       <c r="J25" t="str">
-        <v>46.0%</v>
+        <v>42.9%</v>
       </c>
       <c r="K25">
-        <v>1040000</v>
+        <v>552000</v>
       </c>
       <c r="L25">
-        <v>50000</v>
+        <v>27000</v>
       </c>
       <c r="M25" t="str">
         <v>5.1%</v>
       </c>
       <c r="N25">
-        <v>1196000</v>
+        <v>635000</v>
       </c>
     </row>
     <row r="26">
@@ -3580,40 +3545,40 @@
         <v>Lock&amp;King</v>
       </c>
       <c r="C26" t="str">
-        <v>ẤM &amp; BÌNH</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D26" t="str">
-        <v>LK-1038</v>
+        <v>LK-92</v>
       </c>
       <c r="E26" t="str">
-        <v>Ấm đun nước LK-1038</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F26">
-        <v>235094</v>
+        <v>727600</v>
       </c>
       <c r="G26">
-        <v>300000</v>
+        <v>835000</v>
       </c>
       <c r="H26">
-        <v>525000</v>
+        <v>1590000</v>
       </c>
       <c r="I26">
-        <v>225000</v>
+        <v>755000</v>
       </c>
       <c r="J26" t="str">
-        <v>42.9%</v>
+        <v>47.5%</v>
       </c>
       <c r="K26">
-        <v>552000</v>
+        <v>1670000</v>
       </c>
       <c r="L26">
-        <v>27000</v>
+        <v>80000</v>
       </c>
       <c r="M26" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N26">
-        <v>635000</v>
+        <v>1921000</v>
       </c>
     </row>
     <row r="27">
@@ -3627,37 +3592,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D27" t="str">
-        <v>LK-92</v>
+        <v>LK-586</v>
       </c>
       <c r="E27" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F27">
-        <v>727600</v>
+        <v>366857</v>
       </c>
       <c r="G27">
-        <v>835000</v>
+        <v>430000</v>
       </c>
       <c r="H27">
-        <v>1590000</v>
+        <v>745000</v>
       </c>
       <c r="I27">
-        <v>755000</v>
+        <v>315000</v>
       </c>
       <c r="J27" t="str">
-        <v>47.5%</v>
+        <v>42.3%</v>
       </c>
       <c r="K27">
-        <v>1670000</v>
+        <v>783000</v>
       </c>
       <c r="L27">
-        <v>80000</v>
+        <v>38000</v>
       </c>
       <c r="M27" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N27">
-        <v>1921000</v>
+        <v>901000</v>
       </c>
     </row>
     <row r="28">
@@ -3671,37 +3636,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D28" t="str">
-        <v>LK-586</v>
+        <v>LK-588</v>
       </c>
       <c r="E28" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F28">
-        <v>366857</v>
+        <v>468762</v>
       </c>
       <c r="G28">
-        <v>430000</v>
+        <v>585000</v>
       </c>
       <c r="H28">
-        <v>745000</v>
+        <v>1050000</v>
       </c>
       <c r="I28">
-        <v>315000</v>
+        <v>465000</v>
       </c>
       <c r="J28" t="str">
-        <v>42.3%</v>
+        <v>44.3%</v>
       </c>
       <c r="K28">
-        <v>783000</v>
+        <v>1103000</v>
       </c>
       <c r="L28">
-        <v>38000</v>
+        <v>53000</v>
       </c>
       <c r="M28" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N28">
-        <v>901000</v>
+        <v>1269000</v>
       </c>
     </row>
     <row r="29">
@@ -3715,37 +3680,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D29" t="str">
-        <v>LK-588</v>
+        <v>LK-668</v>
       </c>
       <c r="E29" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
       </c>
       <c r="F29">
-        <v>468762</v>
+        <v>395900</v>
       </c>
       <c r="G29">
-        <v>585000</v>
+        <v>460000</v>
       </c>
       <c r="H29">
-        <v>1050000</v>
+        <v>920000</v>
       </c>
       <c r="I29">
-        <v>465000</v>
+        <v>460000</v>
       </c>
       <c r="J29" t="str">
-        <v>44.3%</v>
+        <v>50.0%</v>
       </c>
       <c r="K29">
-        <v>1103000</v>
+        <v>966000</v>
       </c>
       <c r="L29">
-        <v>53000</v>
+        <v>46000</v>
       </c>
       <c r="M29" t="str">
         <v>5.0%</v>
       </c>
       <c r="N29">
-        <v>1269000</v>
+        <v>1111000</v>
       </c>
     </row>
     <row r="30">
@@ -3759,37 +3724,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D30" t="str">
-        <v>LK-668</v>
+        <v>LK-688</v>
       </c>
       <c r="E30" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
       </c>
       <c r="F30">
-        <v>395900</v>
+        <v>727600</v>
       </c>
       <c r="G30">
-        <v>460000</v>
+        <v>850000</v>
       </c>
       <c r="H30">
-        <v>920000</v>
+        <v>1690000</v>
       </c>
       <c r="I30">
-        <v>460000</v>
+        <v>840000</v>
       </c>
       <c r="J30" t="str">
-        <v>50.0%</v>
+        <v>49.7%</v>
       </c>
       <c r="K30">
-        <v>966000</v>
+        <v>1775000</v>
       </c>
       <c r="L30">
-        <v>46000</v>
+        <v>85000</v>
       </c>
       <c r="M30" t="str">
         <v>5.0%</v>
       </c>
       <c r="N30">
-        <v>1111000</v>
+        <v>2042000</v>
       </c>
     </row>
     <row r="31">
@@ -3803,37 +3768,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D31" t="str">
-        <v>LK-688</v>
+        <v>LK-1003</v>
       </c>
       <c r="E31" t="str">
-        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F31">
-        <v>727600</v>
+        <v>167990</v>
       </c>
       <c r="G31">
-        <v>850000</v>
+        <v>197000</v>
       </c>
       <c r="H31">
-        <v>1690000</v>
+        <v>354000</v>
       </c>
       <c r="I31">
-        <v>840000</v>
+        <v>157000</v>
       </c>
       <c r="J31" t="str">
-        <v>49.7%</v>
+        <v>44.4%</v>
       </c>
       <c r="K31">
-        <v>1775000</v>
+        <v>372000</v>
       </c>
       <c r="L31">
-        <v>85000</v>
+        <v>18000</v>
       </c>
       <c r="M31" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N31">
-        <v>2042000</v>
+        <v>428000</v>
       </c>
     </row>
     <row r="32">
@@ -3847,37 +3812,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D32" t="str">
-        <v>LK-1003</v>
+        <v>LK-1030</v>
       </c>
       <c r="E32" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
       </c>
       <c r="F32">
-        <v>167990</v>
+        <v>795408</v>
       </c>
       <c r="G32">
-        <v>197000</v>
+        <v>1020000</v>
       </c>
       <c r="H32">
-        <v>354000</v>
+        <v>1890000</v>
       </c>
       <c r="I32">
-        <v>157000</v>
+        <v>870000</v>
       </c>
       <c r="J32" t="str">
-        <v>44.4%</v>
+        <v>46.0%</v>
       </c>
       <c r="K32">
-        <v>372000</v>
+        <v>1985000</v>
       </c>
       <c r="L32">
-        <v>18000</v>
+        <v>95000</v>
       </c>
       <c r="M32" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N32">
-        <v>428000</v>
+        <v>2283000</v>
       </c>
     </row>
     <row r="33">
@@ -3891,37 +3856,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D33" t="str">
-        <v>LK-1030</v>
+        <v>LK-1033</v>
       </c>
       <c r="E33" t="str">
-        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
       </c>
       <c r="F33">
-        <v>795408</v>
+        <v>306020</v>
       </c>
       <c r="G33">
-        <v>1020000</v>
+        <v>372000</v>
       </c>
       <c r="H33">
-        <v>1890000</v>
+        <v>670000</v>
       </c>
       <c r="I33">
-        <v>870000</v>
+        <v>298000</v>
       </c>
       <c r="J33" t="str">
-        <v>46.0%</v>
+        <v>44.5%</v>
       </c>
       <c r="K33">
-        <v>1985000</v>
+        <v>704000</v>
       </c>
       <c r="L33">
-        <v>95000</v>
+        <v>34000</v>
       </c>
       <c r="M33" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N33">
-        <v>2283000</v>
+        <v>810000</v>
       </c>
     </row>
     <row r="34">
@@ -3935,37 +3900,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D34" t="str">
-        <v>LK-1033</v>
+        <v>LK-1050</v>
       </c>
       <c r="E34" t="str">
-        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
       </c>
       <c r="F34">
-        <v>306020</v>
+        <v>668157</v>
       </c>
       <c r="G34">
-        <v>372000</v>
+        <v>780000</v>
       </c>
       <c r="H34">
-        <v>670000</v>
+        <v>1495000</v>
       </c>
       <c r="I34">
-        <v>298000</v>
+        <v>715000</v>
       </c>
       <c r="J34" t="str">
-        <v>44.5%</v>
+        <v>47.8%</v>
       </c>
       <c r="K34">
-        <v>704000</v>
+        <v>1570000</v>
       </c>
       <c r="L34">
-        <v>34000</v>
+        <v>75000</v>
       </c>
       <c r="M34" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N34">
-        <v>810000</v>
+        <v>1806000</v>
       </c>
     </row>
     <row r="35">
@@ -3979,37 +3944,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D35" t="str">
-        <v>LK-1050</v>
+        <v>LK-1068</v>
       </c>
       <c r="E35" t="str">
-        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+        <v>Ấm siêu tốc LK-1068</v>
       </c>
       <c r="F35">
-        <v>668157</v>
+        <v>259549</v>
       </c>
       <c r="G35">
-        <v>780000</v>
+        <v>310000</v>
       </c>
       <c r="H35">
-        <v>1495000</v>
+        <v>599000</v>
       </c>
       <c r="I35">
-        <v>715000</v>
+        <v>289000</v>
       </c>
       <c r="J35" t="str">
-        <v>47.8%</v>
+        <v>48.2%</v>
       </c>
       <c r="K35">
-        <v>1570000</v>
+        <v>629000</v>
       </c>
       <c r="L35">
-        <v>75000</v>
+        <v>30000</v>
       </c>
       <c r="M35" t="str">
         <v>5.0%</v>
       </c>
       <c r="N35">
-        <v>1806000</v>
+        <v>724000</v>
       </c>
     </row>
     <row r="36">
@@ -4023,37 +3988,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D36" t="str">
-        <v>LK-1068</v>
+        <v>LK-4160</v>
       </c>
       <c r="E36" t="str">
-        <v>Ấm siêu tốc LK-1068</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
       </c>
       <c r="F36">
-        <v>259549</v>
+        <v>828486</v>
       </c>
       <c r="G36">
-        <v>310000</v>
+        <v>1000000</v>
       </c>
       <c r="H36">
-        <v>599000</v>
+        <v>2350000</v>
       </c>
       <c r="I36">
-        <v>289000</v>
+        <v>1350000</v>
       </c>
       <c r="J36" t="str">
-        <v>48.2%</v>
+        <v>57.4%</v>
       </c>
       <c r="K36">
-        <v>629000</v>
+        <v>2468000</v>
       </c>
       <c r="L36">
-        <v>30000</v>
+        <v>118000</v>
       </c>
       <c r="M36" t="str">
         <v>5.0%</v>
       </c>
       <c r="N36">
-        <v>724000</v>
+        <v>2839000</v>
       </c>
     </row>
     <row r="37">
@@ -4067,37 +4032,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D37" t="str">
-        <v>LK-4160</v>
+        <v>LK-4161</v>
       </c>
       <c r="E37" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
       </c>
       <c r="F37">
-        <v>828486</v>
+        <v>672571</v>
       </c>
       <c r="G37">
-        <v>1000000</v>
+        <v>800000</v>
       </c>
       <c r="H37">
-        <v>2350000</v>
+        <v>1650000</v>
       </c>
       <c r="I37">
-        <v>1350000</v>
+        <v>850000</v>
       </c>
       <c r="J37" t="str">
-        <v>57.4%</v>
+        <v>51.5%</v>
       </c>
       <c r="K37">
-        <v>2468000</v>
+        <v>1733000</v>
       </c>
       <c r="L37">
-        <v>118000</v>
+        <v>83000</v>
       </c>
       <c r="M37" t="str">
         <v>5.0%</v>
       </c>
       <c r="N37">
-        <v>2839000</v>
+        <v>1993000</v>
       </c>
     </row>
     <row r="38">
@@ -4111,37 +4076,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D38" t="str">
-        <v>LK-4161</v>
+        <v>LK-4208A</v>
       </c>
       <c r="E38" t="str">
-        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
       </c>
       <c r="F38">
-        <v>672571</v>
+        <v>399987</v>
       </c>
       <c r="G38">
-        <v>800000</v>
+        <v>510000</v>
       </c>
       <c r="H38">
-        <v>1650000</v>
+        <v>950000</v>
       </c>
       <c r="I38">
-        <v>850000</v>
+        <v>440000</v>
       </c>
       <c r="J38" t="str">
-        <v>51.5%</v>
+        <v>46.3%</v>
       </c>
       <c r="K38">
-        <v>1733000</v>
+        <v>998000</v>
       </c>
       <c r="L38">
-        <v>83000</v>
+        <v>48000</v>
       </c>
       <c r="M38" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N38">
-        <v>1993000</v>
+        <v>1148000</v>
       </c>
     </row>
     <row r="39">
@@ -4155,13 +4120,13 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D39" t="str">
-        <v>LK-4208A</v>
+        <v>LK-4209</v>
       </c>
       <c r="E39" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
       </c>
       <c r="F39">
-        <v>399987</v>
+        <v>389541</v>
       </c>
       <c r="G39">
         <v>510000</v>
@@ -4199,37 +4164,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D40" t="str">
-        <v>LK-4209</v>
+        <v>LK-5301</v>
       </c>
       <c r="E40" t="str">
-        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+        <v>Sưởi để bàn</v>
       </c>
       <c r="F40">
-        <v>389541</v>
+        <v>468762</v>
       </c>
       <c r="G40">
-        <v>510000</v>
+        <v>600000</v>
       </c>
       <c r="H40">
-        <v>950000</v>
+        <v>1190000</v>
       </c>
       <c r="I40">
-        <v>440000</v>
+        <v>590000</v>
       </c>
       <c r="J40" t="str">
-        <v>46.3%</v>
+        <v>49.6%</v>
       </c>
       <c r="K40">
-        <v>998000</v>
+        <v>1250000</v>
       </c>
       <c r="L40">
-        <v>48000</v>
+        <v>60000</v>
       </c>
       <c r="M40" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N40">
-        <v>1148000</v>
+        <v>1438000</v>
       </c>
     </row>
     <row r="41">
@@ -4243,37 +4208,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D41" t="str">
-        <v>LK-5301</v>
+        <v>LK-6015</v>
       </c>
       <c r="E41" t="str">
-        <v>Sưởi để bàn</v>
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
       </c>
       <c r="F41">
-        <v>468762</v>
+        <v>200752</v>
       </c>
       <c r="G41">
-        <v>600000</v>
+        <v>260000</v>
       </c>
       <c r="H41">
-        <v>1190000</v>
+        <v>490000</v>
       </c>
       <c r="I41">
-        <v>590000</v>
+        <v>230000</v>
       </c>
       <c r="J41" t="str">
-        <v>49.6%</v>
+        <v>46.9%</v>
       </c>
       <c r="K41">
-        <v>1250000</v>
+        <v>515000</v>
       </c>
       <c r="L41">
-        <v>60000</v>
+        <v>25000</v>
       </c>
       <c r="M41" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N41">
-        <v>1438000</v>
+        <v>593000</v>
       </c>
     </row>
     <row r="42">
@@ -4287,37 +4252,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D42" t="str">
-        <v>LK-6015</v>
+        <v>LK-6201</v>
       </c>
       <c r="E42" t="str">
-        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
       </c>
       <c r="F42">
-        <v>200752</v>
+        <v>550047</v>
       </c>
       <c r="G42">
-        <v>260000</v>
+        <v>685000</v>
       </c>
       <c r="H42">
-        <v>490000</v>
+        <v>1290000</v>
       </c>
       <c r="I42">
-        <v>230000</v>
+        <v>605000</v>
       </c>
       <c r="J42" t="str">
         <v>46.9%</v>
       </c>
       <c r="K42">
-        <v>515000</v>
+        <v>1355000</v>
       </c>
       <c r="L42">
-        <v>25000</v>
+        <v>65000</v>
       </c>
       <c r="M42" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N42">
-        <v>593000</v>
+        <v>1559000</v>
       </c>
     </row>
     <row r="43">
@@ -4331,37 +4296,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D43" t="str">
-        <v>LK-6201</v>
+        <v>LK-7812</v>
       </c>
       <c r="E43" t="str">
-        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+        <v>Máy làm sữa hạt Lock&amp;King</v>
       </c>
       <c r="F43">
-        <v>550047</v>
+        <v>545604</v>
       </c>
       <c r="G43">
-        <v>685000</v>
+        <v>660000</v>
       </c>
       <c r="H43">
-        <v>1290000</v>
+        <v>1190000</v>
       </c>
       <c r="I43">
-        <v>605000</v>
+        <v>530000</v>
       </c>
       <c r="J43" t="str">
-        <v>46.9%</v>
+        <v>44.5%</v>
       </c>
       <c r="K43">
-        <v>1355000</v>
+        <v>1250000</v>
       </c>
       <c r="L43">
-        <v>65000</v>
+        <v>60000</v>
       </c>
       <c r="M43" t="str">
         <v>5.0%</v>
       </c>
       <c r="N43">
-        <v>1559000</v>
+        <v>1438000</v>
       </c>
     </row>
     <row r="44">
@@ -4375,37 +4340,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D44" t="str">
-        <v>LK-7812</v>
+        <v>LK-9014</v>
       </c>
       <c r="E44" t="str">
-        <v>Máy làm sữa hạt Lock&amp;King</v>
+        <v>Nồi chiên không dầu Lock&amp;king</v>
       </c>
       <c r="F44">
-        <v>545604</v>
+        <v>936250</v>
       </c>
       <c r="G44">
-        <v>660000</v>
+        <v>1130000</v>
       </c>
       <c r="H44">
-        <v>1190000</v>
+        <v>2190000</v>
       </c>
       <c r="I44">
-        <v>530000</v>
+        <v>1060000</v>
       </c>
       <c r="J44" t="str">
-        <v>44.5%</v>
+        <v>48.4%</v>
       </c>
       <c r="K44">
-        <v>1250000</v>
+        <v>2300000</v>
       </c>
       <c r="L44">
-        <v>60000</v>
+        <v>110000</v>
       </c>
       <c r="M44" t="str">
         <v>5.0%</v>
       </c>
       <c r="N44">
-        <v>1438000</v>
+        <v>2645000</v>
       </c>
     </row>
     <row r="45">
@@ -4413,43 +4378,43 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>Lock&amp;King</v>
+        <v>Takin</v>
       </c>
       <c r="C45" t="str">
-        <v>ĐỒ ĐIỆN</v>
+        <v>CHẢO</v>
       </c>
       <c r="D45" t="str">
-        <v>LK-9014</v>
+        <v>TK-2201</v>
       </c>
       <c r="E45" t="str">
-        <v>Nồi chiên không dầu Lock&amp;king</v>
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
       </c>
       <c r="F45">
-        <v>936250</v>
+        <v>203634</v>
       </c>
       <c r="G45">
-        <v>1130000</v>
+        <v>265000</v>
       </c>
       <c r="H45">
-        <v>2190000</v>
+        <v>467000</v>
       </c>
       <c r="I45">
-        <v>1060000</v>
+        <v>202000</v>
       </c>
       <c r="J45" t="str">
-        <v>48.4%</v>
+        <v>43.3%</v>
       </c>
       <c r="K45">
-        <v>2300000</v>
+        <v>491000</v>
       </c>
       <c r="L45">
-        <v>110000</v>
+        <v>24000</v>
       </c>
       <c r="M45" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N45">
-        <v>2645000</v>
+        <v>565000</v>
       </c>
     </row>
     <row r="46">
@@ -4463,37 +4428,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D46" t="str">
-        <v>TK-2201</v>
+        <v>TK-2662</v>
       </c>
       <c r="E46" t="str">
-        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
       </c>
       <c r="F46">
-        <v>203634</v>
+        <v>238375</v>
       </c>
       <c r="G46">
-        <v>265000</v>
+        <v>320000</v>
       </c>
       <c r="H46">
-        <v>467000</v>
+        <v>590000</v>
       </c>
       <c r="I46">
-        <v>202000</v>
+        <v>270000</v>
       </c>
       <c r="J46" t="str">
-        <v>43.3%</v>
+        <v>45.8%</v>
       </c>
       <c r="K46">
-        <v>491000</v>
+        <v>620000</v>
       </c>
       <c r="L46">
-        <v>24000</v>
+        <v>30000</v>
       </c>
       <c r="M46" t="str">
         <v>5.1%</v>
       </c>
       <c r="N46">
-        <v>565000</v>
+        <v>713000</v>
       </c>
     </row>
     <row r="47">
@@ -4507,37 +4472,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D47" t="str">
-        <v>TK-2662</v>
+        <v>TK-2882C</v>
       </c>
       <c r="E47" t="str">
-        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
       </c>
       <c r="F47">
-        <v>238375</v>
+        <v>266199</v>
       </c>
       <c r="G47">
-        <v>320000</v>
+        <v>351000</v>
       </c>
       <c r="H47">
-        <v>590000</v>
+        <v>630000</v>
       </c>
       <c r="I47">
-        <v>270000</v>
+        <v>279000</v>
       </c>
       <c r="J47" t="str">
-        <v>45.8%</v>
+        <v>44.3%</v>
       </c>
       <c r="K47">
-        <v>620000</v>
+        <v>662000</v>
       </c>
       <c r="L47">
-        <v>30000</v>
+        <v>32000</v>
       </c>
       <c r="M47" t="str">
         <v>5.1%</v>
       </c>
       <c r="N47">
-        <v>713000</v>
+        <v>762000</v>
       </c>
     </row>
     <row r="48">
@@ -4551,37 +4516,37 @@
         <v>CHẢO</v>
       </c>
       <c r="D48" t="str">
-        <v>TK-2882C</v>
+        <v>TK-3030C</v>
       </c>
       <c r="E48" t="str">
-        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
       </c>
       <c r="F48">
-        <v>266199</v>
+        <v>290175</v>
       </c>
       <c r="G48">
-        <v>351000</v>
+        <v>375000</v>
       </c>
       <c r="H48">
-        <v>630000</v>
+        <v>750000</v>
       </c>
       <c r="I48">
-        <v>279000</v>
+        <v>375000</v>
       </c>
       <c r="J48" t="str">
-        <v>44.3%</v>
+        <v>50.0%</v>
       </c>
       <c r="K48">
-        <v>662000</v>
+        <v>788000</v>
       </c>
       <c r="L48">
-        <v>32000</v>
+        <v>38000</v>
       </c>
       <c r="M48" t="str">
         <v>5.1%</v>
       </c>
       <c r="N48">
-        <v>762000</v>
+        <v>907000</v>
       </c>
     </row>
     <row r="49">
@@ -4592,40 +4557,40 @@
         <v>Takin</v>
       </c>
       <c r="C49" t="str">
-        <v>CHẢO</v>
+        <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D49" t="str">
-        <v>TK-3030C</v>
+        <v>TK-036A</v>
       </c>
       <c r="E49" t="str">
-        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F49">
-        <v>290175</v>
+        <v>433985</v>
       </c>
       <c r="G49">
-        <v>375000</v>
+        <v>495000</v>
       </c>
       <c r="H49">
-        <v>750000</v>
+        <v>891000</v>
       </c>
       <c r="I49">
-        <v>375000</v>
+        <v>396000</v>
       </c>
       <c r="J49" t="str">
-        <v>50.0%</v>
+        <v>44.4%</v>
       </c>
       <c r="K49">
-        <v>788000</v>
+        <v>936000</v>
       </c>
       <c r="L49">
-        <v>38000</v>
+        <v>45000</v>
       </c>
       <c r="M49" t="str">
         <v>5.1%</v>
       </c>
       <c r="N49">
-        <v>907000</v>
+        <v>1077000</v>
       </c>
     </row>
     <row r="50">
@@ -4639,37 +4604,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D50" t="str">
-        <v>TK-036A</v>
+        <v>TK-0324</v>
       </c>
       <c r="E50" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Nồi táo inox cao cấp size24</v>
       </c>
       <c r="F50">
-        <v>433985</v>
+        <v>188524</v>
       </c>
       <c r="G50">
-        <v>495000</v>
+        <v>245000</v>
       </c>
       <c r="H50">
-        <v>891000</v>
+        <v>441000</v>
       </c>
       <c r="I50">
-        <v>396000</v>
+        <v>196000</v>
       </c>
       <c r="J50" t="str">
         <v>44.4%</v>
       </c>
       <c r="K50">
-        <v>936000</v>
+        <v>464000</v>
       </c>
       <c r="L50">
-        <v>45000</v>
+        <v>23000</v>
       </c>
       <c r="M50" t="str">
-        <v>5.1%</v>
+        <v>5.2%</v>
       </c>
       <c r="N50">
-        <v>1077000</v>
+        <v>534000</v>
       </c>
     </row>
     <row r="51">
@@ -4683,37 +4648,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D51" t="str">
-        <v>TK-0324</v>
+        <v>TK-0348A</v>
       </c>
       <c r="E51" t="str">
-        <v>Nồi táo inox cao cấp size24</v>
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
       </c>
       <c r="F51">
-        <v>188524</v>
+        <v>492000</v>
       </c>
       <c r="G51">
-        <v>245000</v>
+        <v>580000</v>
       </c>
       <c r="H51">
-        <v>441000</v>
+        <v>1044000</v>
       </c>
       <c r="I51">
-        <v>196000</v>
+        <v>464000</v>
       </c>
       <c r="J51" t="str">
         <v>44.4%</v>
       </c>
       <c r="K51">
-        <v>464000</v>
+        <v>1097000</v>
       </c>
       <c r="L51">
-        <v>23000</v>
+        <v>53000</v>
       </c>
       <c r="M51" t="str">
-        <v>5.2%</v>
+        <v>5.1%</v>
       </c>
       <c r="N51">
-        <v>534000</v>
+        <v>1262000</v>
       </c>
     </row>
     <row r="52">
@@ -4727,37 +4692,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D52" t="str">
-        <v>TK-0348A</v>
+        <v>TK-0369</v>
       </c>
       <c r="E52" t="str">
-        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F52">
-        <v>492000</v>
+        <v>419848</v>
       </c>
       <c r="G52">
-        <v>580000</v>
+        <v>535000</v>
       </c>
       <c r="H52">
-        <v>1044000</v>
+        <v>969000</v>
       </c>
       <c r="I52">
-        <v>464000</v>
+        <v>434000</v>
       </c>
       <c r="J52" t="str">
-        <v>44.4%</v>
+        <v>44.8%</v>
       </c>
       <c r="K52">
-        <v>1097000</v>
+        <v>1018000</v>
       </c>
       <c r="L52">
-        <v>53000</v>
+        <v>49000</v>
       </c>
       <c r="M52" t="str">
         <v>5.1%</v>
       </c>
       <c r="N52">
-        <v>1262000</v>
+        <v>1171000</v>
       </c>
     </row>
     <row r="53">
@@ -4771,37 +4736,37 @@
         <v>NỒI &amp; BỘ NỒI</v>
       </c>
       <c r="D53" t="str">
-        <v>TK-0369</v>
+        <v>TK-0488</v>
       </c>
       <c r="E53" t="str">
-        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F53">
-        <v>419848</v>
+        <v>672571</v>
       </c>
       <c r="G53">
-        <v>535000</v>
+        <v>810000</v>
       </c>
       <c r="H53">
-        <v>969000</v>
+        <v>1469000</v>
       </c>
       <c r="I53">
-        <v>434000</v>
+        <v>659000</v>
       </c>
       <c r="J53" t="str">
-        <v>44.8%</v>
+        <v>44.9%</v>
       </c>
       <c r="K53">
-        <v>1018000</v>
+        <v>1543000</v>
       </c>
       <c r="L53">
-        <v>49000</v>
+        <v>74000</v>
       </c>
       <c r="M53" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N53">
-        <v>1171000</v>
+        <v>1775000</v>
       </c>
     </row>
     <row r="54">
@@ -4812,40 +4777,40 @@
         <v>Takin</v>
       </c>
       <c r="C54" t="str">
-        <v>NỒI &amp; BỘ NỒI</v>
+        <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D54" t="str">
-        <v>TK-0488</v>
+        <v>TK-468</v>
       </c>
       <c r="E54" t="str">
-        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+        <v>Sưởi gốm thấp</v>
       </c>
       <c r="F54">
-        <v>672571</v>
+        <v>366857</v>
       </c>
       <c r="G54">
-        <v>810000</v>
+        <v>452000</v>
       </c>
       <c r="H54">
-        <v>1469000</v>
+        <v>900000</v>
       </c>
       <c r="I54">
-        <v>659000</v>
+        <v>448000</v>
       </c>
       <c r="J54" t="str">
-        <v>44.9%</v>
+        <v>49.8%</v>
       </c>
       <c r="K54">
-        <v>1543000</v>
+        <v>945000</v>
       </c>
       <c r="L54">
-        <v>74000</v>
+        <v>45000</v>
       </c>
       <c r="M54" t="str">
         <v>5.0%</v>
       </c>
       <c r="N54">
-        <v>1775000</v>
+        <v>1087000</v>
       </c>
     </row>
     <row r="55">
@@ -4859,37 +4824,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D55" t="str">
-        <v>TK-468</v>
+        <v>TK-469</v>
       </c>
       <c r="E55" t="str">
-        <v>Sưởi gốm thấp</v>
+        <v>Sưởi gốm thân cao</v>
       </c>
       <c r="F55">
-        <v>366857</v>
+        <v>468762</v>
       </c>
       <c r="G55">
-        <v>452000</v>
+        <v>615000</v>
       </c>
       <c r="H55">
-        <v>900000</v>
+        <v>1050000</v>
       </c>
       <c r="I55">
-        <v>448000</v>
+        <v>435000</v>
       </c>
       <c r="J55" t="str">
-        <v>49.8%</v>
+        <v>41.4%</v>
       </c>
       <c r="K55">
-        <v>945000</v>
+        <v>1103000</v>
       </c>
       <c r="L55">
-        <v>45000</v>
+        <v>53000</v>
       </c>
       <c r="M55" t="str">
         <v>5.0%</v>
       </c>
       <c r="N55">
-        <v>1087000</v>
+        <v>1269000</v>
       </c>
     </row>
     <row r="56">
@@ -4903,37 +4868,37 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D56" t="str">
-        <v>TK-469</v>
+        <v>TK-1002</v>
       </c>
       <c r="E56" t="str">
-        <v>Sưởi gốm thân cao</v>
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
       </c>
       <c r="F56">
-        <v>468762</v>
+        <v>128400</v>
       </c>
       <c r="G56">
-        <v>615000</v>
+        <v>158000</v>
       </c>
       <c r="H56">
-        <v>1050000</v>
+        <v>270000</v>
       </c>
       <c r="I56">
-        <v>435000</v>
+        <v>112000</v>
       </c>
       <c r="J56" t="str">
-        <v>41.4%</v>
+        <v>41.5%</v>
       </c>
       <c r="K56">
-        <v>1103000</v>
+        <v>284000</v>
       </c>
       <c r="L56">
-        <v>53000</v>
+        <v>14000</v>
       </c>
       <c r="M56" t="str">
-        <v>5.0%</v>
+        <v>5.2%</v>
       </c>
       <c r="N56">
-        <v>1269000</v>
+        <v>327000</v>
       </c>
     </row>
     <row r="57">
@@ -4947,86 +4912,42 @@
         <v>ĐỒ ĐIỆN</v>
       </c>
       <c r="D57" t="str">
-        <v>TK-1002</v>
+        <v>TK-1003</v>
       </c>
       <c r="E57" t="str">
-        <v>Bộ đèn sưởi 2 bóng Takin</v>
+        <v>Bộ đèn sưởi 3 bóng Takin</v>
       </c>
       <c r="F57">
-        <v>128400</v>
+        <v>157290</v>
       </c>
       <c r="G57">
-        <v>158000</v>
+        <v>194000</v>
       </c>
       <c r="H57">
-        <v>270000</v>
+        <v>330000</v>
       </c>
       <c r="I57">
-        <v>112000</v>
+        <v>136000</v>
       </c>
       <c r="J57" t="str">
-        <v>41.5%</v>
+        <v>41.2%</v>
       </c>
       <c r="K57">
-        <v>284000</v>
+        <v>347000</v>
       </c>
       <c r="L57">
-        <v>14000</v>
+        <v>17000</v>
       </c>
       <c r="M57" t="str">
         <v>5.2%</v>
       </c>
       <c r="N57">
-        <v>327000</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58" t="str">
-        <v>Takin</v>
-      </c>
-      <c r="C58" t="str">
-        <v>ĐỒ ĐIỆN</v>
-      </c>
-      <c r="D58" t="str">
-        <v>TK-1003</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Bộ đèn sưởi 3 bóng Takin</v>
-      </c>
-      <c r="F58">
-        <v>157290</v>
-      </c>
-      <c r="G58">
-        <v>194000</v>
-      </c>
-      <c r="H58">
-        <v>330000</v>
-      </c>
-      <c r="I58">
-        <v>136000</v>
-      </c>
-      <c r="J58" t="str">
-        <v>41.2%</v>
-      </c>
-      <c r="K58">
-        <v>347000</v>
-      </c>
-      <c r="L58">
-        <v>17000</v>
-      </c>
-      <c r="M58" t="str">
-        <v>5.2%</v>
-      </c>
-      <c r="N58">
         <v>400000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(pricing): cap nhat gia facebook cho LK-4160 (1.880.000d) va LK-4161 (1.490.000d)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -1658,19 +1658,19 @@
         <v>1000000</v>
       </c>
       <c r="G36">
-        <v>2350000</v>
+        <v>1880000</v>
       </c>
       <c r="H36">
-        <v>2514500</v>
+        <v>2011600</v>
       </c>
       <c r="I36">
-        <v>2820000</v>
+        <v>2256000</v>
       </c>
       <c r="J36">
-        <v>1350000</v>
+        <v>880000</v>
       </c>
       <c r="K36" t="str">
-        <v>57.4%</v>
+        <v>46.8%</v>
       </c>
     </row>
     <row r="37">
@@ -1693,19 +1693,19 @@
         <v>800000</v>
       </c>
       <c r="G37">
-        <v>1650000</v>
+        <v>1490000</v>
       </c>
       <c r="H37">
-        <v>1765500</v>
+        <v>1594300</v>
       </c>
       <c r="I37">
-        <v>1980000</v>
+        <v>1788000</v>
       </c>
       <c r="J37">
-        <v>850000</v>
+        <v>690000</v>
       </c>
       <c r="K37" t="str">
-        <v>51.5%</v>
+        <v>46.3%</v>
       </c>
     </row>
     <row r="38">
@@ -4000,25 +4000,25 @@
         <v>1000000</v>
       </c>
       <c r="H36">
-        <v>2350000</v>
+        <v>1880000</v>
       </c>
       <c r="I36">
-        <v>1350000</v>
+        <v>880000</v>
       </c>
       <c r="J36" t="str">
-        <v>57.4%</v>
+        <v>46.8%</v>
       </c>
       <c r="K36">
-        <v>2468000</v>
+        <v>1974000</v>
       </c>
       <c r="L36">
-        <v>118000</v>
+        <v>94000</v>
       </c>
       <c r="M36" t="str">
         <v>5.0%</v>
       </c>
       <c r="N36">
-        <v>2839000</v>
+        <v>2271000</v>
       </c>
     </row>
     <row r="37">
@@ -4044,25 +4044,25 @@
         <v>800000</v>
       </c>
       <c r="H37">
-        <v>1650000</v>
+        <v>1490000</v>
       </c>
       <c r="I37">
-        <v>850000</v>
+        <v>690000</v>
       </c>
       <c r="J37" t="str">
-        <v>51.5%</v>
+        <v>46.3%</v>
       </c>
       <c r="K37">
-        <v>1733000</v>
+        <v>1565000</v>
       </c>
       <c r="L37">
-        <v>83000</v>
+        <v>75000</v>
       </c>
       <c r="M37" t="str">
         <v>5.0%</v>
       </c>
       <c r="N37">
-        <v>1993000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="38">

</xml_diff>

<commit_message>
fix(pricing): cap nhat gia LK-2808SA KHONG NAP (NPP Online/Offline: 350.000d, FB: 650.000d)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -640,22 +640,22 @@
         <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA KHÔNG NẮP</v>
       </c>
       <c r="F7">
-        <v>412000</v>
+        <v>350000</v>
       </c>
       <c r="G7">
-        <v>740000</v>
+        <v>650000</v>
       </c>
       <c r="H7">
-        <v>799200</v>
+        <v>702000</v>
       </c>
       <c r="I7">
-        <v>962000</v>
+        <v>845000</v>
       </c>
       <c r="J7">
-        <v>328000</v>
+        <v>300000</v>
       </c>
       <c r="K7" t="str">
-        <v>44.3%</v>
+        <v>46.2%</v>
       </c>
     </row>
     <row r="8">
@@ -2721,28 +2721,28 @@
         <v>320736</v>
       </c>
       <c r="G7">
-        <v>412000</v>
+        <v>350000</v>
       </c>
       <c r="H7">
-        <v>740000</v>
+        <v>650000</v>
       </c>
       <c r="I7">
-        <v>328000</v>
+        <v>300000</v>
       </c>
       <c r="J7" t="str">
-        <v>44.3%</v>
+        <v>46.2%</v>
       </c>
       <c r="K7">
-        <v>777000</v>
+        <v>683000</v>
       </c>
       <c r="L7">
-        <v>37000</v>
+        <v>33000</v>
       </c>
       <c r="M7" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N7">
-        <v>894000</v>
+        <v>786000</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
fix(pricing): lam tron tang gia Facebook len dau nghin voi 3 so 0 cho toan bo san pham
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -468,7 +468,7 @@
         <v>265000</v>
       </c>
       <c r="G2">
-        <v>466960</v>
+        <v>467000</v>
       </c>
       <c r="H2">
         <v>513656</v>
@@ -477,10 +477,10 @@
         <v>607048</v>
       </c>
       <c r="J2">
-        <v>201960</v>
+        <v>202000</v>
       </c>
       <c r="K2" t="str">
-        <v>43.2%</v>
+        <v>43.3%</v>
       </c>
     </row>
     <row r="3">
@@ -1553,7 +1553,7 @@
         <v>372000</v>
       </c>
       <c r="G33">
-        <v>669600</v>
+        <v>670000</v>
       </c>
       <c r="H33">
         <v>723168</v>
@@ -1562,10 +1562,10 @@
         <v>870480</v>
       </c>
       <c r="J33">
-        <v>297600</v>
+        <v>298000</v>
       </c>
       <c r="K33" t="str">
-        <v>44.4%</v>
+        <v>44.5%</v>
       </c>
     </row>
     <row r="34">
@@ -1973,7 +1973,7 @@
         <v>265000</v>
       </c>
       <c r="G45">
-        <v>466960</v>
+        <v>467000</v>
       </c>
       <c r="H45">
         <v>491000</v>
@@ -1982,10 +1982,10 @@
         <v>607048</v>
       </c>
       <c r="J45">
-        <v>201960</v>
+        <v>202000</v>
       </c>
       <c r="K45" t="str">
-        <v>43.2%</v>
+        <v>43.3%</v>
       </c>
     </row>
     <row r="46">

</xml_diff>

<commit_message>
fix(pricing): cap nhat gia san TMDT (+8% cho 5 ma dac biet, +5% cho cac ma con lai, lam tron 1000)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -471,7 +471,7 @@
         <v>467000</v>
       </c>
       <c r="H2">
-        <v>513656</v>
+        <v>491000</v>
       </c>
       <c r="I2">
         <v>607048</v>
@@ -506,7 +506,7 @@
         <v>750000</v>
       </c>
       <c r="H3">
-        <v>788000</v>
+        <v>810000</v>
       </c>
       <c r="I3">
         <v>790000</v>
@@ -541,7 +541,7 @@
         <v>590000</v>
       </c>
       <c r="H4">
-        <v>637200</v>
+        <v>620000</v>
       </c>
       <c r="I4">
         <v>767000</v>
@@ -576,7 +576,7 @@
         <v>850000</v>
       </c>
       <c r="H5">
-        <v>961200</v>
+        <v>918000</v>
       </c>
       <c r="I5">
         <v>1200000</v>
@@ -611,7 +611,7 @@
         <v>630000</v>
       </c>
       <c r="H6">
-        <v>680400</v>
+        <v>662000</v>
       </c>
       <c r="I6">
         <v>819000</v>
@@ -646,7 +646,7 @@
         <v>650000</v>
       </c>
       <c r="H7">
-        <v>702000</v>
+        <v>683000</v>
       </c>
       <c r="I7">
         <v>845000</v>
@@ -716,7 +716,7 @@
         <v>1290000</v>
       </c>
       <c r="H9">
-        <v>1380300</v>
+        <v>1394000</v>
       </c>
       <c r="I9">
         <v>1548000</v>
@@ -751,7 +751,7 @@
         <v>750000</v>
       </c>
       <c r="H10">
-        <v>810000</v>
+        <v>788000</v>
       </c>
       <c r="I10">
         <v>975000</v>
@@ -786,7 +786,7 @@
         <v>830000</v>
       </c>
       <c r="H11">
-        <v>896400</v>
+        <v>872000</v>
       </c>
       <c r="I11">
         <v>1079000</v>
@@ -821,7 +821,7 @@
         <v>990000</v>
       </c>
       <c r="H12">
-        <v>1069200</v>
+        <v>1040000</v>
       </c>
       <c r="I12">
         <v>1287000</v>
@@ -856,7 +856,7 @@
         <v>295000</v>
       </c>
       <c r="H13">
-        <v>324500</v>
+        <v>310000</v>
       </c>
       <c r="I13">
         <v>383500</v>
@@ -891,7 +891,7 @@
         <v>315000</v>
       </c>
       <c r="H14">
-        <v>346500</v>
+        <v>331000</v>
       </c>
       <c r="I14">
         <v>409500</v>
@@ -926,7 +926,7 @@
         <v>395000</v>
       </c>
       <c r="H15">
-        <v>434500</v>
+        <v>415000</v>
       </c>
       <c r="I15">
         <v>513500</v>
@@ -961,7 +961,7 @@
         <v>689000</v>
       </c>
       <c r="H16">
-        <v>744120</v>
+        <v>724000</v>
       </c>
       <c r="I16">
         <v>895700</v>
@@ -996,7 +996,7 @@
         <v>779000</v>
       </c>
       <c r="H17">
-        <v>841320</v>
+        <v>818000</v>
       </c>
       <c r="I17">
         <v>1012700</v>
@@ -1031,7 +1031,7 @@
         <v>889000</v>
       </c>
       <c r="H18">
-        <v>960120</v>
+        <v>934000</v>
       </c>
       <c r="I18">
         <v>1155700</v>
@@ -1066,7 +1066,7 @@
         <v>1049000</v>
       </c>
       <c r="H19">
-        <v>1122430</v>
+        <v>1102000</v>
       </c>
       <c r="I19">
         <v>1258800</v>
@@ -1101,7 +1101,7 @@
         <v>2090000</v>
       </c>
       <c r="H20">
-        <v>2780930</v>
+        <v>2195000</v>
       </c>
       <c r="I20">
         <v>3118800</v>
@@ -1136,7 +1136,7 @@
         <v>990000</v>
       </c>
       <c r="H21">
-        <v>1069200</v>
+        <v>1040000</v>
       </c>
       <c r="I21">
         <v>1287000</v>
@@ -1171,7 +1171,7 @@
         <v>1690000</v>
       </c>
       <c r="H22">
-        <v>1808300</v>
+        <v>1775000</v>
       </c>
       <c r="I22">
         <v>2028000</v>
@@ -1206,7 +1206,7 @@
         <v>820000</v>
       </c>
       <c r="H23">
-        <v>885600</v>
+        <v>886000</v>
       </c>
       <c r="I23">
         <v>1066000</v>
@@ -1241,7 +1241,7 @@
         <v>990000</v>
       </c>
       <c r="H24">
-        <v>1069200</v>
+        <v>1070000</v>
       </c>
       <c r="I24">
         <v>1287000</v>
@@ -1276,7 +1276,7 @@
         <v>525000</v>
       </c>
       <c r="H25">
-        <v>567000</v>
+        <v>552000</v>
       </c>
       <c r="I25">
         <v>682500</v>
@@ -1311,7 +1311,7 @@
         <v>1590000</v>
       </c>
       <c r="H26">
-        <v>1701300</v>
+        <v>1670000</v>
       </c>
       <c r="I26">
         <v>1908000</v>
@@ -1346,7 +1346,7 @@
         <v>745000</v>
       </c>
       <c r="H27">
-        <v>804600</v>
+        <v>783000</v>
       </c>
       <c r="I27">
         <v>968500</v>
@@ -1381,7 +1381,7 @@
         <v>1050000</v>
       </c>
       <c r="H28">
-        <v>1123500</v>
+        <v>1103000</v>
       </c>
       <c r="I28">
         <v>1260000</v>
@@ -1416,7 +1416,7 @@
         <v>920000</v>
       </c>
       <c r="H29">
-        <v>993600</v>
+        <v>966000</v>
       </c>
       <c r="I29">
         <v>1196000</v>
@@ -1451,7 +1451,7 @@
         <v>1690000</v>
       </c>
       <c r="H30">
-        <v>1808300</v>
+        <v>1775000</v>
       </c>
       <c r="I30">
         <v>2028000</v>
@@ -1486,7 +1486,7 @@
         <v>354000</v>
       </c>
       <c r="H31">
-        <v>389400</v>
+        <v>372000</v>
       </c>
       <c r="I31">
         <v>460200</v>
@@ -1521,7 +1521,7 @@
         <v>1890000</v>
       </c>
       <c r="H32">
-        <v>1984500</v>
+        <v>1985000</v>
       </c>
       <c r="I32">
         <v>2063000</v>
@@ -1556,7 +1556,7 @@
         <v>670000</v>
       </c>
       <c r="H33">
-        <v>723168</v>
+        <v>704000</v>
       </c>
       <c r="I33">
         <v>870480</v>
@@ -1591,7 +1591,7 @@
         <v>1495000</v>
       </c>
       <c r="H34">
-        <v>1915300</v>
+        <v>1570000</v>
       </c>
       <c r="I34">
         <v>2148000</v>
@@ -1626,7 +1626,7 @@
         <v>599000</v>
       </c>
       <c r="H35">
-        <v>646920</v>
+        <v>629000</v>
       </c>
       <c r="I35">
         <v>778700</v>
@@ -1661,7 +1661,7 @@
         <v>1880000</v>
       </c>
       <c r="H36">
-        <v>2011600</v>
+        <v>1974000</v>
       </c>
       <c r="I36">
         <v>2256000</v>
@@ -1696,7 +1696,7 @@
         <v>1490000</v>
       </c>
       <c r="H37">
-        <v>1594300</v>
+        <v>1565000</v>
       </c>
       <c r="I37">
         <v>1788000</v>
@@ -1731,7 +1731,7 @@
         <v>950000</v>
       </c>
       <c r="H38">
-        <v>1026000</v>
+        <v>998000</v>
       </c>
       <c r="I38">
         <v>1235000</v>
@@ -1766,7 +1766,7 @@
         <v>950000</v>
       </c>
       <c r="H39">
-        <v>1026000</v>
+        <v>998000</v>
       </c>
       <c r="I39">
         <v>1235000</v>
@@ -1801,7 +1801,7 @@
         <v>1190000</v>
       </c>
       <c r="H40">
-        <v>1273300</v>
+        <v>1250000</v>
       </c>
       <c r="I40">
         <v>1428000</v>
@@ -1836,7 +1836,7 @@
         <v>490000</v>
       </c>
       <c r="H41">
-        <v>539000</v>
+        <v>515000</v>
       </c>
       <c r="I41">
         <v>637000</v>
@@ -1871,7 +1871,7 @@
         <v>1290000</v>
       </c>
       <c r="H42">
-        <v>1380300</v>
+        <v>1355000</v>
       </c>
       <c r="I42">
         <v>1548000</v>
@@ -1906,7 +1906,7 @@
         <v>1190000</v>
       </c>
       <c r="H43">
-        <v>1444500</v>
+        <v>1250000</v>
       </c>
       <c r="I43">
         <v>1620000</v>
@@ -1941,7 +1941,7 @@
         <v>2190000</v>
       </c>
       <c r="H44">
-        <v>2343300</v>
+        <v>2300000</v>
       </c>
       <c r="I44">
         <v>2628000</v>
@@ -2469,7 +2469,7 @@
         <v>% Biên LN FB / NPP Online</v>
       </c>
       <c r="K1" t="str">
-        <v>Giá Sàn TMĐT (+5% FB, Tròn Nghìn)</v>
+        <v>Giá Sàn TMĐT (+5%/+8% FB, Tròn Nghìn)</v>
       </c>
       <c r="L1" t="str">
         <v>Chênh Lệch TMĐT vs FB (VNĐ)</v>
@@ -2557,16 +2557,16 @@
         <v>47.3%</v>
       </c>
       <c r="K3">
-        <v>788000</v>
+        <v>810000</v>
       </c>
       <c r="L3">
-        <v>38000</v>
+        <v>60000</v>
       </c>
       <c r="M3" t="str">
-        <v>5.1%</v>
+        <v>8.0%</v>
       </c>
       <c r="N3">
-        <v>907000</v>
+        <v>932000</v>
       </c>
     </row>
     <row r="4">
@@ -2645,16 +2645,16 @@
         <v>47.1%</v>
       </c>
       <c r="K5">
-        <v>893000</v>
+        <v>918000</v>
       </c>
       <c r="L5">
-        <v>43000</v>
+        <v>68000</v>
       </c>
       <c r="M5" t="str">
-        <v>5.1%</v>
+        <v>8.0%</v>
       </c>
       <c r="N5">
-        <v>1027000</v>
+        <v>1056000</v>
       </c>
     </row>
     <row r="6">
@@ -2821,16 +2821,16 @@
         <v>50.0%</v>
       </c>
       <c r="K9">
-        <v>1355000</v>
+        <v>1394000</v>
       </c>
       <c r="L9">
-        <v>65000</v>
+        <v>104000</v>
       </c>
       <c r="M9" t="str">
-        <v>5.0%</v>
+        <v>8.1%</v>
       </c>
       <c r="N9">
-        <v>1559000</v>
+        <v>1604000</v>
       </c>
     </row>
     <row r="10">
@@ -3437,16 +3437,16 @@
         <v>42.7%</v>
       </c>
       <c r="K23">
-        <v>861000</v>
+        <v>886000</v>
       </c>
       <c r="L23">
-        <v>41000</v>
+        <v>66000</v>
       </c>
       <c r="M23" t="str">
-        <v>5.0%</v>
+        <v>8.0%</v>
       </c>
       <c r="N23">
-        <v>991000</v>
+        <v>1019000</v>
       </c>
     </row>
     <row r="24">
@@ -3481,16 +3481,16 @@
         <v>46.0%</v>
       </c>
       <c r="K24">
-        <v>1040000</v>
+        <v>1070000</v>
       </c>
       <c r="L24">
-        <v>50000</v>
+        <v>80000</v>
       </c>
       <c r="M24" t="str">
-        <v>5.1%</v>
+        <v>8.1%</v>
       </c>
       <c r="N24">
-        <v>1196000</v>
+        <v>1231000</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
fix(pricing): tang gia niem yet len 20% so voi gia san TMDT cho tat ca cac ma (lam tron 1000)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -474,7 +474,7 @@
         <v>491000</v>
       </c>
       <c r="I2">
-        <v>607048</v>
+        <v>590000</v>
       </c>
       <c r="J2">
         <v>202000</v>
@@ -509,7 +509,7 @@
         <v>810000</v>
       </c>
       <c r="I3">
-        <v>790000</v>
+        <v>972000</v>
       </c>
       <c r="J3">
         <v>355000</v>
@@ -544,7 +544,7 @@
         <v>620000</v>
       </c>
       <c r="I4">
-        <v>767000</v>
+        <v>744000</v>
       </c>
       <c r="J4">
         <v>270000</v>
@@ -579,7 +579,7 @@
         <v>918000</v>
       </c>
       <c r="I5">
-        <v>1200000</v>
+        <v>1102000</v>
       </c>
       <c r="J5">
         <v>400000</v>
@@ -614,7 +614,7 @@
         <v>662000</v>
       </c>
       <c r="I6">
-        <v>819000</v>
+        <v>795000</v>
       </c>
       <c r="J6">
         <v>279000</v>
@@ -649,7 +649,7 @@
         <v>683000</v>
       </c>
       <c r="I7">
-        <v>845000</v>
+        <v>820000</v>
       </c>
       <c r="J7">
         <v>300000</v>
@@ -684,7 +684,7 @@
         <v>788000</v>
       </c>
       <c r="I8">
-        <v>825000</v>
+        <v>946000</v>
       </c>
       <c r="J8">
         <v>375000</v>
@@ -719,7 +719,7 @@
         <v>1394000</v>
       </c>
       <c r="I9">
-        <v>1548000</v>
+        <v>1673000</v>
       </c>
       <c r="J9">
         <v>645000</v>
@@ -754,7 +754,7 @@
         <v>788000</v>
       </c>
       <c r="I10">
-        <v>975000</v>
+        <v>946000</v>
       </c>
       <c r="J10">
         <v>336000</v>
@@ -789,7 +789,7 @@
         <v>872000</v>
       </c>
       <c r="I11">
-        <v>1079000</v>
+        <v>1047000</v>
       </c>
       <c r="J11">
         <v>360000</v>
@@ -824,7 +824,7 @@
         <v>1040000</v>
       </c>
       <c r="I12">
-        <v>1287000</v>
+        <v>1248000</v>
       </c>
       <c r="J12">
         <v>450000</v>
@@ -859,7 +859,7 @@
         <v>310000</v>
       </c>
       <c r="I13">
-        <v>383500</v>
+        <v>372000</v>
       </c>
       <c r="J13">
         <v>125000</v>
@@ -894,7 +894,7 @@
         <v>331000</v>
       </c>
       <c r="I14">
-        <v>409500</v>
+        <v>398000</v>
       </c>
       <c r="J14">
         <v>130000</v>
@@ -929,7 +929,7 @@
         <v>415000</v>
       </c>
       <c r="I15">
-        <v>513500</v>
+        <v>498000</v>
       </c>
       <c r="J15">
         <v>165000</v>
@@ -964,7 +964,7 @@
         <v>724000</v>
       </c>
       <c r="I16">
-        <v>895700</v>
+        <v>869000</v>
       </c>
       <c r="J16">
         <v>364000</v>
@@ -999,7 +999,7 @@
         <v>818000</v>
       </c>
       <c r="I17">
-        <v>1012700</v>
+        <v>982000</v>
       </c>
       <c r="J17">
         <v>439000</v>
@@ -1034,7 +1034,7 @@
         <v>934000</v>
       </c>
       <c r="I18">
-        <v>1155700</v>
+        <v>1121000</v>
       </c>
       <c r="J18">
         <v>499000</v>
@@ -1069,7 +1069,7 @@
         <v>1102000</v>
       </c>
       <c r="I19">
-        <v>1258800</v>
+        <v>1323000</v>
       </c>
       <c r="J19">
         <v>589000</v>
@@ -1104,7 +1104,7 @@
         <v>2195000</v>
       </c>
       <c r="I20">
-        <v>3118800</v>
+        <v>2634000</v>
       </c>
       <c r="J20">
         <v>990000</v>
@@ -1139,7 +1139,7 @@
         <v>1040000</v>
       </c>
       <c r="I21">
-        <v>1287000</v>
+        <v>1248000</v>
       </c>
       <c r="J21">
         <v>440000</v>
@@ -1174,7 +1174,7 @@
         <v>1775000</v>
       </c>
       <c r="I22">
-        <v>2028000</v>
+        <v>2130000</v>
       </c>
       <c r="J22">
         <v>730000</v>
@@ -1209,7 +1209,7 @@
         <v>886000</v>
       </c>
       <c r="I23">
-        <v>1066000</v>
+        <v>1064000</v>
       </c>
       <c r="J23">
         <v>350000</v>
@@ -1244,7 +1244,7 @@
         <v>1070000</v>
       </c>
       <c r="I24">
-        <v>1287000</v>
+        <v>1284000</v>
       </c>
       <c r="J24">
         <v>455000</v>
@@ -1279,7 +1279,7 @@
         <v>552000</v>
       </c>
       <c r="I25">
-        <v>682500</v>
+        <v>663000</v>
       </c>
       <c r="J25">
         <v>225000</v>
@@ -1314,7 +1314,7 @@
         <v>1670000</v>
       </c>
       <c r="I26">
-        <v>1908000</v>
+        <v>2004000</v>
       </c>
       <c r="J26">
         <v>755000</v>
@@ -1349,7 +1349,7 @@
         <v>783000</v>
       </c>
       <c r="I27">
-        <v>968500</v>
+        <v>940000</v>
       </c>
       <c r="J27">
         <v>315000</v>
@@ -1384,7 +1384,7 @@
         <v>1103000</v>
       </c>
       <c r="I28">
-        <v>1260000</v>
+        <v>1324000</v>
       </c>
       <c r="J28">
         <v>465000</v>
@@ -1419,7 +1419,7 @@
         <v>966000</v>
       </c>
       <c r="I29">
-        <v>1196000</v>
+        <v>1160000</v>
       </c>
       <c r="J29">
         <v>460000</v>
@@ -1454,7 +1454,7 @@
         <v>1775000</v>
       </c>
       <c r="I30">
-        <v>2028000</v>
+        <v>2130000</v>
       </c>
       <c r="J30">
         <v>840000</v>
@@ -1489,7 +1489,7 @@
         <v>372000</v>
       </c>
       <c r="I31">
-        <v>460200</v>
+        <v>447000</v>
       </c>
       <c r="J31">
         <v>157000</v>
@@ -1524,7 +1524,7 @@
         <v>1985000</v>
       </c>
       <c r="I32">
-        <v>2063000</v>
+        <v>2382000</v>
       </c>
       <c r="J32">
         <v>870000</v>
@@ -1559,7 +1559,7 @@
         <v>704000</v>
       </c>
       <c r="I33">
-        <v>870480</v>
+        <v>845000</v>
       </c>
       <c r="J33">
         <v>298000</v>
@@ -1594,7 +1594,7 @@
         <v>1570000</v>
       </c>
       <c r="I34">
-        <v>2148000</v>
+        <v>1884000</v>
       </c>
       <c r="J34">
         <v>715000</v>
@@ -1629,7 +1629,7 @@
         <v>629000</v>
       </c>
       <c r="I35">
-        <v>778700</v>
+        <v>755000</v>
       </c>
       <c r="J35">
         <v>289000</v>
@@ -1664,7 +1664,7 @@
         <v>1974000</v>
       </c>
       <c r="I36">
-        <v>2256000</v>
+        <v>2369000</v>
       </c>
       <c r="J36">
         <v>880000</v>
@@ -1699,7 +1699,7 @@
         <v>1565000</v>
       </c>
       <c r="I37">
-        <v>1788000</v>
+        <v>1878000</v>
       </c>
       <c r="J37">
         <v>690000</v>
@@ -1734,7 +1734,7 @@
         <v>998000</v>
       </c>
       <c r="I38">
-        <v>1235000</v>
+        <v>1198000</v>
       </c>
       <c r="J38">
         <v>440000</v>
@@ -1769,7 +1769,7 @@
         <v>998000</v>
       </c>
       <c r="I39">
-        <v>1235000</v>
+        <v>1198000</v>
       </c>
       <c r="J39">
         <v>440000</v>
@@ -1804,7 +1804,7 @@
         <v>1250000</v>
       </c>
       <c r="I40">
-        <v>1428000</v>
+        <v>1500000</v>
       </c>
       <c r="J40">
         <v>590000</v>
@@ -1839,7 +1839,7 @@
         <v>515000</v>
       </c>
       <c r="I41">
-        <v>637000</v>
+        <v>618000</v>
       </c>
       <c r="J41">
         <v>230000</v>
@@ -1874,7 +1874,7 @@
         <v>1355000</v>
       </c>
       <c r="I42">
-        <v>1548000</v>
+        <v>1626000</v>
       </c>
       <c r="J42">
         <v>605000</v>
@@ -1909,7 +1909,7 @@
         <v>1250000</v>
       </c>
       <c r="I43">
-        <v>1620000</v>
+        <v>1500000</v>
       </c>
       <c r="J43">
         <v>530000</v>
@@ -1944,7 +1944,7 @@
         <v>2300000</v>
       </c>
       <c r="I44">
-        <v>2628000</v>
+        <v>2760000</v>
       </c>
       <c r="J44">
         <v>1060000</v>
@@ -1979,7 +1979,7 @@
         <v>491000</v>
       </c>
       <c r="I45">
-        <v>607048</v>
+        <v>590000</v>
       </c>
       <c r="J45">
         <v>202000</v>
@@ -2014,7 +2014,7 @@
         <v>620000</v>
       </c>
       <c r="I46">
-        <v>767000</v>
+        <v>744000</v>
       </c>
       <c r="J46">
         <v>270000</v>
@@ -2049,7 +2049,7 @@
         <v>662000</v>
       </c>
       <c r="I47">
-        <v>819000</v>
+        <v>795000</v>
       </c>
       <c r="J47">
         <v>279000</v>
@@ -2084,7 +2084,7 @@
         <v>788000</v>
       </c>
       <c r="I48">
-        <v>825000</v>
+        <v>946000</v>
       </c>
       <c r="J48">
         <v>375000</v>
@@ -2119,7 +2119,7 @@
         <v>936000</v>
       </c>
       <c r="I49">
-        <v>1158300</v>
+        <v>1124000</v>
       </c>
       <c r="J49">
         <v>396000</v>
@@ -2154,7 +2154,7 @@
         <v>464000</v>
       </c>
       <c r="I50">
-        <v>573300</v>
+        <v>557000</v>
       </c>
       <c r="J50">
         <v>196000</v>
@@ -2189,7 +2189,7 @@
         <v>1097000</v>
       </c>
       <c r="I51">
-        <v>1252800</v>
+        <v>1317000</v>
       </c>
       <c r="J51">
         <v>464000</v>
@@ -2224,7 +2224,7 @@
         <v>1018000</v>
       </c>
       <c r="I52">
-        <v>1259700</v>
+        <v>1222000</v>
       </c>
       <c r="J52">
         <v>434000</v>
@@ -2259,7 +2259,7 @@
         <v>1543000</v>
       </c>
       <c r="I53">
-        <v>1762800</v>
+        <v>1852000</v>
       </c>
       <c r="J53">
         <v>659000</v>
@@ -2294,7 +2294,7 @@
         <v>945000</v>
       </c>
       <c r="I54">
-        <v>1170000</v>
+        <v>1134000</v>
       </c>
       <c r="J54">
         <v>448000</v>
@@ -2329,7 +2329,7 @@
         <v>1103000</v>
       </c>
       <c r="I55">
-        <v>1260000</v>
+        <v>1324000</v>
       </c>
       <c r="J55">
         <v>435000</v>
@@ -2364,7 +2364,7 @@
         <v>284000</v>
       </c>
       <c r="I56">
-        <v>351000</v>
+        <v>341000</v>
       </c>
       <c r="J56">
         <v>112000</v>
@@ -2399,7 +2399,7 @@
         <v>347000</v>
       </c>
       <c r="I57">
-        <v>429000</v>
+        <v>417000</v>
       </c>
       <c r="J57">
         <v>136000</v>
@@ -2478,7 +2478,7 @@
         <v>% Biên Độ TMĐT vs FB</v>
       </c>
       <c r="N1" t="str">
-        <v>Giá Niêm Yết (+15% TMĐT, Tròn Nghìn)</v>
+        <v>Giá Niêm Yết (+20% TMĐT, Tròn Nghìn)</v>
       </c>
     </row>
     <row r="2">
@@ -2522,7 +2522,7 @@
         <v>5.1%</v>
       </c>
       <c r="N2">
-        <v>565000</v>
+        <v>590000</v>
       </c>
     </row>
     <row r="3">
@@ -2566,7 +2566,7 @@
         <v>8.0%</v>
       </c>
       <c r="N3">
-        <v>932000</v>
+        <v>972000</v>
       </c>
     </row>
     <row r="4">
@@ -2610,7 +2610,7 @@
         <v>5.1%</v>
       </c>
       <c r="N4">
-        <v>713000</v>
+        <v>744000</v>
       </c>
     </row>
     <row r="5">
@@ -2654,7 +2654,7 @@
         <v>8.0%</v>
       </c>
       <c r="N5">
-        <v>1056000</v>
+        <v>1102000</v>
       </c>
     </row>
     <row r="6">
@@ -2698,7 +2698,7 @@
         <v>5.1%</v>
       </c>
       <c r="N6">
-        <v>762000</v>
+        <v>795000</v>
       </c>
     </row>
     <row r="7">
@@ -2742,7 +2742,7 @@
         <v>5.1%</v>
       </c>
       <c r="N7">
-        <v>786000</v>
+        <v>820000</v>
       </c>
     </row>
     <row r="8">
@@ -2786,7 +2786,7 @@
         <v>5.1%</v>
       </c>
       <c r="N8">
-        <v>907000</v>
+        <v>946000</v>
       </c>
     </row>
     <row r="9">
@@ -2830,7 +2830,7 @@
         <v>8.1%</v>
       </c>
       <c r="N9">
-        <v>1604000</v>
+        <v>1673000</v>
       </c>
     </row>
     <row r="10">
@@ -2874,7 +2874,7 @@
         <v>5.1%</v>
       </c>
       <c r="N10">
-        <v>907000</v>
+        <v>946000</v>
       </c>
     </row>
     <row r="11">
@@ -2918,7 +2918,7 @@
         <v>5.1%</v>
       </c>
       <c r="N11">
-        <v>1003000</v>
+        <v>1047000</v>
       </c>
     </row>
     <row r="12">
@@ -2962,7 +2962,7 @@
         <v>5.1%</v>
       </c>
       <c r="N12">
-        <v>1196000</v>
+        <v>1248000</v>
       </c>
     </row>
     <row r="13">
@@ -3006,7 +3006,7 @@
         <v>5.1%</v>
       </c>
       <c r="N13">
-        <v>357000</v>
+        <v>372000</v>
       </c>
     </row>
     <row r="14">
@@ -3050,7 +3050,7 @@
         <v>5.1%</v>
       </c>
       <c r="N14">
-        <v>381000</v>
+        <v>398000</v>
       </c>
     </row>
     <row r="15">
@@ -3094,7 +3094,7 @@
         <v>5.1%</v>
       </c>
       <c r="N15">
-        <v>478000</v>
+        <v>498000</v>
       </c>
     </row>
     <row r="16">
@@ -3138,7 +3138,7 @@
         <v>5.1%</v>
       </c>
       <c r="N16">
-        <v>833000</v>
+        <v>869000</v>
       </c>
     </row>
     <row r="17">
@@ -3182,7 +3182,7 @@
         <v>5.0%</v>
       </c>
       <c r="N17">
-        <v>941000</v>
+        <v>982000</v>
       </c>
     </row>
     <row r="18">
@@ -3226,7 +3226,7 @@
         <v>5.1%</v>
       </c>
       <c r="N18">
-        <v>1075000</v>
+        <v>1121000</v>
       </c>
     </row>
     <row r="19">
@@ -3270,7 +3270,7 @@
         <v>5.1%</v>
       </c>
       <c r="N19">
-        <v>1268000</v>
+        <v>1323000</v>
       </c>
     </row>
     <row r="20">
@@ -3314,7 +3314,7 @@
         <v>5.0%</v>
       </c>
       <c r="N20">
-        <v>2525000</v>
+        <v>2634000</v>
       </c>
     </row>
     <row r="21">
@@ -3358,7 +3358,7 @@
         <v>5.1%</v>
       </c>
       <c r="N21">
-        <v>1196000</v>
+        <v>1248000</v>
       </c>
     </row>
     <row r="22">
@@ -3402,7 +3402,7 @@
         <v>5.0%</v>
       </c>
       <c r="N22">
-        <v>2042000</v>
+        <v>2130000</v>
       </c>
     </row>
     <row r="23">
@@ -3446,7 +3446,7 @@
         <v>8.0%</v>
       </c>
       <c r="N23">
-        <v>1019000</v>
+        <v>1064000</v>
       </c>
     </row>
     <row r="24">
@@ -3490,7 +3490,7 @@
         <v>8.1%</v>
       </c>
       <c r="N24">
-        <v>1231000</v>
+        <v>1284000</v>
       </c>
     </row>
     <row r="25">
@@ -3534,7 +3534,7 @@
         <v>5.1%</v>
       </c>
       <c r="N25">
-        <v>635000</v>
+        <v>663000</v>
       </c>
     </row>
     <row r="26">
@@ -3578,7 +3578,7 @@
         <v>5.0%</v>
       </c>
       <c r="N26">
-        <v>1921000</v>
+        <v>2004000</v>
       </c>
     </row>
     <row r="27">
@@ -3622,7 +3622,7 @@
         <v>5.1%</v>
       </c>
       <c r="N27">
-        <v>901000</v>
+        <v>940000</v>
       </c>
     </row>
     <row r="28">
@@ -3666,7 +3666,7 @@
         <v>5.0%</v>
       </c>
       <c r="N28">
-        <v>1269000</v>
+        <v>1324000</v>
       </c>
     </row>
     <row r="29">
@@ -3710,7 +3710,7 @@
         <v>5.0%</v>
       </c>
       <c r="N29">
-        <v>1111000</v>
+        <v>1160000</v>
       </c>
     </row>
     <row r="30">
@@ -3754,7 +3754,7 @@
         <v>5.0%</v>
       </c>
       <c r="N30">
-        <v>2042000</v>
+        <v>2130000</v>
       </c>
     </row>
     <row r="31">
@@ -3798,7 +3798,7 @@
         <v>5.1%</v>
       </c>
       <c r="N31">
-        <v>428000</v>
+        <v>447000</v>
       </c>
     </row>
     <row r="32">
@@ -3842,7 +3842,7 @@
         <v>5.0%</v>
       </c>
       <c r="N32">
-        <v>2283000</v>
+        <v>2382000</v>
       </c>
     </row>
     <row r="33">
@@ -3886,7 +3886,7 @@
         <v>5.1%</v>
       </c>
       <c r="N33">
-        <v>810000</v>
+        <v>845000</v>
       </c>
     </row>
     <row r="34">
@@ -3930,7 +3930,7 @@
         <v>5.0%</v>
       </c>
       <c r="N34">
-        <v>1806000</v>
+        <v>1884000</v>
       </c>
     </row>
     <row r="35">
@@ -3974,7 +3974,7 @@
         <v>5.0%</v>
       </c>
       <c r="N35">
-        <v>724000</v>
+        <v>755000</v>
       </c>
     </row>
     <row r="36">
@@ -4018,7 +4018,7 @@
         <v>5.0%</v>
       </c>
       <c r="N36">
-        <v>2271000</v>
+        <v>2369000</v>
       </c>
     </row>
     <row r="37">
@@ -4062,7 +4062,7 @@
         <v>5.0%</v>
       </c>
       <c r="N37">
-        <v>1800000</v>
+        <v>1878000</v>
       </c>
     </row>
     <row r="38">
@@ -4106,7 +4106,7 @@
         <v>5.1%</v>
       </c>
       <c r="N38">
-        <v>1148000</v>
+        <v>1198000</v>
       </c>
     </row>
     <row r="39">
@@ -4150,7 +4150,7 @@
         <v>5.1%</v>
       </c>
       <c r="N39">
-        <v>1148000</v>
+        <v>1198000</v>
       </c>
     </row>
     <row r="40">
@@ -4194,7 +4194,7 @@
         <v>5.0%</v>
       </c>
       <c r="N40">
-        <v>1438000</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="41">
@@ -4238,7 +4238,7 @@
         <v>5.1%</v>
       </c>
       <c r="N41">
-        <v>593000</v>
+        <v>618000</v>
       </c>
     </row>
     <row r="42">
@@ -4282,7 +4282,7 @@
         <v>5.0%</v>
       </c>
       <c r="N42">
-        <v>1559000</v>
+        <v>1626000</v>
       </c>
     </row>
     <row r="43">
@@ -4326,7 +4326,7 @@
         <v>5.0%</v>
       </c>
       <c r="N43">
-        <v>1438000</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="44">
@@ -4370,7 +4370,7 @@
         <v>5.0%</v>
       </c>
       <c r="N44">
-        <v>2645000</v>
+        <v>2760000</v>
       </c>
     </row>
     <row r="45">
@@ -4414,7 +4414,7 @@
         <v>5.1%</v>
       </c>
       <c r="N45">
-        <v>565000</v>
+        <v>590000</v>
       </c>
     </row>
     <row r="46">
@@ -4458,7 +4458,7 @@
         <v>5.1%</v>
       </c>
       <c r="N46">
-        <v>713000</v>
+        <v>744000</v>
       </c>
     </row>
     <row r="47">
@@ -4502,7 +4502,7 @@
         <v>5.1%</v>
       </c>
       <c r="N47">
-        <v>762000</v>
+        <v>795000</v>
       </c>
     </row>
     <row r="48">
@@ -4546,7 +4546,7 @@
         <v>5.1%</v>
       </c>
       <c r="N48">
-        <v>907000</v>
+        <v>946000</v>
       </c>
     </row>
     <row r="49">
@@ -4590,7 +4590,7 @@
         <v>5.1%</v>
       </c>
       <c r="N49">
-        <v>1077000</v>
+        <v>1124000</v>
       </c>
     </row>
     <row r="50">
@@ -4634,7 +4634,7 @@
         <v>5.2%</v>
       </c>
       <c r="N50">
-        <v>534000</v>
+        <v>557000</v>
       </c>
     </row>
     <row r="51">
@@ -4678,7 +4678,7 @@
         <v>5.1%</v>
       </c>
       <c r="N51">
-        <v>1262000</v>
+        <v>1317000</v>
       </c>
     </row>
     <row r="52">
@@ -4722,7 +4722,7 @@
         <v>5.1%</v>
       </c>
       <c r="N52">
-        <v>1171000</v>
+        <v>1222000</v>
       </c>
     </row>
     <row r="53">
@@ -4766,7 +4766,7 @@
         <v>5.0%</v>
       </c>
       <c r="N53">
-        <v>1775000</v>
+        <v>1852000</v>
       </c>
     </row>
     <row r="54">
@@ -4810,7 +4810,7 @@
         <v>5.0%</v>
       </c>
       <c r="N54">
-        <v>1087000</v>
+        <v>1134000</v>
       </c>
     </row>
     <row r="55">
@@ -4854,7 +4854,7 @@
         <v>5.0%</v>
       </c>
       <c r="N55">
-        <v>1269000</v>
+        <v>1324000</v>
       </c>
     </row>
     <row r="56">
@@ -4898,7 +4898,7 @@
         <v>5.2%</v>
       </c>
       <c r="N56">
-        <v>327000</v>
+        <v>341000</v>
       </c>
     </row>
     <row r="57">
@@ -4942,7 +4942,7 @@
         <v>5.2%</v>
       </c>
       <c r="N57">
-        <v>400000</v>
+        <v>417000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(pricing): them module thong ke bien dong gia NPP Online (cu vs moi & kenh ban)
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Bang_Gia_Chuan_56_Ma" sheetId="1" r:id="rId1"/>
     <sheet name="ChenhLech_Gia_FB_TMDT_NY" sheetId="2" r:id="rId2"/>
+    <sheet name="BienDong_Gia_NPP" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -4950,4 +4951,2195 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N57"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L57"/>
+  <cols>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Thương Hiệu</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Phân Loại</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Model (Mã Sản Phẩm)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Tên Sản Phẩm</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Giá NPP Cũ (VNĐ)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Giá Điều Chỉnh Mới (VNĐ)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Chênh Lệch (VNĐ)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>% Tăng/Giảm</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Trạng Thái</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Giá Facebook (VNĐ)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Giá Sàn TMĐT (VNĐ)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C2" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D2" t="str">
+        <v>LK-2202A</v>
+      </c>
+      <c r="E2" t="str">
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) LK-2202A</v>
+      </c>
+      <c r="F2">
+        <v>260000</v>
+      </c>
+      <c r="G2">
+        <v>265000</v>
+      </c>
+      <c r="H2">
+        <v>5000</v>
+      </c>
+      <c r="I2" t="str">
+        <v>1.9%</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K2">
+        <v>467000</v>
+      </c>
+      <c r="L2">
+        <v>491000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>LK-2433</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Chảo Belly Lock&amp;King</v>
+      </c>
+      <c r="F3">
+        <v>410000</v>
+      </c>
+      <c r="G3">
+        <v>395000</v>
+      </c>
+      <c r="H3">
+        <v>-15000</v>
+      </c>
+      <c r="I3" t="str">
+        <v>-3.7%</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K3">
+        <v>750000</v>
+      </c>
+      <c r="L3">
+        <v>810000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>LK-2606A</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Chảo cạn Titanium Lock&amp;king 26cm</v>
+      </c>
+      <c r="F4">
+        <v>310000</v>
+      </c>
+      <c r="G4">
+        <v>320000</v>
+      </c>
+      <c r="H4">
+        <v>10000</v>
+      </c>
+      <c r="I4" t="str">
+        <v>3.2%</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K4">
+        <v>590000</v>
+      </c>
+      <c r="L4">
+        <v>620000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>LK-2633</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Chảo Belly Lock&amp;King Titanium 26cm</v>
+      </c>
+      <c r="F5">
+        <v>470000</v>
+      </c>
+      <c r="G5">
+        <v>450000</v>
+      </c>
+      <c r="H5">
+        <v>-20000</v>
+      </c>
+      <c r="I5" t="str">
+        <v>-4.3%</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K5">
+        <v>850000</v>
+      </c>
+      <c r="L5">
+        <v>918000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D6" t="str">
+        <v>LK-2808</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+      </c>
+      <c r="F6">
+        <v>341000</v>
+      </c>
+      <c r="G6">
+        <v>351000</v>
+      </c>
+      <c r="H6">
+        <v>10000</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2.9%</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K6">
+        <v>630000</v>
+      </c>
+      <c r="L6">
+        <v>662000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D7" t="str">
+        <v>LK-2808SA KHÔNG NẮP</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Chảo sâu Titan vàng 28*9cm (2,3 mm) LK-2808SA KHÔNG NẮP</v>
+      </c>
+      <c r="F7">
+        <v>412000</v>
+      </c>
+      <c r="G7">
+        <v>350000</v>
+      </c>
+      <c r="H7">
+        <v>-62000</v>
+      </c>
+      <c r="I7" t="str">
+        <v>-15.0%</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K7">
+        <v>650000</v>
+      </c>
+      <c r="L7">
+        <v>683000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D8" t="str">
+        <v>LK-3003</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Chảo cạn titanium Lock&amp;King 30cm</v>
+      </c>
+      <c r="F8">
+        <v>360000</v>
+      </c>
+      <c r="G8">
+        <v>375000</v>
+      </c>
+      <c r="H8">
+        <v>15000</v>
+      </c>
+      <c r="I8" t="str">
+        <v>4.2%</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K8">
+        <v>750000</v>
+      </c>
+      <c r="L8">
+        <v>788000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D9" t="str">
+        <v>LK-3212</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Chảo xào lớn</v>
+      </c>
+      <c r="F9">
+        <v>645000</v>
+      </c>
+      <c r="G9">
+        <v>645000</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K9">
+        <v>1290000</v>
+      </c>
+      <c r="L9">
+        <v>1394000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C10" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D10" t="str">
+        <v>LK-30NC1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Nồi luộc gà Lock&amp;King size 30</v>
+      </c>
+      <c r="F10">
+        <v>399000</v>
+      </c>
+      <c r="G10">
+        <v>414000</v>
+      </c>
+      <c r="H10">
+        <v>15000</v>
+      </c>
+      <c r="I10" t="str">
+        <v>3.8%</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K10">
+        <v>750000</v>
+      </c>
+      <c r="L10">
+        <v>788000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C11" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D11" t="str">
+        <v>LK-32NC1</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Nồi luộc gà Lock&amp;King size 32</v>
+      </c>
+      <c r="F11">
+        <v>455000</v>
+      </c>
+      <c r="G11">
+        <v>470000</v>
+      </c>
+      <c r="H11">
+        <v>15000</v>
+      </c>
+      <c r="I11" t="str">
+        <v>3.3%</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K11">
+        <v>830000</v>
+      </c>
+      <c r="L11">
+        <v>872000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C12" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D12" t="str">
+        <v>LK-336A</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Bộ nồi 3 Lock&amp;King ( 18,20,24 )</v>
+      </c>
+      <c r="F12">
+        <v>540000</v>
+      </c>
+      <c r="G12">
+        <v>540000</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K12">
+        <v>990000</v>
+      </c>
+      <c r="L12">
+        <v>1040000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C13" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D13" t="str">
+        <v>LK-3018A</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Nồi lẻ Lock&amp;king 18</v>
+      </c>
+      <c r="F13">
+        <v>170000</v>
+      </c>
+      <c r="G13">
+        <v>170000</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K13">
+        <v>295000</v>
+      </c>
+      <c r="L13">
+        <v>310000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C14" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D14" t="str">
+        <v>LK-3020A</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Nồi lẻ Lock&amp;king 20</v>
+      </c>
+      <c r="F14">
+        <v>185000</v>
+      </c>
+      <c r="G14">
+        <v>185000</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K14">
+        <v>315000</v>
+      </c>
+      <c r="L14">
+        <v>331000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C15" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D15" t="str">
+        <v>LK-3024</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Nồi lẻ Lock&amp;king 24</v>
+      </c>
+      <c r="F15">
+        <v>230000</v>
+      </c>
+      <c r="G15">
+        <v>230000</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K15">
+        <v>395000</v>
+      </c>
+      <c r="L15">
+        <v>415000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C16" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D16" t="str">
+        <v>LK-3116</v>
+      </c>
+      <c r="E16" t="str">
+        <v>16*9CM Quánh liền khối titan (2.2mm) LK-3116</v>
+      </c>
+      <c r="F16">
+        <v>325000</v>
+      </c>
+      <c r="G16">
+        <v>325000</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K16">
+        <v>689000</v>
+      </c>
+      <c r="L16">
+        <v>724000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C17" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D17" t="str">
+        <v>LK-3118</v>
+      </c>
+      <c r="E17" t="str">
+        <v>18*10CM Nồi lẻ kèm nắp (2.3mm) LK-3118</v>
+      </c>
+      <c r="F17">
+        <v>372000</v>
+      </c>
+      <c r="G17">
+        <v>340000</v>
+      </c>
+      <c r="H17">
+        <v>-32000</v>
+      </c>
+      <c r="I17" t="str">
+        <v>-8.6%</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K17">
+        <v>779000</v>
+      </c>
+      <c r="L17">
+        <v>818000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C18" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D18" t="str">
+        <v>LK-3120</v>
+      </c>
+      <c r="E18" t="str">
+        <v>20*12CM Nồi lẻ kèm nắp (2.3mm) LK-3120</v>
+      </c>
+      <c r="F18">
+        <v>420000</v>
+      </c>
+      <c r="G18">
+        <v>390000</v>
+      </c>
+      <c r="H18">
+        <v>-30000</v>
+      </c>
+      <c r="I18" t="str">
+        <v>-7.1%</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K18">
+        <v>889000</v>
+      </c>
+      <c r="L18">
+        <v>934000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C19" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D19" t="str">
+        <v>LK-3124</v>
+      </c>
+      <c r="E19" t="str">
+        <v>24*14CM Nồi lẻ kèm nắp (2.3mm) LK-3124</v>
+      </c>
+      <c r="F19">
+        <v>500000</v>
+      </c>
+      <c r="G19">
+        <v>460000</v>
+      </c>
+      <c r="H19">
+        <v>-40000</v>
+      </c>
+      <c r="I19" t="str">
+        <v>-8.0%</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K19">
+        <v>1049000</v>
+      </c>
+      <c r="L19">
+        <v>1102000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C20" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D20" t="str">
+        <v>LK-3338</v>
+      </c>
+      <c r="E20" t="str">
+        <v>18+20+24CM Bộ nồi 3 liền khối kèm nắp (2.3mm) LK-3338</v>
+      </c>
+      <c r="F20">
+        <v>1240000</v>
+      </c>
+      <c r="G20">
+        <v>1100000</v>
+      </c>
+      <c r="H20">
+        <v>-140000</v>
+      </c>
+      <c r="I20" t="str">
+        <v>-11.3%</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K20">
+        <v>2090000</v>
+      </c>
+      <c r="L20">
+        <v>2195000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C21" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D21" t="str">
+        <v>LK-3386A</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Bộ nồi 3 Inox 5 đáy Lock&amp;king (18.20.24) (1t/4c)</v>
+      </c>
+      <c r="F21">
+        <v>530000</v>
+      </c>
+      <c r="G21">
+        <v>550000</v>
+      </c>
+      <c r="H21">
+        <v>20000</v>
+      </c>
+      <c r="I21" t="str">
+        <v>3.8%</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K21">
+        <v>990000</v>
+      </c>
+      <c r="L21">
+        <v>1040000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C22" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D22" t="str">
+        <v>LK-3568A</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Bộ nồi 5 Inox 5 đáy Lock&amp;king (Q16.18.20.24.C24) (1t/2c)</v>
+      </c>
+      <c r="F22">
+        <v>940000</v>
+      </c>
+      <c r="G22">
+        <v>960000</v>
+      </c>
+      <c r="H22">
+        <v>20000</v>
+      </c>
+      <c r="I22" t="str">
+        <v>2.1%</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K22">
+        <v>1690000</v>
+      </c>
+      <c r="L22">
+        <v>1775000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C23" t="str">
+        <v>NỒI TĂNG ÁP</v>
+      </c>
+      <c r="D23" t="str">
+        <v>LK-3122</v>
+      </c>
+      <c r="E23" t="str">
+        <v>22*13.5CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3122</v>
+      </c>
+      <c r="F23">
+        <v>460000</v>
+      </c>
+      <c r="G23">
+        <v>470000</v>
+      </c>
+      <c r="H23">
+        <v>10000</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2.2%</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K23">
+        <v>820000</v>
+      </c>
+      <c r="L23">
+        <v>886000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C24" t="str">
+        <v>NỒI TĂNG ÁP</v>
+      </c>
+      <c r="D24" t="str">
+        <v>LK-3126</v>
+      </c>
+      <c r="E24" t="str">
+        <v>26*14CM Nồi áp suất kèm xửng hấp đa năng (1.8mm) LK-3126</v>
+      </c>
+      <c r="F24">
+        <v>525000</v>
+      </c>
+      <c r="G24">
+        <v>535000</v>
+      </c>
+      <c r="H24">
+        <v>10000</v>
+      </c>
+      <c r="I24" t="str">
+        <v>1.9%</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K24">
+        <v>990000</v>
+      </c>
+      <c r="L24">
+        <v>1070000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C25" t="str">
+        <v>ẤM &amp; BÌNH</v>
+      </c>
+      <c r="D25" t="str">
+        <v>LK-1038</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Ấm đun nước LK-1038</v>
+      </c>
+      <c r="F25">
+        <v>300000</v>
+      </c>
+      <c r="G25">
+        <v>300000</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K25">
+        <v>525000</v>
+      </c>
+      <c r="L25">
+        <v>552000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C26" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D26" t="str">
+        <v>LK-92</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Nồi chiên không dầu Lock&amp;king</v>
+      </c>
+      <c r="F26">
+        <v>835000</v>
+      </c>
+      <c r="G26">
+        <v>835000</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K26">
+        <v>1590000</v>
+      </c>
+      <c r="L26">
+        <v>1670000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C27" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D27" t="str">
+        <v>LK-586</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Sưởi gốm thấp</v>
+      </c>
+      <c r="F27">
+        <v>430000</v>
+      </c>
+      <c r="G27">
+        <v>430000</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K27">
+        <v>745000</v>
+      </c>
+      <c r="L27">
+        <v>783000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C28" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D28" t="str">
+        <v>LK-588</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Sưởi gốm thân cao</v>
+      </c>
+      <c r="F28">
+        <v>585000</v>
+      </c>
+      <c r="G28">
+        <v>585000</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K28">
+        <v>1050000</v>
+      </c>
+      <c r="L28">
+        <v>1103000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C29" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D29" t="str">
+        <v>LK-668</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 1500W</v>
+      </c>
+      <c r="F29">
+        <v>460000</v>
+      </c>
+      <c r="G29">
+        <v>460000</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K29">
+        <v>920000</v>
+      </c>
+      <c r="L29">
+        <v>966000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C30" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D30" t="str">
+        <v>LK-688</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Tủ sấy quần áo cao cấp Lock&amp;king 2400W</v>
+      </c>
+      <c r="F30">
+        <v>850000</v>
+      </c>
+      <c r="G30">
+        <v>850000</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K30">
+        <v>1690000</v>
+      </c>
+      <c r="L30">
+        <v>1775000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C31" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D31" t="str">
+        <v>LK-1003</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+      </c>
+      <c r="F31">
+        <v>197000</v>
+      </c>
+      <c r="G31">
+        <v>197000</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K31">
+        <v>354000</v>
+      </c>
+      <c r="L31">
+        <v>372000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C32" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D32" t="str">
+        <v>LK-1030</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Bình thủy điện 3L Lock&amp;King (4c/t)</v>
+      </c>
+      <c r="F32">
+        <v>1020000</v>
+      </c>
+      <c r="G32">
+        <v>1020000</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K32">
+        <v>1890000</v>
+      </c>
+      <c r="L32">
+        <v>1985000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C33" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D33" t="str">
+        <v>LK-1033</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Bộ đèn sưởi 3 bóng Lock&amp;King</v>
+      </c>
+      <c r="F33">
+        <v>372000</v>
+      </c>
+      <c r="G33">
+        <v>372000</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K33">
+        <v>670000</v>
+      </c>
+      <c r="L33">
+        <v>704000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C34" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D34" t="str">
+        <v>LK-1050</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Bình Thủy Điện Lock&amp;King LK-1050</v>
+      </c>
+      <c r="F34">
+        <v>890000</v>
+      </c>
+      <c r="G34">
+        <v>780000</v>
+      </c>
+      <c r="H34">
+        <v>-110000</v>
+      </c>
+      <c r="I34" t="str">
+        <v>-12.4%</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K34">
+        <v>1495000</v>
+      </c>
+      <c r="L34">
+        <v>1570000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C35" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D35" t="str">
+        <v>LK-1068</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Ấm siêu tốc LK-1068</v>
+      </c>
+      <c r="F35">
+        <v>340000</v>
+      </c>
+      <c r="G35">
+        <v>310000</v>
+      </c>
+      <c r="H35">
+        <v>-30000</v>
+      </c>
+      <c r="I35" t="str">
+        <v>-8.8%</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K35">
+        <v>599000</v>
+      </c>
+      <c r="L35">
+        <v>629000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C36" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D36" t="str">
+        <v>LK-4160</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Nồi áp suất điện Lock&amp;King LK-4160</v>
+      </c>
+      <c r="F36">
+        <v>1080000</v>
+      </c>
+      <c r="G36">
+        <v>1000000</v>
+      </c>
+      <c r="H36">
+        <v>-80000</v>
+      </c>
+      <c r="I36" t="str">
+        <v>-7.4%</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K36">
+        <v>1880000</v>
+      </c>
+      <c r="L36">
+        <v>1974000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C37" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D37" t="str">
+        <v>LK-4161</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Nồi áp suất điện Lock&amp;King LK-4161</v>
+      </c>
+      <c r="F37">
+        <v>850000</v>
+      </c>
+      <c r="G37">
+        <v>800000</v>
+      </c>
+      <c r="H37">
+        <v>-50000</v>
+      </c>
+      <c r="I37" t="str">
+        <v>-5.9%</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K37">
+        <v>1490000</v>
+      </c>
+      <c r="L37">
+        <v>1565000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C38" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D38" t="str">
+        <v>LK-4208A</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4208A</v>
+      </c>
+      <c r="F38">
+        <v>510000</v>
+      </c>
+      <c r="G38">
+        <v>510000</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K38">
+        <v>950000</v>
+      </c>
+      <c r="L38">
+        <v>998000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C39" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D39" t="str">
+        <v>LK-4209</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Nồi Nấu Chậm Lock&amp;King LK-4209</v>
+      </c>
+      <c r="F39">
+        <v>510000</v>
+      </c>
+      <c r="G39">
+        <v>510000</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K39">
+        <v>950000</v>
+      </c>
+      <c r="L39">
+        <v>998000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C40" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D40" t="str">
+        <v>LK-5301</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Sưởi để bàn</v>
+      </c>
+      <c r="F40">
+        <v>600000</v>
+      </c>
+      <c r="G40">
+        <v>600000</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K40">
+        <v>1190000</v>
+      </c>
+      <c r="L40">
+        <v>1250000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C41" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D41" t="str">
+        <v>LK-6015</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Nồi Nấu Đa Năng Lock&amp;King</v>
+      </c>
+      <c r="F41">
+        <v>260000</v>
+      </c>
+      <c r="G41">
+        <v>260000</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K41">
+        <v>490000</v>
+      </c>
+      <c r="L41">
+        <v>515000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C42" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D42" t="str">
+        <v>LK-6201</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Nồi nấu lẩu đi kèm xửng hấp</v>
+      </c>
+      <c r="F42">
+        <v>685000</v>
+      </c>
+      <c r="G42">
+        <v>685000</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K42">
+        <v>1290000</v>
+      </c>
+      <c r="L42">
+        <v>1355000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C43" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D43" t="str">
+        <v>LK-7812</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Máy làm sữa hạt Lock&amp;King</v>
+      </c>
+      <c r="F43">
+        <v>710000</v>
+      </c>
+      <c r="G43">
+        <v>660000</v>
+      </c>
+      <c r="H43">
+        <v>-50000</v>
+      </c>
+      <c r="I43" t="str">
+        <v>-7.0%</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K43">
+        <v>1190000</v>
+      </c>
+      <c r="L43">
+        <v>1250000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Lock&amp;King</v>
+      </c>
+      <c r="C44" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D44" t="str">
+        <v>LK-9014</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Nồi chiên không dầu Lock&amp;king</v>
+      </c>
+      <c r="F44">
+        <v>1130000</v>
+      </c>
+      <c r="G44">
+        <v>1130000</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J44" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K44">
+        <v>2190000</v>
+      </c>
+      <c r="L44">
+        <v>2300000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C45" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D45" t="str">
+        <v>TK-2201</v>
+      </c>
+      <c r="E45" t="str">
+        <v>chảo cạn Titan vàng 22*5,5cm (2,2 mm) TK-2201</v>
+      </c>
+      <c r="F45">
+        <v>260000</v>
+      </c>
+      <c r="G45">
+        <v>265000</v>
+      </c>
+      <c r="H45">
+        <v>5000</v>
+      </c>
+      <c r="I45" t="str">
+        <v>1.9%</v>
+      </c>
+      <c r="J45" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K45">
+        <v>467000</v>
+      </c>
+      <c r="L45">
+        <v>491000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C46" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D46" t="str">
+        <v>TK-2662</v>
+      </c>
+      <c r="E46" t="str">
+        <v>26*6.5CM Chảo cạn titan-TK-2662 (2.2mm)</v>
+      </c>
+      <c r="F46">
+        <v>310000</v>
+      </c>
+      <c r="G46">
+        <v>320000</v>
+      </c>
+      <c r="H46">
+        <v>10000</v>
+      </c>
+      <c r="I46" t="str">
+        <v>3.2%</v>
+      </c>
+      <c r="J46" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K46">
+        <v>590000</v>
+      </c>
+      <c r="L46">
+        <v>620000</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C47" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D47" t="str">
+        <v>TK-2882C</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Chảo cạn Titan vàng 28*7cm (2,3 mm)</v>
+      </c>
+      <c r="F47">
+        <v>341000</v>
+      </c>
+      <c r="G47">
+        <v>351000</v>
+      </c>
+      <c r="H47">
+        <v>10000</v>
+      </c>
+      <c r="I47" t="str">
+        <v>2.9%</v>
+      </c>
+      <c r="J47" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K47">
+        <v>630000</v>
+      </c>
+      <c r="L47">
+        <v>662000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C48" t="str">
+        <v>CHẢO</v>
+      </c>
+      <c r="D48" t="str">
+        <v>TK-3030C</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Chảo cạn Titan vàng 30*7cm (2,3 mm)</v>
+      </c>
+      <c r="F48">
+        <v>360000</v>
+      </c>
+      <c r="G48">
+        <v>375000</v>
+      </c>
+      <c r="H48">
+        <v>15000</v>
+      </c>
+      <c r="I48" t="str">
+        <v>4.2%</v>
+      </c>
+      <c r="J48" t="str">
+        <v>Tăng giá</v>
+      </c>
+      <c r="K48">
+        <v>750000</v>
+      </c>
+      <c r="L48">
+        <v>788000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C49" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D49" t="str">
+        <v>TK-036A</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F49">
+        <v>515000</v>
+      </c>
+      <c r="G49">
+        <v>495000</v>
+      </c>
+      <c r="H49">
+        <v>-20000</v>
+      </c>
+      <c r="I49" t="str">
+        <v>-3.9%</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Giảm giá</v>
+      </c>
+      <c r="K49">
+        <v>891000</v>
+      </c>
+      <c r="L49">
+        <v>936000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C50" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D50" t="str">
+        <v>TK-0324</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Nồi táo inox cao cấp size24</v>
+      </c>
+      <c r="F50">
+        <v>245000</v>
+      </c>
+      <c r="G50">
+        <v>245000</v>
+      </c>
+      <c r="H50">
+        <v>0</v>
+      </c>
+      <c r="I50" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K50">
+        <v>441000</v>
+      </c>
+      <c r="L50">
+        <v>464000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C51" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D51" t="str">
+        <v>TK-0348A</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Bộ nồi Táo Takin 3 món inox cao cấp</v>
+      </c>
+      <c r="F51">
+        <v>580000</v>
+      </c>
+      <c r="G51">
+        <v>580000</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K51">
+        <v>1044000</v>
+      </c>
+      <c r="L51">
+        <v>1097000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C52" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D52" t="str">
+        <v>TK-0369</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F52">
+        <v>535000</v>
+      </c>
+      <c r="G52">
+        <v>535000</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K52">
+        <v>969000</v>
+      </c>
+      <c r="L52">
+        <v>1018000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C53" t="str">
+        <v>NỒI &amp; BỘ NỒI</v>
+      </c>
+      <c r="D53" t="str">
+        <v>TK-0488</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Bộ nồi Takin 4 món 5 đáy inox cao cấp</v>
+      </c>
+      <c r="F53">
+        <v>810000</v>
+      </c>
+      <c r="G53">
+        <v>810000</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J53" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K53">
+        <v>1469000</v>
+      </c>
+      <c r="L53">
+        <v>1543000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C54" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D54" t="str">
+        <v>TK-468</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Sưởi gốm thấp</v>
+      </c>
+      <c r="F54">
+        <v>452000</v>
+      </c>
+      <c r="G54">
+        <v>452000</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K54">
+        <v>900000</v>
+      </c>
+      <c r="L54">
+        <v>945000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C55" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D55" t="str">
+        <v>TK-469</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Sưởi gốm thân cao</v>
+      </c>
+      <c r="F55">
+        <v>615000</v>
+      </c>
+      <c r="G55">
+        <v>615000</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K55">
+        <v>1050000</v>
+      </c>
+      <c r="L55">
+        <v>1103000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C56" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D56" t="str">
+        <v>TK-1002</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Bộ đèn sưởi 2 bóng Takin</v>
+      </c>
+      <c r="F56">
+        <v>158000</v>
+      </c>
+      <c r="G56">
+        <v>158000</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J56" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K56">
+        <v>270000</v>
+      </c>
+      <c r="L56">
+        <v>284000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Takin</v>
+      </c>
+      <c r="C57" t="str">
+        <v>ĐỒ ĐIỆN</v>
+      </c>
+      <c r="D57" t="str">
+        <v>TK-1003</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Bộ đèn sưởi 3 bóng Takin</v>
+      </c>
+      <c r="F57">
+        <v>194000</v>
+      </c>
+      <c r="G57">
+        <v>194000</v>
+      </c>
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57" t="str">
+        <v>0.0%</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Giữ nguyên</v>
+      </c>
+      <c r="K57">
+        <v>330000</v>
+      </c>
+      <c r="L57">
+        <v>347000</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L57"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(pricing): cap nhat gia NPP, Facebook, TMDT, Niem Yet va Loi Nhuan cho LK-3116, LK-3118, LK-3120, LK-3124 va TK-036A
</commit_message>
<xml_diff>
--- a/bang_gia_chuan_lock_and_king_takin.xlsx
+++ b/bang_gia_chuan_lock_and_king_takin.xlsx
@@ -959,19 +959,19 @@
         <v>325000</v>
       </c>
       <c r="G16">
-        <v>689000</v>
+        <v>630000</v>
       </c>
       <c r="H16">
-        <v>724000</v>
+        <v>662000</v>
       </c>
       <c r="I16">
-        <v>869000</v>
+        <v>795000</v>
       </c>
       <c r="J16">
-        <v>364000</v>
+        <v>305000</v>
       </c>
       <c r="K16" t="str">
-        <v>52.8%</v>
+        <v>48.4%</v>
       </c>
     </row>
     <row r="17">
@@ -994,19 +994,19 @@
         <v>340000</v>
       </c>
       <c r="G17">
-        <v>779000</v>
+        <v>650000</v>
       </c>
       <c r="H17">
-        <v>818000</v>
+        <v>683000</v>
       </c>
       <c r="I17">
-        <v>982000</v>
+        <v>820000</v>
       </c>
       <c r="J17">
-        <v>439000</v>
+        <v>310000</v>
       </c>
       <c r="K17" t="str">
-        <v>56.4%</v>
+        <v>47.7%</v>
       </c>
     </row>
     <row r="18">
@@ -1029,19 +1029,19 @@
         <v>390000</v>
       </c>
       <c r="G18">
-        <v>889000</v>
+        <v>740000</v>
       </c>
       <c r="H18">
-        <v>934000</v>
+        <v>777000</v>
       </c>
       <c r="I18">
-        <v>1121000</v>
+        <v>933000</v>
       </c>
       <c r="J18">
-        <v>499000</v>
+        <v>350000</v>
       </c>
       <c r="K18" t="str">
-        <v>56.1%</v>
+        <v>47.3%</v>
       </c>
     </row>
     <row r="19">
@@ -1064,19 +1064,19 @@
         <v>460000</v>
       </c>
       <c r="G19">
-        <v>1049000</v>
+        <v>880000</v>
       </c>
       <c r="H19">
-        <v>1102000</v>
+        <v>924000</v>
       </c>
       <c r="I19">
-        <v>1323000</v>
+        <v>1109000</v>
       </c>
       <c r="J19">
-        <v>589000</v>
+        <v>420000</v>
       </c>
       <c r="K19" t="str">
-        <v>56.1%</v>
+        <v>47.7%</v>
       </c>
     </row>
     <row r="20">
@@ -2111,7 +2111,7 @@
         <v>Bộ nồi Takin 3 món 5 đáy inox cao cấp</v>
       </c>
       <c r="F49">
-        <v>495000</v>
+        <v>515000</v>
       </c>
       <c r="G49">
         <v>891000</v>
@@ -2123,10 +2123,10 @@
         <v>1124000</v>
       </c>
       <c r="J49">
-        <v>396000</v>
+        <v>376000</v>
       </c>
       <c r="K49" t="str">
-        <v>44.4%</v>
+        <v>42.2%</v>
       </c>
     </row>
     <row r="50">
@@ -3121,25 +3121,25 @@
         <v>325000</v>
       </c>
       <c r="H16">
-        <v>689000</v>
+        <v>630000</v>
       </c>
       <c r="I16">
-        <v>364000</v>
+        <v>305000</v>
       </c>
       <c r="J16" t="str">
-        <v>52.8%</v>
+        <v>48.4%</v>
       </c>
       <c r="K16">
-        <v>724000</v>
+        <v>662000</v>
       </c>
       <c r="L16">
-        <v>35000</v>
+        <v>32000</v>
       </c>
       <c r="M16" t="str">
         <v>5.1%</v>
       </c>
       <c r="N16">
-        <v>869000</v>
+        <v>795000</v>
       </c>
     </row>
     <row r="17">
@@ -3165,25 +3165,25 @@
         <v>340000</v>
       </c>
       <c r="H17">
-        <v>779000</v>
+        <v>650000</v>
       </c>
       <c r="I17">
-        <v>439000</v>
+        <v>310000</v>
       </c>
       <c r="J17" t="str">
-        <v>56.4%</v>
+        <v>47.7%</v>
       </c>
       <c r="K17">
-        <v>818000</v>
+        <v>683000</v>
       </c>
       <c r="L17">
-        <v>39000</v>
+        <v>33000</v>
       </c>
       <c r="M17" t="str">
-        <v>5.0%</v>
+        <v>5.1%</v>
       </c>
       <c r="N17">
-        <v>982000</v>
+        <v>820000</v>
       </c>
     </row>
     <row r="18">
@@ -3209,25 +3209,25 @@
         <v>390000</v>
       </c>
       <c r="H18">
-        <v>889000</v>
+        <v>740000</v>
       </c>
       <c r="I18">
-        <v>499000</v>
+        <v>350000</v>
       </c>
       <c r="J18" t="str">
-        <v>56.1%</v>
+        <v>47.3%</v>
       </c>
       <c r="K18">
-        <v>934000</v>
+        <v>777000</v>
       </c>
       <c r="L18">
-        <v>45000</v>
+        <v>37000</v>
       </c>
       <c r="M18" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N18">
-        <v>1121000</v>
+        <v>933000</v>
       </c>
     </row>
     <row r="19">
@@ -3253,25 +3253,25 @@
         <v>460000</v>
       </c>
       <c r="H19">
-        <v>1049000</v>
+        <v>880000</v>
       </c>
       <c r="I19">
-        <v>589000</v>
+        <v>420000</v>
       </c>
       <c r="J19" t="str">
-        <v>56.1%</v>
+        <v>47.7%</v>
       </c>
       <c r="K19">
-        <v>1102000</v>
+        <v>924000</v>
       </c>
       <c r="L19">
-        <v>53000</v>
+        <v>44000</v>
       </c>
       <c r="M19" t="str">
-        <v>5.1%</v>
+        <v>5.0%</v>
       </c>
       <c r="N19">
-        <v>1323000</v>
+        <v>1109000</v>
       </c>
     </row>
     <row r="20">
@@ -4570,16 +4570,16 @@
         <v>433985</v>
       </c>
       <c r="G49">
-        <v>495000</v>
+        <v>515000</v>
       </c>
       <c r="H49">
         <v>891000</v>
       </c>
       <c r="I49">
-        <v>396000</v>
+        <v>376000</v>
       </c>
       <c r="J49" t="str">
-        <v>44.4%</v>
+        <v>42.2%</v>
       </c>
       <c r="K49">
         <v>936000</v>
@@ -5573,10 +5573,10 @@
         <v>Giữ nguyên</v>
       </c>
       <c r="K16">
-        <v>689000</v>
+        <v>630000</v>
       </c>
       <c r="L16">
-        <v>724000</v>
+        <v>662000</v>
       </c>
     </row>
     <row r="17">
@@ -5611,10 +5611,10 @@
         <v>Giảm giá</v>
       </c>
       <c r="K17">
-        <v>779000</v>
+        <v>650000</v>
       </c>
       <c r="L17">
-        <v>818000</v>
+        <v>683000</v>
       </c>
     </row>
     <row r="18">
@@ -5649,10 +5649,10 @@
         <v>Giảm giá</v>
       </c>
       <c r="K18">
-        <v>889000</v>
+        <v>740000</v>
       </c>
       <c r="L18">
-        <v>934000</v>
+        <v>777000</v>
       </c>
     </row>
     <row r="19">
@@ -5687,10 +5687,10 @@
         <v>Giảm giá</v>
       </c>
       <c r="K19">
-        <v>1049000</v>
+        <v>880000</v>
       </c>
       <c r="L19">
-        <v>1102000</v>
+        <v>924000</v>
       </c>
     </row>
     <row r="20">
@@ -6815,16 +6815,16 @@
         <v>515000</v>
       </c>
       <c r="G49">
-        <v>495000</v>
+        <v>515000</v>
       </c>
       <c r="H49">
-        <v>-20000</v>
+        <v>0</v>
       </c>
       <c r="I49" t="str">
-        <v>-3.9%</v>
+        <v>0.0%</v>
       </c>
       <c r="J49" t="str">
-        <v>Giảm giá</v>
+        <v>Giữ nguyên</v>
       </c>
       <c r="K49">
         <v>891000</v>

</xml_diff>